<commit_message>
feat(diarias): perfis de policiais, geração conjunta e impressão de PDF
- Perfis de Diárias: campos, validação, persistência e painel em Configurações > Policial > Diárias
- Geração conjunta dos nove campos (mapa, requerimentos, declaração) com plano de impressão
- Impressão em processo isolado (GDI) com ordem, vias e primeira página da escala
- Modelos atualizados (mapa .xlsx com fontes/fórmulas, requerimentos, meios próprios)
- FFmpeg: waveform, prévia de áudio da junção, marcadores de transição e layout dos players
- Ícones/estilos das ferramentas e ajustes de layout (IMEI, QR Code, histórico)
</commit_message>
<xml_diff>
--- a/modelos/modelo_mapa.xlsx
+++ b/modelos/modelo_mapa.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gustavo\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{591A7257-DA92-43CB-9846-32E7278D18CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98ECFAE4-9925-4457-8878-6CC21F0332D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{807D5CED-EEB3-4DB9-8087-ADFB5AE7F696}"/>
   </bookViews>
@@ -35,6 +35,8 @@
     <definedName name="Z_FF834EEA_98EE_4D52_930D_AE89D7F4F75B_.wvu.Cols" localSheetId="0" hidden="1">'Limite 50%'!$AF:$AZ</definedName>
     <definedName name="Z_FF834EEA_98EE_4D52_930D_AE89D7F4F75B_.wvu.PrintArea" localSheetId="0" hidden="1">'Limite 50%'!$A$1:$AE$51</definedName>
     <definedName name="Z_FF834EEA_98EE_4D52_930D_AE89D7F4F75B_.wvu.Rows" localSheetId="0" hidden="1">'Limite 50%'!$53:$152</definedName>
+    <definedName name="_SIG_DIARIAS_B34_TEMPLATE_001" hidden="1">"PGlzPjx0PkFzc3VtaXIgbyBQbGFudMOjbyBuYSBDZW50cmFsIGRlIFBvbMOtY2lhIEp1ZGljacOhcmlhIGRlIHt7e2NpZGFkZV9wbGFudGFvfX19LVNQLCBjb25mb3JtZSBkZXRlcm1pbmHDp8OjbyBjb250aWRhIG5hIEVzY2FsYSByZWZlcmVudGUgYSB7e3tkYXRh"</definedName>
+    <definedName name="_SIG_DIARIAS_B34_TEMPLATE_002" hidden="1">"X2lkYX19fTwvdD48L2lzPg=="</definedName>
   </definedNames>
   <calcPr calcId="191029" calcMode="manual" fullPrecision="0"/>
   <customWorkbookViews>
@@ -607,7 +609,7 @@
     <t>215626/2026</t>
   </si>
   <si>
-    <t>Assumir o Plantão na Central de Polícia Judiciária de Taquarituba-SP, conforme determinação contida na Escala referente a {{{data_ida}}}</t>
+    <t>Assumir o Plantão na Central de Polícia Judiciária de {{{cidade_plantao}}}-SP, conforme determinação contida na Escala referente a {{{data_ida}}}</t>
   </si>
 </sst>
 </file>
@@ -2267,12 +2269,6 @@
     <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="14" fontId="44" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="4" fontId="25" fillId="0" borderId="31" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
@@ -2357,28 +2353,12 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
     <xf numFmtId="49" fontId="29" fillId="0" borderId="24" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="24" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="38" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="38" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="49" fontId="25" fillId="2" borderId="11" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -2459,6 +2439,22 @@
       <alignment horizontal="left"/>
       <protection hidden="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="24" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="38" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="38" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="41" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
       <protection locked="0"/>
@@ -2495,6 +2491,18 @@
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="45" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="46" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="42" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
@@ -2526,18 +2534,6 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="31" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="45" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="46" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="46" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2594,6 +2590,12 @@
     <xf numFmtId="165" fontId="8" fillId="2" borderId="27" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -3696,33 +3698,33 @@
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
-      <c r="F2" s="266" t="s">
-        <v>0</v>
-      </c>
-      <c r="G2" s="266"/>
-      <c r="H2" s="266"/>
-      <c r="I2" s="266"/>
-      <c r="J2" s="266"/>
-      <c r="K2" s="266"/>
-      <c r="L2" s="266"/>
-      <c r="M2" s="266"/>
-      <c r="N2" s="266"/>
-      <c r="O2" s="266"/>
-      <c r="P2" s="266"/>
-      <c r="Q2" s="266"/>
-      <c r="R2" s="266"/>
-      <c r="S2" s="266"/>
-      <c r="T2" s="266"/>
-      <c r="U2" s="266"/>
-      <c r="V2" s="266"/>
-      <c r="W2" s="266"/>
-      <c r="X2" s="266"/>
-      <c r="Y2" s="266"/>
-      <c r="Z2" s="266"/>
-      <c r="AA2" s="266"/>
-      <c r="AB2" s="266"/>
-      <c r="AC2" s="266"/>
-      <c r="AD2" s="266"/>
+      <c r="F2" s="264" t="s">
+        <v>0</v>
+      </c>
+      <c r="G2" s="264"/>
+      <c r="H2" s="264"/>
+      <c r="I2" s="264"/>
+      <c r="J2" s="264"/>
+      <c r="K2" s="264"/>
+      <c r="L2" s="264"/>
+      <c r="M2" s="264"/>
+      <c r="N2" s="264"/>
+      <c r="O2" s="264"/>
+      <c r="P2" s="264"/>
+      <c r="Q2" s="264"/>
+      <c r="R2" s="264"/>
+      <c r="S2" s="264"/>
+      <c r="T2" s="264"/>
+      <c r="U2" s="264"/>
+      <c r="V2" s="264"/>
+      <c r="W2" s="264"/>
+      <c r="X2" s="264"/>
+      <c r="Y2" s="264"/>
+      <c r="Z2" s="264"/>
+      <c r="AA2" s="264"/>
+      <c r="AB2" s="264"/>
+      <c r="AC2" s="264"/>
+      <c r="AD2" s="264"/>
       <c r="AE2" s="5"/>
       <c r="AF2" s="6"/>
       <c r="AG2" s="6"/>
@@ -3730,33 +3732,33 @@
     <row r="3" spans="1:38" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2"/>
       <c r="B3" s="7"/>
-      <c r="F3" s="267" t="s">
+      <c r="F3" s="265" t="s">
         <v>1</v>
       </c>
-      <c r="G3" s="267"/>
-      <c r="H3" s="267"/>
-      <c r="I3" s="267"/>
-      <c r="J3" s="267"/>
-      <c r="K3" s="267"/>
-      <c r="L3" s="267"/>
-      <c r="M3" s="267"/>
-      <c r="N3" s="267"/>
-      <c r="O3" s="267"/>
-      <c r="P3" s="267"/>
-      <c r="Q3" s="267"/>
-      <c r="R3" s="267"/>
-      <c r="S3" s="267"/>
-      <c r="T3" s="267"/>
-      <c r="U3" s="267"/>
-      <c r="V3" s="267"/>
-      <c r="W3" s="267"/>
-      <c r="X3" s="267"/>
-      <c r="Y3" s="267"/>
-      <c r="Z3" s="267"/>
-      <c r="AA3" s="267"/>
-      <c r="AB3" s="267"/>
-      <c r="AC3" s="267"/>
-      <c r="AD3" s="267"/>
+      <c r="G3" s="265"/>
+      <c r="H3" s="265"/>
+      <c r="I3" s="265"/>
+      <c r="J3" s="265"/>
+      <c r="K3" s="265"/>
+      <c r="L3" s="265"/>
+      <c r="M3" s="265"/>
+      <c r="N3" s="265"/>
+      <c r="O3" s="265"/>
+      <c r="P3" s="265"/>
+      <c r="Q3" s="265"/>
+      <c r="R3" s="265"/>
+      <c r="S3" s="265"/>
+      <c r="T3" s="265"/>
+      <c r="U3" s="265"/>
+      <c r="V3" s="265"/>
+      <c r="W3" s="265"/>
+      <c r="X3" s="265"/>
+      <c r="Y3" s="265"/>
+      <c r="Z3" s="265"/>
+      <c r="AA3" s="265"/>
+      <c r="AB3" s="265"/>
+      <c r="AC3" s="265"/>
+      <c r="AD3" s="265"/>
       <c r="AE3" s="8"/>
       <c r="AF3" s="6"/>
       <c r="AG3" s="6"/>
@@ -3764,33 +3766,33 @@
     <row r="4" spans="1:38" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2"/>
       <c r="B4" s="7"/>
-      <c r="F4" s="267" t="s">
+      <c r="F4" s="265" t="s">
         <v>2</v>
       </c>
-      <c r="G4" s="267"/>
-      <c r="H4" s="267"/>
-      <c r="I4" s="267"/>
-      <c r="J4" s="267"/>
-      <c r="K4" s="267"/>
-      <c r="L4" s="267"/>
-      <c r="M4" s="267"/>
-      <c r="N4" s="267"/>
-      <c r="O4" s="267"/>
-      <c r="P4" s="267"/>
-      <c r="Q4" s="267"/>
-      <c r="R4" s="267"/>
-      <c r="S4" s="267"/>
-      <c r="T4" s="267"/>
-      <c r="U4" s="267"/>
-      <c r="V4" s="267"/>
-      <c r="W4" s="267"/>
-      <c r="X4" s="267"/>
-      <c r="Y4" s="267"/>
-      <c r="Z4" s="267"/>
-      <c r="AA4" s="267"/>
-      <c r="AB4" s="267"/>
-      <c r="AC4" s="267"/>
-      <c r="AD4" s="267"/>
+      <c r="G4" s="265"/>
+      <c r="H4" s="265"/>
+      <c r="I4" s="265"/>
+      <c r="J4" s="265"/>
+      <c r="K4" s="265"/>
+      <c r="L4" s="265"/>
+      <c r="M4" s="265"/>
+      <c r="N4" s="265"/>
+      <c r="O4" s="265"/>
+      <c r="P4" s="265"/>
+      <c r="Q4" s="265"/>
+      <c r="R4" s="265"/>
+      <c r="S4" s="265"/>
+      <c r="T4" s="265"/>
+      <c r="U4" s="265"/>
+      <c r="V4" s="265"/>
+      <c r="W4" s="265"/>
+      <c r="X4" s="265"/>
+      <c r="Y4" s="265"/>
+      <c r="Z4" s="265"/>
+      <c r="AA4" s="265"/>
+      <c r="AB4" s="265"/>
+      <c r="AC4" s="265"/>
+      <c r="AD4" s="265"/>
       <c r="AE4" s="8"/>
       <c r="AF4" s="6"/>
       <c r="AG4" s="6"/>
@@ -3801,33 +3803,33 @@
       <c r="C5" s="10"/>
       <c r="D5" s="10"/>
       <c r="E5" s="10"/>
-      <c r="F5" s="268" t="s">
+      <c r="F5" s="266" t="s">
         <v>3</v>
       </c>
-      <c r="G5" s="268"/>
-      <c r="H5" s="268"/>
-      <c r="I5" s="268"/>
-      <c r="J5" s="268"/>
-      <c r="K5" s="268"/>
-      <c r="L5" s="268"/>
-      <c r="M5" s="268"/>
-      <c r="N5" s="268"/>
-      <c r="O5" s="268"/>
-      <c r="P5" s="268"/>
-      <c r="Q5" s="268"/>
-      <c r="R5" s="268"/>
-      <c r="S5" s="268"/>
-      <c r="T5" s="268"/>
-      <c r="U5" s="268"/>
-      <c r="V5" s="268"/>
-      <c r="W5" s="268"/>
-      <c r="X5" s="268"/>
-      <c r="Y5" s="268"/>
-      <c r="Z5" s="268"/>
-      <c r="AA5" s="268"/>
-      <c r="AB5" s="268"/>
-      <c r="AC5" s="268"/>
-      <c r="AD5" s="268"/>
+      <c r="G5" s="266"/>
+      <c r="H5" s="266"/>
+      <c r="I5" s="266"/>
+      <c r="J5" s="266"/>
+      <c r="K5" s="266"/>
+      <c r="L5" s="266"/>
+      <c r="M5" s="266"/>
+      <c r="N5" s="266"/>
+      <c r="O5" s="266"/>
+      <c r="P5" s="266"/>
+      <c r="Q5" s="266"/>
+      <c r="R5" s="266"/>
+      <c r="S5" s="266"/>
+      <c r="T5" s="266"/>
+      <c r="U5" s="266"/>
+      <c r="V5" s="266"/>
+      <c r="W5" s="266"/>
+      <c r="X5" s="266"/>
+      <c r="Y5" s="266"/>
+      <c r="Z5" s="266"/>
+      <c r="AA5" s="266"/>
+      <c r="AB5" s="266"/>
+      <c r="AC5" s="266"/>
+      <c r="AD5" s="266"/>
       <c r="AE5" s="11"/>
       <c r="AF5" s="6"/>
       <c r="AG5" s="6"/>
@@ -3882,44 +3884,52 @@
     </row>
     <row r="8" spans="1:38" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2"/>
-      <c r="B8" s="269" t="s">
-        <v>165</v>
-      </c>
-      <c r="C8" s="269"/>
-      <c r="D8" s="269"/>
-      <c r="E8" s="269"/>
-      <c r="F8" s="269"/>
-      <c r="G8" s="269"/>
-      <c r="H8" s="269"/>
-      <c r="I8" s="269"/>
-      <c r="J8" s="269"/>
-      <c r="K8" s="269"/>
-      <c r="L8" s="269"/>
-      <c r="M8" s="269"/>
-      <c r="N8" s="270" t="s">
-        <v>166</v>
-      </c>
-      <c r="O8" s="270"/>
-      <c r="P8" s="270"/>
-      <c r="Q8" s="270"/>
-      <c r="R8" s="270"/>
-      <c r="S8" s="270"/>
-      <c r="T8" s="271" t="s">
-        <v>162</v>
-      </c>
-      <c r="U8" s="271"/>
-      <c r="V8" s="271"/>
-      <c r="W8" s="271"/>
-      <c r="X8" s="271"/>
-      <c r="Y8" s="271"/>
-      <c r="Z8" s="271"/>
-      <c r="AA8" s="271"/>
-      <c r="AB8" s="271"/>
-      <c r="AC8" s="272">
-        <v>46244</v>
-      </c>
-      <c r="AD8" s="272"/>
-      <c r="AE8" s="272"/>
+      <c r="B8" s="267" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="C8" s="267"/>
+      <c r="D8" s="267"/>
+      <c r="E8" s="267"/>
+      <c r="F8" s="267"/>
+      <c r="G8" s="267"/>
+      <c r="H8" s="267"/>
+      <c r="I8" s="267"/>
+      <c r="J8" s="267"/>
+      <c r="K8" s="267"/>
+      <c r="L8" s="267"/>
+      <c r="M8" s="267"/>
+      <c r="N8" s="268" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="O8" s="268"/>
+      <c r="P8" s="268"/>
+      <c r="Q8" s="268"/>
+      <c r="R8" s="268"/>
+      <c r="S8" s="268"/>
+      <c r="T8" s="269" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="U8" s="269"/>
+      <c r="V8" s="269"/>
+      <c r="W8" s="269"/>
+      <c r="X8" s="269"/>
+      <c r="Y8" s="269"/>
+      <c r="Z8" s="269"/>
+      <c r="AA8" s="269"/>
+      <c r="AB8" s="269"/>
+      <c r="AC8" s="270" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="AD8" s="270"/>
+      <c r="AE8" s="270"/>
       <c r="AF8" s="6"/>
       <c r="AG8" s="6"/>
       <c r="AH8" s="21"/>
@@ -3951,11 +3961,11 @@
       <c r="P9" s="29"/>
       <c r="Q9" s="29"/>
       <c r="R9" s="26"/>
-      <c r="S9" s="256" t="s">
+      <c r="S9" s="254" t="s">
         <v>12</v>
       </c>
-      <c r="T9" s="256"/>
-      <c r="U9" s="256"/>
+      <c r="T9" s="254"/>
+      <c r="U9" s="254"/>
       <c r="V9" s="30" t="s">
         <v>13</v>
       </c>
@@ -3975,95 +3985,105 @@
     </row>
     <row r="10" spans="1:38" s="20" customFormat="1" ht="8.4499999999999993" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
-      <c r="B10" s="257" t="s">
-        <v>170</v>
-      </c>
-      <c r="C10" s="257"/>
-      <c r="D10" s="257"/>
-      <c r="E10" s="258" t="s">
-        <v>171</v>
-      </c>
-      <c r="F10" s="258"/>
-      <c r="G10" s="258"/>
-      <c r="H10" s="258"/>
-      <c r="I10" s="258"/>
-      <c r="J10" s="258"/>
-      <c r="K10" s="259">
-        <v>7581.47</v>
-      </c>
-      <c r="L10" s="260"/>
-      <c r="M10" s="261"/>
-      <c r="N10" s="265">
+      <c r="B10" s="255" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="C10" s="255"/>
+      <c r="D10" s="255"/>
+      <c r="E10" s="256" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="F10" s="256"/>
+      <c r="G10" s="256"/>
+      <c r="H10" s="256"/>
+      <c r="I10" s="256"/>
+      <c r="J10" s="256"/>
+      <c r="K10" s="257" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="L10" s="258"/>
+      <c r="M10" s="259"/>
+      <c r="N10" s="263">
         <f>+K10/2</f>
         <v>3790.74</v>
       </c>
-      <c r="O10" s="265"/>
-      <c r="P10" s="265"/>
-      <c r="Q10" s="265"/>
-      <c r="R10" s="265"/>
+      <c r="O10" s="263"/>
+      <c r="P10" s="263"/>
+      <c r="Q10" s="263"/>
+      <c r="R10" s="263"/>
       <c r="S10" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="T10" s="256" t="s">
+      <c r="T10" s="254" t="s">
         <v>17</v>
       </c>
-      <c r="U10" s="256"/>
-      <c r="V10" s="247">
-        <v>38.42</v>
-      </c>
-      <c r="W10" s="247"/>
-      <c r="X10" s="247"/>
-      <c r="Y10" s="247"/>
-      <c r="Z10" s="248">
-        <v>7</v>
-      </c>
-      <c r="AA10" s="249" t="s">
+      <c r="U10" s="254"/>
+      <c r="V10" s="248" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="W10" s="248"/>
+      <c r="X10" s="248"/>
+      <c r="Y10" s="248"/>
+      <c r="Z10" s="249" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="AA10" s="250" t="s">
         <v>18</v>
       </c>
-      <c r="AB10" s="249"/>
-      <c r="AC10" s="250">
+      <c r="AB10" s="250"/>
+      <c r="AC10" s="251">
         <f>+Z10*V10</f>
         <v>268.94</v>
       </c>
-      <c r="AD10" s="250"/>
-      <c r="AE10" s="250"/>
+      <c r="AD10" s="251"/>
+      <c r="AE10" s="251"/>
       <c r="AF10" s="6"/>
       <c r="AG10" s="6"/>
     </row>
     <row r="11" spans="1:38" ht="11.1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
-      <c r="B11" s="257"/>
-      <c r="C11" s="257"/>
-      <c r="D11" s="257"/>
-      <c r="E11" s="258"/>
-      <c r="F11" s="258"/>
-      <c r="G11" s="258"/>
-      <c r="H11" s="258"/>
-      <c r="I11" s="258"/>
-      <c r="J11" s="258"/>
-      <c r="K11" s="262"/>
-      <c r="L11" s="263"/>
-      <c r="M11" s="264"/>
-      <c r="N11" s="265"/>
-      <c r="O11" s="265"/>
-      <c r="P11" s="265"/>
-      <c r="Q11" s="265"/>
-      <c r="R11" s="265"/>
+      <c r="B11" s="255"/>
+      <c r="C11" s="255"/>
+      <c r="D11" s="255"/>
+      <c r="E11" s="256"/>
+      <c r="F11" s="256"/>
+      <c r="G11" s="256"/>
+      <c r="H11" s="256"/>
+      <c r="I11" s="256"/>
+      <c r="J11" s="256"/>
+      <c r="K11" s="260"/>
+      <c r="L11" s="261"/>
+      <c r="M11" s="262"/>
+      <c r="N11" s="263"/>
+      <c r="O11" s="263"/>
+      <c r="P11" s="263"/>
+      <c r="Q11" s="263"/>
+      <c r="R11" s="263"/>
       <c r="S11" s="35"/>
-      <c r="T11" s="251" t="s">
+      <c r="T11" s="252" t="s">
         <v>19</v>
       </c>
-      <c r="U11" s="251"/>
-      <c r="V11" s="247"/>
-      <c r="W11" s="247"/>
-      <c r="X11" s="247"/>
-      <c r="Y11" s="247"/>
-      <c r="Z11" s="248"/>
-      <c r="AA11" s="249"/>
-      <c r="AB11" s="249"/>
-      <c r="AC11" s="250"/>
-      <c r="AD11" s="250"/>
-      <c r="AE11" s="250"/>
+      <c r="U11" s="252"/>
+      <c r="V11" s="248"/>
+      <c r="W11" s="248"/>
+      <c r="X11" s="248"/>
+      <c r="Y11" s="248"/>
+      <c r="Z11" s="249"/>
+      <c r="AA11" s="250"/>
+      <c r="AB11" s="250"/>
+      <c r="AC11" s="251"/>
+      <c r="AD11" s="251"/>
+      <c r="AE11" s="251"/>
       <c r="AF11" s="6"/>
       <c r="AG11" s="6"/>
     </row>
@@ -4105,48 +4125,48 @@
     </row>
     <row r="13" spans="1:38" s="45" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="2"/>
-      <c r="B13" s="252" t="s">
+      <c r="B13" s="242" t="s">
         <v>20</v>
       </c>
-      <c r="C13" s="252"/>
-      <c r="D13" s="252"/>
-      <c r="E13" s="252"/>
+      <c r="C13" s="242"/>
+      <c r="D13" s="242"/>
+      <c r="E13" s="242"/>
       <c r="F13" s="43" t="s">
         <v>21</v>
       </c>
-      <c r="G13" s="253" t="s">
+      <c r="G13" s="243" t="s">
         <v>22</v>
       </c>
-      <c r="H13" s="253"/>
-      <c r="I13" s="253"/>
-      <c r="J13" s="254" t="s">
+      <c r="H13" s="243"/>
+      <c r="I13" s="243"/>
+      <c r="J13" s="244" t="s">
         <v>23</v>
       </c>
-      <c r="K13" s="254"/>
-      <c r="L13" s="254" t="s">
+      <c r="K13" s="244"/>
+      <c r="L13" s="244" t="s">
         <v>24</v>
       </c>
-      <c r="M13" s="254"/>
-      <c r="N13" s="254"/>
-      <c r="O13" s="254"/>
-      <c r="P13" s="255" t="s">
+      <c r="M13" s="244"/>
+      <c r="N13" s="244"/>
+      <c r="O13" s="244"/>
+      <c r="P13" s="253" t="s">
         <v>25</v>
       </c>
-      <c r="Q13" s="255"/>
-      <c r="R13" s="255"/>
-      <c r="S13" s="255"/>
-      <c r="T13" s="255"/>
-      <c r="U13" s="255"/>
-      <c r="V13" s="255"/>
-      <c r="W13" s="255"/>
-      <c r="X13" s="255"/>
-      <c r="Y13" s="255"/>
-      <c r="Z13" s="255"/>
-      <c r="AA13" s="255"/>
-      <c r="AB13" s="255"/>
-      <c r="AC13" s="255"/>
-      <c r="AD13" s="255"/>
-      <c r="AE13" s="244" t="s">
+      <c r="Q13" s="253"/>
+      <c r="R13" s="253"/>
+      <c r="S13" s="253"/>
+      <c r="T13" s="253"/>
+      <c r="U13" s="253"/>
+      <c r="V13" s="253"/>
+      <c r="W13" s="253"/>
+      <c r="X13" s="253"/>
+      <c r="Y13" s="253"/>
+      <c r="Z13" s="253"/>
+      <c r="AA13" s="253"/>
+      <c r="AB13" s="253"/>
+      <c r="AC13" s="253"/>
+      <c r="AD13" s="253"/>
+      <c r="AE13" s="245" t="s">
         <v>26</v>
       </c>
       <c r="AF13" s="6"/>
@@ -4155,66 +4175,66 @@
     </row>
     <row r="14" spans="1:38" s="45" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="2"/>
-      <c r="B14" s="252"/>
-      <c r="C14" s="252"/>
-      <c r="D14" s="252"/>
-      <c r="E14" s="252"/>
+      <c r="B14" s="242"/>
+      <c r="C14" s="242"/>
+      <c r="D14" s="242"/>
+      <c r="E14" s="242"/>
       <c r="F14" s="46" t="s">
         <v>27</v>
       </c>
-      <c r="G14" s="253"/>
-      <c r="H14" s="253"/>
-      <c r="I14" s="253"/>
-      <c r="J14" s="254"/>
-      <c r="K14" s="254"/>
-      <c r="L14" s="254"/>
-      <c r="M14" s="254"/>
-      <c r="N14" s="254"/>
-      <c r="O14" s="254"/>
-      <c r="P14" s="245" t="s">
+      <c r="G14" s="243"/>
+      <c r="H14" s="243"/>
+      <c r="I14" s="243"/>
+      <c r="J14" s="244"/>
+      <c r="K14" s="244"/>
+      <c r="L14" s="244"/>
+      <c r="M14" s="244"/>
+      <c r="N14" s="244"/>
+      <c r="O14" s="244"/>
+      <c r="P14" s="246" t="s">
         <v>28</v>
       </c>
-      <c r="Q14" s="245" t="s">
+      <c r="Q14" s="246" t="s">
         <v>29</v>
       </c>
-      <c r="R14" s="245" t="s">
+      <c r="R14" s="246" t="s">
         <v>30</v>
       </c>
-      <c r="S14" s="245"/>
-      <c r="T14" s="245"/>
-      <c r="U14" s="245"/>
-      <c r="V14" s="245"/>
-      <c r="W14" s="245" t="s">
+      <c r="S14" s="246"/>
+      <c r="T14" s="246"/>
+      <c r="U14" s="246"/>
+      <c r="V14" s="246"/>
+      <c r="W14" s="246" t="s">
         <v>31</v>
       </c>
-      <c r="X14" s="245"/>
-      <c r="Y14" s="245"/>
-      <c r="Z14" s="245"/>
-      <c r="AA14" s="245"/>
-      <c r="AB14" s="245"/>
-      <c r="AC14" s="245" t="s">
+      <c r="X14" s="246"/>
+      <c r="Y14" s="246"/>
+      <c r="Z14" s="246"/>
+      <c r="AA14" s="246"/>
+      <c r="AB14" s="246"/>
+      <c r="AC14" s="246" t="s">
         <v>28</v>
       </c>
-      <c r="AD14" s="246" t="s">
+      <c r="AD14" s="247" t="s">
         <v>32</v>
       </c>
-      <c r="AE14" s="244"/>
+      <c r="AE14" s="245"/>
       <c r="AF14" s="6"/>
       <c r="AG14" s="6"/>
       <c r="AH14" s="47"/>
     </row>
     <row r="15" spans="1:38" s="57" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="48"/>
-      <c r="B15" s="252"/>
-      <c r="C15" s="252"/>
-      <c r="D15" s="252"/>
-      <c r="E15" s="252"/>
+      <c r="B15" s="242"/>
+      <c r="C15" s="242"/>
+      <c r="D15" s="242"/>
+      <c r="E15" s="242"/>
       <c r="F15" s="49" t="s">
         <v>31</v>
       </c>
-      <c r="G15" s="253"/>
-      <c r="H15" s="253"/>
-      <c r="I15" s="253"/>
+      <c r="G15" s="243"/>
+      <c r="H15" s="243"/>
+      <c r="I15" s="243"/>
       <c r="J15" s="52" t="s">
         <v>33</v>
       </c>
@@ -4224,13 +4244,13 @@
       <c r="L15" s="51" t="s">
         <v>33</v>
       </c>
-      <c r="M15" s="240" t="s">
+      <c r="M15" s="238" t="s">
         <v>34</v>
       </c>
-      <c r="N15" s="240"/>
-      <c r="O15" s="240"/>
-      <c r="P15" s="245"/>
-      <c r="Q15" s="245"/>
+      <c r="N15" s="238"/>
+      <c r="O15" s="238"/>
+      <c r="P15" s="246"/>
+      <c r="Q15" s="246"/>
       <c r="R15" s="52" t="s">
         <v>28</v>
       </c>
@@ -4240,27 +4260,27 @@
       <c r="T15" s="52" t="s">
         <v>28</v>
       </c>
-      <c r="U15" s="240" t="s">
+      <c r="U15" s="238" t="s">
         <v>36</v>
       </c>
-      <c r="V15" s="240"/>
+      <c r="V15" s="238"/>
       <c r="W15" s="52" t="s">
         <v>28</v>
       </c>
-      <c r="X15" s="240" t="s">
+      <c r="X15" s="238" t="s">
         <v>37</v>
       </c>
-      <c r="Y15" s="240"/>
+      <c r="Y15" s="238"/>
       <c r="Z15" s="52" t="s">
         <v>28</v>
       </c>
-      <c r="AA15" s="240" t="s">
+      <c r="AA15" s="238" t="s">
         <v>38</v>
       </c>
-      <c r="AB15" s="240"/>
-      <c r="AC15" s="245"/>
-      <c r="AD15" s="246"/>
-      <c r="AE15" s="244"/>
+      <c r="AB15" s="238"/>
+      <c r="AC15" s="246"/>
+      <c r="AD15" s="247"/>
+      <c r="AE15" s="245"/>
       <c r="AF15" s="53"/>
       <c r="AG15" s="53"/>
       <c r="AH15" s="54"/>
@@ -4271,34 +4291,46 @@
     </row>
     <row r="16" spans="1:38" s="38" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A16" s="2"/>
-      <c r="B16" s="241" t="s">
-        <v>169</v>
-      </c>
-      <c r="C16" s="241"/>
-      <c r="D16" s="241"/>
-      <c r="E16" s="241"/>
+      <c r="B16" s="239" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="C16" s="239"/>
+      <c r="D16" s="239"/>
+      <c r="E16" s="239"/>
       <c r="F16" s="58">
         <v>5</v>
       </c>
-      <c r="G16" s="242" t="s">
-        <v>172</v>
-      </c>
-      <c r="H16" s="242"/>
-      <c r="I16" s="242"/>
-      <c r="J16" s="59">
-        <v>12</v>
-      </c>
-      <c r="K16" s="60">
-        <v>0.72916666666666696</v>
-      </c>
-      <c r="L16" s="61">
-        <v>13</v>
-      </c>
-      <c r="M16" s="237">
-        <v>0.35416666666666702</v>
-      </c>
-      <c r="N16" s="237"/>
-      <c r="O16" s="237"/>
+      <c r="G16" s="240" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="H16" s="240"/>
+      <c r="I16" s="240"/>
+      <c r="J16" s="59" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="K16" s="60" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="L16" s="61" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="M16" s="235" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="N16" s="235"/>
+      <c r="O16" s="235"/>
       <c r="P16" s="62"/>
       <c r="Q16" s="63">
         <f t="shared" ref="Q16:Q27" si="0">IF(P16="",0,VLOOKUP(F16,AN$107:AZ$111,3,FALSE)*P16)</f>
@@ -4310,28 +4342,34 @@
         <v>0</v>
       </c>
       <c r="T16" s="61"/>
-      <c r="U16" s="243">
+      <c r="U16" s="241">
         <f t="shared" ref="U16:U27" si="2">IF(T16="",0,VLOOKUP(F16,AN$107:AZ$111,7,FALSE)*T16)</f>
         <v>0</v>
       </c>
-      <c r="V16" s="243" t="e">
+      <c r="V16" s="241" t="e">
         <f t="shared" ref="V16:V27" si="3">IF(U16="",0,VLOOKUP(J$16,AT$107:AV$111,3,FALSE)*U16)</f>
         <v>#N/A</v>
       </c>
-      <c r="W16" s="61">
-        <v>0</v>
-      </c>
-      <c r="X16" s="243">
+      <c r="W16" s="61" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="X16" s="241">
         <f>IF(W16="",0,VLOOKUP(F16,AN$107:AZ$111,9,FALSE)*W16)</f>
-        <v>0</v>
-      </c>
-      <c r="Y16" s="243"/>
-      <c r="Z16" s="61"/>
-      <c r="AA16" s="239">
+        <v>53.78</v>
+      </c>
+      <c r="Y16" s="241"/>
+      <c r="Z16" s="61" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="AA16" s="237">
         <f>IF(Z16="",0,VLOOKUP(F16,AN$107:AZ$111,11,FALSE)*Z16)</f>
         <v>0</v>
       </c>
-      <c r="AB16" s="239"/>
+      <c r="AB16" s="237"/>
       <c r="AC16" s="59"/>
       <c r="AD16" s="63">
         <f t="shared" ref="AD16:AD27" si="4">IF(AC16="",0,VLOOKUP(F16,AN$107:AZ$111,13,FALSE)*AC16)</f>
@@ -4339,7 +4377,7 @@
       </c>
       <c r="AE16" s="64">
         <f t="shared" ref="AE16:AE27" si="5">+Q16+S16+U16+X16+AA16+AD16</f>
-        <v>0</v>
+        <v>53.78</v>
       </c>
       <c r="AF16" s="6"/>
       <c r="AG16" s="6"/>
@@ -4351,20 +4389,20 @@
     </row>
     <row r="17" spans="1:38" s="38" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A17" s="2"/>
-      <c r="B17" s="235"/>
-      <c r="C17" s="235"/>
-      <c r="D17" s="235"/>
-      <c r="E17" s="235"/>
+      <c r="B17" s="233"/>
+      <c r="C17" s="233"/>
+      <c r="D17" s="233"/>
+      <c r="E17" s="233"/>
       <c r="F17" s="58"/>
-      <c r="G17" s="236"/>
-      <c r="H17" s="236"/>
-      <c r="I17" s="236"/>
+      <c r="G17" s="234"/>
+      <c r="H17" s="234"/>
+      <c r="I17" s="234"/>
       <c r="J17" s="69"/>
       <c r="K17" s="60"/>
       <c r="L17" s="70"/>
-      <c r="M17" s="237"/>
-      <c r="N17" s="237"/>
-      <c r="O17" s="237"/>
+      <c r="M17" s="235"/>
+      <c r="N17" s="235"/>
+      <c r="O17" s="235"/>
       <c r="P17" s="70"/>
       <c r="Q17" s="71">
         <f t="shared" si="0"/>
@@ -4376,26 +4414,26 @@
         <v>0</v>
       </c>
       <c r="T17" s="70"/>
-      <c r="U17" s="239">
+      <c r="U17" s="237">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="V17" s="239" t="e">
+      <c r="V17" s="237" t="e">
         <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="W17" s="70"/>
-      <c r="X17" s="239">
+      <c r="X17" s="237">
         <f t="shared" ref="X17:X27" si="6">IF(W17="",0,VLOOKUP(F17,AN$107:AZ$111,9,FALSE)*W17)</f>
         <v>0</v>
       </c>
-      <c r="Y17" s="239"/>
+      <c r="Y17" s="237"/>
       <c r="Z17" s="70"/>
-      <c r="AA17" s="239">
+      <c r="AA17" s="237">
         <f t="shared" ref="AA17:AA27" si="7">IF(Z17="",0,VLOOKUP(F17,AN$107:AZ$111,11,FALSE)*Z17)</f>
         <v>0</v>
       </c>
-      <c r="AB17" s="239"/>
+      <c r="AB17" s="237"/>
       <c r="AC17" s="70"/>
       <c r="AD17" s="71">
         <f t="shared" si="4"/>
@@ -4415,20 +4453,20 @@
     </row>
     <row r="18" spans="1:38" s="38" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A18" s="2"/>
-      <c r="B18" s="235"/>
-      <c r="C18" s="235"/>
-      <c r="D18" s="235"/>
-      <c r="E18" s="235"/>
+      <c r="B18" s="233"/>
+      <c r="C18" s="233"/>
+      <c r="D18" s="233"/>
+      <c r="E18" s="233"/>
       <c r="F18" s="58"/>
-      <c r="G18" s="236"/>
-      <c r="H18" s="236"/>
-      <c r="I18" s="236"/>
+      <c r="G18" s="234"/>
+      <c r="H18" s="234"/>
+      <c r="I18" s="234"/>
       <c r="J18" s="69"/>
       <c r="K18" s="60"/>
       <c r="L18" s="70"/>
-      <c r="M18" s="237"/>
-      <c r="N18" s="237"/>
-      <c r="O18" s="237"/>
+      <c r="M18" s="235"/>
+      <c r="N18" s="235"/>
+      <c r="O18" s="235"/>
       <c r="P18" s="70"/>
       <c r="Q18" s="71">
         <f t="shared" si="0"/>
@@ -4440,26 +4478,26 @@
         <v>0</v>
       </c>
       <c r="T18" s="70"/>
-      <c r="U18" s="239">
+      <c r="U18" s="237">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="V18" s="239" t="e">
+      <c r="V18" s="237" t="e">
         <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="W18" s="70"/>
-      <c r="X18" s="239">
+      <c r="X18" s="237">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="Y18" s="239"/>
+      <c r="Y18" s="237"/>
       <c r="Z18" s="70"/>
-      <c r="AA18" s="239">
+      <c r="AA18" s="237">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="AB18" s="239"/>
+      <c r="AB18" s="237"/>
       <c r="AC18" s="70"/>
       <c r="AD18" s="71">
         <f t="shared" si="4"/>
@@ -4479,20 +4517,20 @@
     </row>
     <row r="19" spans="1:38" s="38" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A19" s="2"/>
-      <c r="B19" s="235"/>
-      <c r="C19" s="235"/>
-      <c r="D19" s="235"/>
-      <c r="E19" s="235"/>
+      <c r="B19" s="233"/>
+      <c r="C19" s="233"/>
+      <c r="D19" s="233"/>
+      <c r="E19" s="233"/>
       <c r="F19" s="58"/>
-      <c r="G19" s="236"/>
-      <c r="H19" s="236"/>
-      <c r="I19" s="236"/>
+      <c r="G19" s="234"/>
+      <c r="H19" s="234"/>
+      <c r="I19" s="234"/>
       <c r="J19" s="69"/>
       <c r="K19" s="60"/>
       <c r="L19" s="70"/>
-      <c r="M19" s="237"/>
-      <c r="N19" s="237"/>
-      <c r="O19" s="237"/>
+      <c r="M19" s="235"/>
+      <c r="N19" s="235"/>
+      <c r="O19" s="235"/>
       <c r="P19" s="70"/>
       <c r="Q19" s="71">
         <f t="shared" si="0"/>
@@ -4504,26 +4542,26 @@
         <v>0</v>
       </c>
       <c r="T19" s="70"/>
-      <c r="U19" s="239">
+      <c r="U19" s="237">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="V19" s="239" t="e">
+      <c r="V19" s="237" t="e">
         <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="W19" s="70"/>
-      <c r="X19" s="239">
+      <c r="X19" s="237">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="Y19" s="239"/>
+      <c r="Y19" s="237"/>
       <c r="Z19" s="70"/>
-      <c r="AA19" s="239">
+      <c r="AA19" s="237">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="AB19" s="239"/>
+      <c r="AB19" s="237"/>
       <c r="AC19" s="70"/>
       <c r="AD19" s="71">
         <f t="shared" si="4"/>
@@ -4543,20 +4581,20 @@
     </row>
     <row r="20" spans="1:38" s="38" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A20" s="2"/>
-      <c r="B20" s="235"/>
-      <c r="C20" s="235"/>
-      <c r="D20" s="235"/>
-      <c r="E20" s="235"/>
+      <c r="B20" s="233"/>
+      <c r="C20" s="233"/>
+      <c r="D20" s="233"/>
+      <c r="E20" s="233"/>
       <c r="F20" s="58"/>
-      <c r="G20" s="236"/>
-      <c r="H20" s="236"/>
-      <c r="I20" s="236"/>
+      <c r="G20" s="234"/>
+      <c r="H20" s="234"/>
+      <c r="I20" s="234"/>
       <c r="J20" s="70"/>
       <c r="K20" s="60"/>
       <c r="L20" s="70"/>
-      <c r="M20" s="237"/>
-      <c r="N20" s="237"/>
-      <c r="O20" s="237"/>
+      <c r="M20" s="235"/>
+      <c r="N20" s="235"/>
+      <c r="O20" s="235"/>
       <c r="P20" s="70"/>
       <c r="Q20" s="71">
         <f t="shared" si="0"/>
@@ -4568,26 +4606,26 @@
         <v>0</v>
       </c>
       <c r="T20" s="70"/>
-      <c r="U20" s="239">
+      <c r="U20" s="237">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="V20" s="239" t="e">
+      <c r="V20" s="237" t="e">
         <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="W20" s="70"/>
-      <c r="X20" s="239">
+      <c r="X20" s="237">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="Y20" s="239"/>
+      <c r="Y20" s="237"/>
       <c r="Z20" s="70"/>
-      <c r="AA20" s="239">
+      <c r="AA20" s="237">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="AB20" s="239"/>
+      <c r="AB20" s="237"/>
       <c r="AC20" s="70"/>
       <c r="AD20" s="71">
         <f t="shared" si="4"/>
@@ -4607,20 +4645,20 @@
     </row>
     <row r="21" spans="1:38" s="38" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A21" s="2"/>
-      <c r="B21" s="235"/>
-      <c r="C21" s="235"/>
-      <c r="D21" s="235"/>
-      <c r="E21" s="235"/>
+      <c r="B21" s="233"/>
+      <c r="C21" s="233"/>
+      <c r="D21" s="233"/>
+      <c r="E21" s="233"/>
       <c r="F21" s="58"/>
-      <c r="G21" s="236"/>
-      <c r="H21" s="236"/>
-      <c r="I21" s="236"/>
+      <c r="G21" s="234"/>
+      <c r="H21" s="234"/>
+      <c r="I21" s="234"/>
       <c r="J21" s="70"/>
       <c r="K21" s="60"/>
       <c r="L21" s="70"/>
-      <c r="M21" s="237"/>
-      <c r="N21" s="237"/>
-      <c r="O21" s="237"/>
+      <c r="M21" s="235"/>
+      <c r="N21" s="235"/>
+      <c r="O21" s="235"/>
       <c r="P21" s="70"/>
       <c r="Q21" s="71">
         <f t="shared" si="0"/>
@@ -4632,26 +4670,26 @@
         <v>0</v>
       </c>
       <c r="T21" s="70"/>
-      <c r="U21" s="239">
+      <c r="U21" s="237">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="V21" s="239" t="e">
+      <c r="V21" s="237" t="e">
         <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="W21" s="70"/>
-      <c r="X21" s="239">
+      <c r="X21" s="237">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="Y21" s="239"/>
+      <c r="Y21" s="237"/>
       <c r="Z21" s="70"/>
-      <c r="AA21" s="239">
+      <c r="AA21" s="237">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="AB21" s="239"/>
+      <c r="AB21" s="237"/>
       <c r="AC21" s="70"/>
       <c r="AD21" s="71">
         <f t="shared" si="4"/>
@@ -4671,20 +4709,20 @@
     </row>
     <row r="22" spans="1:38" s="38" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A22" s="2"/>
-      <c r="B22" s="235"/>
-      <c r="C22" s="235"/>
-      <c r="D22" s="235"/>
-      <c r="E22" s="235"/>
+      <c r="B22" s="233"/>
+      <c r="C22" s="233"/>
+      <c r="D22" s="233"/>
+      <c r="E22" s="233"/>
       <c r="F22" s="58"/>
-      <c r="G22" s="236"/>
-      <c r="H22" s="236"/>
-      <c r="I22" s="236"/>
+      <c r="G22" s="234"/>
+      <c r="H22" s="234"/>
+      <c r="I22" s="234"/>
       <c r="J22" s="70"/>
       <c r="K22" s="60"/>
       <c r="L22" s="70"/>
-      <c r="M22" s="237"/>
-      <c r="N22" s="237"/>
-      <c r="O22" s="237"/>
+      <c r="M22" s="235"/>
+      <c r="N22" s="235"/>
+      <c r="O22" s="235"/>
       <c r="P22" s="70"/>
       <c r="Q22" s="71">
         <f t="shared" si="0"/>
@@ -4696,26 +4734,26 @@
         <v>0</v>
       </c>
       <c r="T22" s="70"/>
-      <c r="U22" s="239">
+      <c r="U22" s="237">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="V22" s="239" t="e">
+      <c r="V22" s="237" t="e">
         <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="W22" s="70"/>
-      <c r="X22" s="239">
+      <c r="X22" s="237">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="Y22" s="239"/>
+      <c r="Y22" s="237"/>
       <c r="Z22" s="70"/>
-      <c r="AA22" s="239">
+      <c r="AA22" s="237">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="AB22" s="239"/>
+      <c r="AB22" s="237"/>
       <c r="AC22" s="69"/>
       <c r="AD22" s="71">
         <f t="shared" si="4"/>
@@ -4735,20 +4773,20 @@
     </row>
     <row r="23" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A23" s="2"/>
-      <c r="B23" s="235"/>
-      <c r="C23" s="235"/>
-      <c r="D23" s="235"/>
-      <c r="E23" s="235"/>
+      <c r="B23" s="233"/>
+      <c r="C23" s="233"/>
+      <c r="D23" s="233"/>
+      <c r="E23" s="233"/>
       <c r="F23" s="58"/>
-      <c r="G23" s="236"/>
-      <c r="H23" s="236"/>
-      <c r="I23" s="236"/>
+      <c r="G23" s="234"/>
+      <c r="H23" s="234"/>
+      <c r="I23" s="234"/>
       <c r="J23" s="75"/>
       <c r="K23" s="60"/>
       <c r="L23" s="70"/>
-      <c r="M23" s="237"/>
-      <c r="N23" s="237"/>
-      <c r="O23" s="237"/>
+      <c r="M23" s="235"/>
+      <c r="N23" s="235"/>
+      <c r="O23" s="235"/>
       <c r="P23" s="70"/>
       <c r="Q23" s="71">
         <f t="shared" si="0"/>
@@ -4760,26 +4798,26 @@
         <v>0</v>
       </c>
       <c r="T23" s="75"/>
-      <c r="U23" s="239">
+      <c r="U23" s="237">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="V23" s="239" t="e">
+      <c r="V23" s="237" t="e">
         <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="W23" s="75"/>
-      <c r="X23" s="239">
+      <c r="X23" s="237">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="Y23" s="239"/>
+      <c r="Y23" s="237"/>
       <c r="Z23" s="75"/>
-      <c r="AA23" s="239">
+      <c r="AA23" s="237">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="AB23" s="239"/>
+      <c r="AB23" s="237"/>
       <c r="AC23" s="76"/>
       <c r="AD23" s="71">
         <f t="shared" si="4"/>
@@ -4797,20 +4835,20 @@
     </row>
     <row r="24" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A24" s="2"/>
-      <c r="B24" s="235"/>
-      <c r="C24" s="235"/>
-      <c r="D24" s="235"/>
-      <c r="E24" s="235"/>
+      <c r="B24" s="233"/>
+      <c r="C24" s="233"/>
+      <c r="D24" s="233"/>
+      <c r="E24" s="233"/>
       <c r="F24" s="58"/>
-      <c r="G24" s="236"/>
-      <c r="H24" s="236"/>
-      <c r="I24" s="236"/>
+      <c r="G24" s="234"/>
+      <c r="H24" s="234"/>
+      <c r="I24" s="234"/>
       <c r="J24" s="75"/>
       <c r="K24" s="60"/>
       <c r="L24" s="70"/>
-      <c r="M24" s="237"/>
-      <c r="N24" s="237"/>
-      <c r="O24" s="237"/>
+      <c r="M24" s="235"/>
+      <c r="N24" s="235"/>
+      <c r="O24" s="235"/>
       <c r="P24" s="70"/>
       <c r="Q24" s="71">
         <f t="shared" si="0"/>
@@ -4822,26 +4860,26 @@
         <v>0</v>
       </c>
       <c r="T24" s="75"/>
-      <c r="U24" s="239">
+      <c r="U24" s="237">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="V24" s="239" t="e">
+      <c r="V24" s="237" t="e">
         <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="W24" s="75"/>
-      <c r="X24" s="239">
+      <c r="X24" s="237">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="Y24" s="239"/>
+      <c r="Y24" s="237"/>
       <c r="Z24" s="75"/>
-      <c r="AA24" s="239">
+      <c r="AA24" s="237">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="AB24" s="239"/>
+      <c r="AB24" s="237"/>
       <c r="AC24" s="76"/>
       <c r="AD24" s="71">
         <f t="shared" si="4"/>
@@ -4859,20 +4897,20 @@
     </row>
     <row r="25" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A25" s="2"/>
-      <c r="B25" s="235"/>
-      <c r="C25" s="235"/>
-      <c r="D25" s="235"/>
-      <c r="E25" s="235"/>
+      <c r="B25" s="233"/>
+      <c r="C25" s="233"/>
+      <c r="D25" s="233"/>
+      <c r="E25" s="233"/>
       <c r="F25" s="58"/>
-      <c r="G25" s="236"/>
-      <c r="H25" s="236"/>
-      <c r="I25" s="236"/>
+      <c r="G25" s="234"/>
+      <c r="H25" s="234"/>
+      <c r="I25" s="234"/>
       <c r="J25" s="75"/>
       <c r="K25" s="60"/>
       <c r="L25" s="70"/>
-      <c r="M25" s="237"/>
-      <c r="N25" s="237"/>
-      <c r="O25" s="237"/>
+      <c r="M25" s="235"/>
+      <c r="N25" s="235"/>
+      <c r="O25" s="235"/>
       <c r="P25" s="70"/>
       <c r="Q25" s="71">
         <f t="shared" si="0"/>
@@ -4884,26 +4922,26 @@
         <v>0</v>
       </c>
       <c r="T25" s="75"/>
-      <c r="U25" s="239">
+      <c r="U25" s="237">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="V25" s="239" t="e">
+      <c r="V25" s="237" t="e">
         <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="W25" s="75"/>
-      <c r="X25" s="239">
+      <c r="X25" s="237">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="Y25" s="239"/>
+      <c r="Y25" s="237"/>
       <c r="Z25" s="75"/>
-      <c r="AA25" s="239">
+      <c r="AA25" s="237">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="AB25" s="239"/>
+      <c r="AB25" s="237"/>
       <c r="AC25" s="76"/>
       <c r="AD25" s="71">
         <f t="shared" si="4"/>
@@ -4921,20 +4959,20 @@
     </row>
     <row r="26" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A26" s="2"/>
-      <c r="B26" s="235"/>
-      <c r="C26" s="235"/>
-      <c r="D26" s="235"/>
-      <c r="E26" s="235"/>
+      <c r="B26" s="233"/>
+      <c r="C26" s="233"/>
+      <c r="D26" s="233"/>
+      <c r="E26" s="233"/>
       <c r="F26" s="58"/>
-      <c r="G26" s="236"/>
-      <c r="H26" s="236"/>
-      <c r="I26" s="236"/>
+      <c r="G26" s="234"/>
+      <c r="H26" s="234"/>
+      <c r="I26" s="234"/>
       <c r="J26" s="75"/>
       <c r="K26" s="60"/>
       <c r="L26" s="70"/>
-      <c r="M26" s="237"/>
-      <c r="N26" s="237"/>
-      <c r="O26" s="237"/>
+      <c r="M26" s="235"/>
+      <c r="N26" s="235"/>
+      <c r="O26" s="235"/>
       <c r="P26" s="70"/>
       <c r="Q26" s="71">
         <f t="shared" si="0"/>
@@ -4946,26 +4984,26 @@
         <v>0</v>
       </c>
       <c r="T26" s="75"/>
-      <c r="U26" s="239">
+      <c r="U26" s="237">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="V26" s="239" t="e">
+      <c r="V26" s="237" t="e">
         <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="W26" s="75"/>
-      <c r="X26" s="239">
+      <c r="X26" s="237">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="Y26" s="239"/>
+      <c r="Y26" s="237"/>
       <c r="Z26" s="75"/>
-      <c r="AA26" s="239">
+      <c r="AA26" s="237">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="AB26" s="239"/>
+      <c r="AB26" s="237"/>
       <c r="AC26" s="76"/>
       <c r="AD26" s="71">
         <f t="shared" si="4"/>
@@ -4983,20 +5021,20 @@
     </row>
     <row r="27" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A27" s="2"/>
-      <c r="B27" s="235"/>
-      <c r="C27" s="235"/>
-      <c r="D27" s="235"/>
-      <c r="E27" s="235"/>
+      <c r="B27" s="233"/>
+      <c r="C27" s="233"/>
+      <c r="D27" s="233"/>
+      <c r="E27" s="233"/>
       <c r="F27" s="58"/>
-      <c r="G27" s="236"/>
-      <c r="H27" s="236"/>
-      <c r="I27" s="236"/>
+      <c r="G27" s="234"/>
+      <c r="H27" s="234"/>
+      <c r="I27" s="234"/>
       <c r="J27" s="75"/>
       <c r="K27" s="60"/>
       <c r="L27" s="70"/>
-      <c r="M27" s="237"/>
-      <c r="N27" s="237"/>
-      <c r="O27" s="237"/>
+      <c r="M27" s="235"/>
+      <c r="N27" s="235"/>
+      <c r="O27" s="235"/>
       <c r="P27" s="70"/>
       <c r="Q27" s="80">
         <f t="shared" si="0"/>
@@ -5008,26 +5046,26 @@
         <v>0</v>
       </c>
       <c r="T27" s="81"/>
-      <c r="U27" s="238">
+      <c r="U27" s="236">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="V27" s="238" t="e">
+      <c r="V27" s="236" t="e">
         <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="W27" s="81"/>
-      <c r="X27" s="238">
+      <c r="X27" s="236">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="Y27" s="238"/>
+      <c r="Y27" s="236"/>
       <c r="Z27" s="81"/>
-      <c r="AA27" s="238">
+      <c r="AA27" s="236">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="AB27" s="238"/>
+      <c r="AB27" s="236"/>
       <c r="AC27" s="82"/>
       <c r="AD27" s="80">
         <f t="shared" si="4"/>
@@ -5045,47 +5083,51 @@
     </row>
     <row r="28" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A28" s="2"/>
-      <c r="B28" s="230" t="s">
+      <c r="B28" s="224" t="s">
         <v>39</v>
       </c>
-      <c r="C28" s="230"/>
-      <c r="D28" s="230"/>
-      <c r="E28" s="230"/>
-      <c r="F28" s="230"/>
-      <c r="G28" s="230"/>
-      <c r="H28" s="231" t="s">
+      <c r="C28" s="224"/>
+      <c r="D28" s="224"/>
+      <c r="E28" s="224"/>
+      <c r="F28" s="224"/>
+      <c r="G28" s="224"/>
+      <c r="H28" s="225" t="s">
         <v>40</v>
       </c>
-      <c r="I28" s="231"/>
-      <c r="J28" s="232" t="s">
-        <v>167</v>
-      </c>
-      <c r="K28" s="232"/>
-      <c r="L28" s="232"/>
-      <c r="M28" s="231" t="s">
+      <c r="I28" s="225"/>
+      <c r="J28" s="226" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="K28" s="226"/>
+      <c r="L28" s="226"/>
+      <c r="M28" s="225" t="s">
         <v>41</v>
       </c>
-      <c r="N28" s="231"/>
-      <c r="O28" s="231"/>
-      <c r="P28" s="231"/>
-      <c r="Q28" s="231"/>
-      <c r="R28" s="231"/>
-      <c r="S28" s="231"/>
-      <c r="T28" s="233" t="s">
-        <v>168</v>
-      </c>
-      <c r="U28" s="233"/>
-      <c r="V28" s="233"/>
-      <c r="W28" s="233"/>
-      <c r="X28" s="233"/>
-      <c r="Y28" s="233"/>
-      <c r="Z28" s="233"/>
-      <c r="AA28" s="234" t="s">
+      <c r="N28" s="225"/>
+      <c r="O28" s="225"/>
+      <c r="P28" s="225"/>
+      <c r="Q28" s="225"/>
+      <c r="R28" s="225"/>
+      <c r="S28" s="225"/>
+      <c r="T28" s="227" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="U28" s="227"/>
+      <c r="V28" s="227"/>
+      <c r="W28" s="227"/>
+      <c r="X28" s="227"/>
+      <c r="Y28" s="227"/>
+      <c r="Z28" s="227"/>
+      <c r="AA28" s="228" t="s">
         <v>42</v>
       </c>
-      <c r="AB28" s="234"/>
-      <c r="AC28" s="234"/>
-      <c r="AD28" s="234"/>
+      <c r="AB28" s="228"/>
+      <c r="AC28" s="228"/>
+      <c r="AD28" s="228"/>
       <c r="AE28" s="83">
         <f>IF(AH29&gt;N10,-N10+AH29,0)</f>
         <v>0</v>
@@ -5100,84 +5142,84 @@
     </row>
     <row r="29" spans="1:38" ht="13.7" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="2"/>
-      <c r="B29" s="224" t="s">
+      <c r="B29" s="218" t="s">
         <v>44</v>
       </c>
-      <c r="C29" s="224"/>
-      <c r="D29" s="224"/>
-      <c r="E29" s="224"/>
-      <c r="F29" s="224"/>
-      <c r="G29" s="224"/>
-      <c r="H29" s="224"/>
-      <c r="I29" s="224"/>
-      <c r="J29" s="224"/>
-      <c r="K29" s="224"/>
-      <c r="L29" s="224"/>
-      <c r="M29" s="224"/>
-      <c r="N29" s="224"/>
-      <c r="O29" s="224"/>
-      <c r="P29" s="224"/>
-      <c r="Q29" s="224"/>
-      <c r="R29" s="224"/>
-      <c r="S29" s="224"/>
-      <c r="T29" s="224"/>
-      <c r="U29" s="225" t="s">
+      <c r="C29" s="218"/>
+      <c r="D29" s="218"/>
+      <c r="E29" s="218"/>
+      <c r="F29" s="218"/>
+      <c r="G29" s="218"/>
+      <c r="H29" s="218"/>
+      <c r="I29" s="218"/>
+      <c r="J29" s="218"/>
+      <c r="K29" s="218"/>
+      <c r="L29" s="218"/>
+      <c r="M29" s="218"/>
+      <c r="N29" s="218"/>
+      <c r="O29" s="218"/>
+      <c r="P29" s="218"/>
+      <c r="Q29" s="218"/>
+      <c r="R29" s="218"/>
+      <c r="S29" s="218"/>
+      <c r="T29" s="218"/>
+      <c r="U29" s="219" t="s">
         <v>45</v>
       </c>
-      <c r="V29" s="225"/>
-      <c r="W29" s="225"/>
-      <c r="X29" s="225"/>
-      <c r="Y29" s="225"/>
-      <c r="Z29" s="225"/>
-      <c r="AA29" s="225"/>
-      <c r="AB29" s="225"/>
-      <c r="AC29" s="225"/>
-      <c r="AD29" s="225"/>
+      <c r="V29" s="219"/>
+      <c r="W29" s="219"/>
+      <c r="X29" s="219"/>
+      <c r="Y29" s="219"/>
+      <c r="Z29" s="219"/>
+      <c r="AA29" s="219"/>
+      <c r="AB29" s="219"/>
+      <c r="AC29" s="219"/>
+      <c r="AD29" s="219"/>
       <c r="AE29" s="84">
         <f>+AH29-AE28</f>
-        <v>0</v>
+        <v>53.78</v>
       </c>
       <c r="AF29" s="6"/>
       <c r="AG29" s="6"/>
       <c r="AH29" s="85">
         <f>SUM(AE16:AE27)</f>
-        <v>0</v>
+        <v>53.78</v>
       </c>
       <c r="AJ29" s="78"/>
     </row>
     <row r="30" spans="1:38" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="2"/>
-      <c r="B30" s="224"/>
-      <c r="C30" s="224"/>
-      <c r="D30" s="224"/>
-      <c r="E30" s="224"/>
-      <c r="F30" s="224"/>
-      <c r="G30" s="224"/>
-      <c r="H30" s="224"/>
-      <c r="I30" s="224"/>
-      <c r="J30" s="224"/>
-      <c r="K30" s="224"/>
-      <c r="L30" s="224"/>
-      <c r="M30" s="224"/>
-      <c r="N30" s="224"/>
-      <c r="O30" s="224"/>
-      <c r="P30" s="224"/>
-      <c r="Q30" s="224"/>
-      <c r="R30" s="224"/>
-      <c r="S30" s="224"/>
-      <c r="T30" s="224"/>
-      <c r="U30" s="226" t="s">
+      <c r="B30" s="218"/>
+      <c r="C30" s="218"/>
+      <c r="D30" s="218"/>
+      <c r="E30" s="218"/>
+      <c r="F30" s="218"/>
+      <c r="G30" s="218"/>
+      <c r="H30" s="218"/>
+      <c r="I30" s="218"/>
+      <c r="J30" s="218"/>
+      <c r="K30" s="218"/>
+      <c r="L30" s="218"/>
+      <c r="M30" s="218"/>
+      <c r="N30" s="218"/>
+      <c r="O30" s="218"/>
+      <c r="P30" s="218"/>
+      <c r="Q30" s="218"/>
+      <c r="R30" s="218"/>
+      <c r="S30" s="218"/>
+      <c r="T30" s="218"/>
+      <c r="U30" s="220" t="s">
         <v>46</v>
       </c>
-      <c r="V30" s="226"/>
-      <c r="W30" s="226"/>
-      <c r="X30" s="226"/>
-      <c r="Y30" s="226"/>
-      <c r="Z30" s="226"/>
-      <c r="AA30" s="226"/>
-      <c r="AB30" s="226"/>
-      <c r="AC30" s="226"/>
-      <c r="AD30" s="226"/>
+      <c r="V30" s="220"/>
+      <c r="W30" s="220"/>
+      <c r="X30" s="220"/>
+      <c r="Y30" s="220"/>
+      <c r="Z30" s="220"/>
+      <c r="AA30" s="220"/>
+      <c r="AB30" s="220"/>
+      <c r="AC30" s="220"/>
+      <c r="AD30" s="220"/>
       <c r="AE30" s="86"/>
       <c r="AF30" s="6"/>
       <c r="AG30" s="6"/>
@@ -5186,40 +5228,40 @@
     </row>
     <row r="31" spans="1:38" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="2"/>
-      <c r="B31" s="224"/>
-      <c r="C31" s="224"/>
-      <c r="D31" s="224"/>
-      <c r="E31" s="224"/>
-      <c r="F31" s="224"/>
-      <c r="G31" s="224"/>
-      <c r="H31" s="224"/>
-      <c r="I31" s="224"/>
-      <c r="J31" s="224"/>
-      <c r="K31" s="224"/>
-      <c r="L31" s="224"/>
-      <c r="M31" s="224"/>
-      <c r="N31" s="224"/>
-      <c r="O31" s="224"/>
-      <c r="P31" s="224"/>
-      <c r="Q31" s="224"/>
-      <c r="R31" s="224"/>
-      <c r="S31" s="224"/>
-      <c r="T31" s="224"/>
-      <c r="U31" s="227" t="s">
+      <c r="B31" s="218"/>
+      <c r="C31" s="218"/>
+      <c r="D31" s="218"/>
+      <c r="E31" s="218"/>
+      <c r="F31" s="218"/>
+      <c r="G31" s="218"/>
+      <c r="H31" s="218"/>
+      <c r="I31" s="218"/>
+      <c r="J31" s="218"/>
+      <c r="K31" s="218"/>
+      <c r="L31" s="218"/>
+      <c r="M31" s="218"/>
+      <c r="N31" s="218"/>
+      <c r="O31" s="218"/>
+      <c r="P31" s="218"/>
+      <c r="Q31" s="218"/>
+      <c r="R31" s="218"/>
+      <c r="S31" s="218"/>
+      <c r="T31" s="218"/>
+      <c r="U31" s="221" t="s">
         <v>47</v>
       </c>
-      <c r="V31" s="227"/>
-      <c r="W31" s="227"/>
-      <c r="X31" s="227"/>
-      <c r="Y31" s="227"/>
-      <c r="Z31" s="227"/>
-      <c r="AA31" s="227"/>
-      <c r="AB31" s="227"/>
-      <c r="AC31" s="227"/>
-      <c r="AD31" s="227"/>
+      <c r="V31" s="221"/>
+      <c r="W31" s="221"/>
+      <c r="X31" s="221"/>
+      <c r="Y31" s="221"/>
+      <c r="Z31" s="221"/>
+      <c r="AA31" s="221"/>
+      <c r="AB31" s="221"/>
+      <c r="AC31" s="221"/>
+      <c r="AD31" s="221"/>
       <c r="AE31" s="87">
         <f>+AE29-AE30</f>
-        <v>0</v>
+        <v>53.78</v>
       </c>
       <c r="AF31" s="6"/>
       <c r="AG31" s="6"/>
@@ -5265,154 +5307,156 @@
     </row>
     <row r="33" spans="1:32" ht="9.9499999999999993" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2"/>
-      <c r="B33" s="228" t="s">
+      <c r="B33" s="222" t="s">
         <v>48</v>
       </c>
-      <c r="C33" s="228"/>
-      <c r="D33" s="228"/>
-      <c r="E33" s="228"/>
-      <c r="F33" s="228"/>
-      <c r="G33" s="228"/>
-      <c r="H33" s="228"/>
-      <c r="I33" s="228"/>
-      <c r="J33" s="228"/>
-      <c r="K33" s="228"/>
-      <c r="L33" s="228"/>
-      <c r="M33" s="228"/>
-      <c r="N33" s="228"/>
-      <c r="O33" s="228"/>
-      <c r="P33" s="228"/>
-      <c r="Q33" s="228"/>
+      <c r="C33" s="222"/>
+      <c r="D33" s="222"/>
+      <c r="E33" s="222"/>
+      <c r="F33" s="222"/>
+      <c r="G33" s="222"/>
+      <c r="H33" s="222"/>
+      <c r="I33" s="222"/>
+      <c r="J33" s="222"/>
+      <c r="K33" s="222"/>
+      <c r="L33" s="222"/>
+      <c r="M33" s="222"/>
+      <c r="N33" s="222"/>
+      <c r="O33" s="222"/>
+      <c r="P33" s="222"/>
+      <c r="Q33" s="222"/>
       <c r="R33" s="91"/>
-      <c r="S33" s="229" t="s">
+      <c r="S33" s="223" t="s">
         <v>49</v>
       </c>
-      <c r="T33" s="229"/>
-      <c r="U33" s="229"/>
-      <c r="V33" s="229"/>
-      <c r="W33" s="229"/>
-      <c r="X33" s="229"/>
-      <c r="Y33" s="229"/>
-      <c r="Z33" s="229"/>
-      <c r="AA33" s="229"/>
-      <c r="AB33" s="229"/>
-      <c r="AC33" s="229"/>
-      <c r="AD33" s="229"/>
-      <c r="AE33" s="229"/>
+      <c r="T33" s="223"/>
+      <c r="U33" s="223"/>
+      <c r="V33" s="223"/>
+      <c r="W33" s="223"/>
+      <c r="X33" s="223"/>
+      <c r="Y33" s="223"/>
+      <c r="Z33" s="223"/>
+      <c r="AA33" s="223"/>
+      <c r="AB33" s="223"/>
+      <c r="AC33" s="223"/>
+      <c r="AD33" s="223"/>
+      <c r="AE33" s="223"/>
       <c r="AF33" s="6"/>
     </row>
     <row r="34" spans="1:32" ht="12.6" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A34" s="2"/>
-      <c r="B34" s="215" t="s">
-        <v>174</v>
-      </c>
-      <c r="C34" s="216"/>
-      <c r="D34" s="216"/>
-      <c r="E34" s="216"/>
-      <c r="F34" s="216"/>
-      <c r="G34" s="216"/>
-      <c r="H34" s="216"/>
-      <c r="I34" s="216"/>
-      <c r="J34" s="216"/>
-      <c r="K34" s="216"/>
-      <c r="L34" s="216"/>
-      <c r="M34" s="216"/>
-      <c r="N34" s="216"/>
-      <c r="O34" s="216"/>
-      <c r="P34" s="216"/>
-      <c r="Q34" s="217"/>
+      <c r="B34" s="209" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="C34" s="210"/>
+      <c r="D34" s="210"/>
+      <c r="E34" s="210"/>
+      <c r="F34" s="210"/>
+      <c r="G34" s="210"/>
+      <c r="H34" s="210"/>
+      <c r="I34" s="210"/>
+      <c r="J34" s="210"/>
+      <c r="K34" s="210"/>
+      <c r="L34" s="210"/>
+      <c r="M34" s="210"/>
+      <c r="N34" s="210"/>
+      <c r="O34" s="210"/>
+      <c r="P34" s="210"/>
+      <c r="Q34" s="211"/>
       <c r="R34" s="92"/>
-      <c r="S34" s="229"/>
-      <c r="T34" s="229"/>
-      <c r="U34" s="229"/>
-      <c r="V34" s="229"/>
-      <c r="W34" s="229"/>
-      <c r="X34" s="229"/>
-      <c r="Y34" s="229"/>
-      <c r="Z34" s="229"/>
-      <c r="AA34" s="229"/>
-      <c r="AB34" s="229"/>
-      <c r="AC34" s="229"/>
-      <c r="AD34" s="229"/>
-      <c r="AE34" s="229"/>
+      <c r="S34" s="223"/>
+      <c r="T34" s="223"/>
+      <c r="U34" s="223"/>
+      <c r="V34" s="223"/>
+      <c r="W34" s="223"/>
+      <c r="X34" s="223"/>
+      <c r="Y34" s="223"/>
+      <c r="Z34" s="223"/>
+      <c r="AA34" s="223"/>
+      <c r="AB34" s="223"/>
+      <c r="AC34" s="223"/>
+      <c r="AD34" s="223"/>
+      <c r="AE34" s="223"/>
       <c r="AF34" s="6"/>
     </row>
     <row r="35" spans="1:32" ht="12.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="2"/>
-      <c r="B35" s="218"/>
-      <c r="C35" s="219"/>
-      <c r="D35" s="219"/>
-      <c r="E35" s="219"/>
-      <c r="F35" s="219"/>
-      <c r="G35" s="219"/>
-      <c r="H35" s="219"/>
-      <c r="I35" s="219"/>
-      <c r="J35" s="219"/>
-      <c r="K35" s="219"/>
-      <c r="L35" s="219"/>
-      <c r="M35" s="219"/>
-      <c r="N35" s="219"/>
-      <c r="O35" s="219"/>
-      <c r="P35" s="219"/>
-      <c r="Q35" s="220"/>
+      <c r="B35" s="212"/>
+      <c r="C35" s="213"/>
+      <c r="D35" s="213"/>
+      <c r="E35" s="213"/>
+      <c r="F35" s="213"/>
+      <c r="G35" s="213"/>
+      <c r="H35" s="213"/>
+      <c r="I35" s="213"/>
+      <c r="J35" s="213"/>
+      <c r="K35" s="213"/>
+      <c r="L35" s="213"/>
+      <c r="M35" s="213"/>
+      <c r="N35" s="213"/>
+      <c r="O35" s="213"/>
+      <c r="P35" s="213"/>
+      <c r="Q35" s="214"/>
       <c r="R35" s="93"/>
-      <c r="S35" s="213" t="s">
+      <c r="S35" s="232" t="s">
         <v>21</v>
       </c>
-      <c r="T35" s="211" t="s">
+      <c r="T35" s="230" t="s">
         <v>51</v>
       </c>
-      <c r="U35" s="211"/>
-      <c r="V35" s="211"/>
-      <c r="W35" s="211"/>
-      <c r="X35" s="214" t="s">
+      <c r="U35" s="230"/>
+      <c r="V35" s="230"/>
+      <c r="W35" s="230"/>
+      <c r="X35" s="207" t="s">
         <v>29</v>
       </c>
-      <c r="Y35" s="214"/>
-      <c r="Z35" s="214" t="s">
+      <c r="Y35" s="207"/>
+      <c r="Z35" s="207" t="s">
         <v>30</v>
       </c>
-      <c r="AA35" s="214"/>
-      <c r="AB35" s="214"/>
-      <c r="AC35" s="214" t="s">
+      <c r="AA35" s="207"/>
+      <c r="AB35" s="207"/>
+      <c r="AC35" s="207" t="s">
         <v>31</v>
       </c>
-      <c r="AD35" s="214"/>
-      <c r="AE35" s="210" t="s">
+      <c r="AD35" s="207"/>
+      <c r="AE35" s="229" t="s">
         <v>32</v>
       </c>
       <c r="AF35" s="6"/>
     </row>
     <row r="36" spans="1:32" ht="12.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="2"/>
-      <c r="B36" s="218"/>
-      <c r="C36" s="219"/>
-      <c r="D36" s="219"/>
-      <c r="E36" s="219"/>
-      <c r="F36" s="219"/>
-      <c r="G36" s="219"/>
-      <c r="H36" s="219"/>
-      <c r="I36" s="219"/>
-      <c r="J36" s="219"/>
-      <c r="K36" s="219"/>
-      <c r="L36" s="219"/>
-      <c r="M36" s="219"/>
-      <c r="N36" s="219"/>
-      <c r="O36" s="219"/>
-      <c r="P36" s="219"/>
-      <c r="Q36" s="220"/>
+      <c r="B36" s="212"/>
+      <c r="C36" s="213"/>
+      <c r="D36" s="213"/>
+      <c r="E36" s="213"/>
+      <c r="F36" s="213"/>
+      <c r="G36" s="213"/>
+      <c r="H36" s="213"/>
+      <c r="I36" s="213"/>
+      <c r="J36" s="213"/>
+      <c r="K36" s="213"/>
+      <c r="L36" s="213"/>
+      <c r="M36" s="213"/>
+      <c r="N36" s="213"/>
+      <c r="O36" s="213"/>
+      <c r="P36" s="213"/>
+      <c r="Q36" s="214"/>
       <c r="R36" s="93"/>
-      <c r="S36" s="213"/>
-      <c r="T36" s="211"/>
-      <c r="U36" s="211"/>
-      <c r="V36" s="211"/>
-      <c r="W36" s="211"/>
-      <c r="X36" s="214"/>
-      <c r="Y36" s="214"/>
-      <c r="Z36" s="211" t="s">
+      <c r="S36" s="232"/>
+      <c r="T36" s="230"/>
+      <c r="U36" s="230"/>
+      <c r="V36" s="230"/>
+      <c r="W36" s="230"/>
+      <c r="X36" s="207"/>
+      <c r="Y36" s="207"/>
+      <c r="Z36" s="230" t="s">
         <v>52</v>
       </c>
-      <c r="AA36" s="211"/>
+      <c r="AA36" s="230"/>
       <c r="AB36" s="94" t="s">
         <v>53</v>
       </c>
@@ -5422,95 +5466,95 @@
       <c r="AD36" s="94" t="s">
         <v>55</v>
       </c>
-      <c r="AE36" s="210"/>
+      <c r="AE36" s="229"/>
     </row>
     <row r="37" spans="1:32" ht="12.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="2"/>
-      <c r="B37" s="218"/>
-      <c r="C37" s="219"/>
-      <c r="D37" s="219"/>
-      <c r="E37" s="219"/>
-      <c r="F37" s="219"/>
-      <c r="G37" s="219"/>
-      <c r="H37" s="219"/>
-      <c r="I37" s="219"/>
-      <c r="J37" s="219"/>
-      <c r="K37" s="219"/>
-      <c r="L37" s="219"/>
-      <c r="M37" s="219"/>
-      <c r="N37" s="219"/>
-      <c r="O37" s="219"/>
-      <c r="P37" s="219"/>
-      <c r="Q37" s="220"/>
+      <c r="B37" s="212"/>
+      <c r="C37" s="213"/>
+      <c r="D37" s="213"/>
+      <c r="E37" s="213"/>
+      <c r="F37" s="213"/>
+      <c r="G37" s="213"/>
+      <c r="H37" s="213"/>
+      <c r="I37" s="213"/>
+      <c r="J37" s="213"/>
+      <c r="K37" s="213"/>
+      <c r="L37" s="213"/>
+      <c r="M37" s="213"/>
+      <c r="N37" s="213"/>
+      <c r="O37" s="213"/>
+      <c r="P37" s="213"/>
+      <c r="Q37" s="214"/>
       <c r="R37" s="93"/>
-      <c r="S37" s="212">
+      <c r="S37" s="231">
         <v>1</v>
       </c>
-      <c r="T37" s="208" t="s">
+      <c r="T37" s="206" t="s">
         <v>56</v>
       </c>
-      <c r="U37" s="208"/>
-      <c r="V37" s="208"/>
-      <c r="W37" s="208"/>
-      <c r="X37" s="198">
+      <c r="U37" s="206"/>
+      <c r="V37" s="206"/>
+      <c r="W37" s="206"/>
+      <c r="X37" s="196">
         <f>+AM107</f>
         <v>537.88</v>
       </c>
-      <c r="Y37" s="198"/>
-      <c r="Z37" s="198">
+      <c r="Y37" s="196"/>
+      <c r="Z37" s="196">
         <f>+AR107</f>
         <v>107.57</v>
       </c>
-      <c r="AA37" s="198"/>
-      <c r="AB37" s="198">
+      <c r="AA37" s="196"/>
+      <c r="AB37" s="196">
         <f>+AT107</f>
         <v>215.15</v>
       </c>
-      <c r="AC37" s="198">
+      <c r="AC37" s="196">
         <f>+AV107</f>
         <v>107.57</v>
       </c>
-      <c r="AD37" s="198">
+      <c r="AD37" s="196">
         <f>+AX107</f>
         <v>215.15</v>
       </c>
-      <c r="AE37" s="199">
+      <c r="AE37" s="197">
         <f>+AZ107</f>
         <v>268.94</v>
       </c>
     </row>
     <row r="38" spans="1:32" ht="12.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2"/>
-      <c r="B38" s="221"/>
-      <c r="C38" s="222"/>
-      <c r="D38" s="222"/>
-      <c r="E38" s="222"/>
-      <c r="F38" s="222"/>
-      <c r="G38" s="222"/>
-      <c r="H38" s="222"/>
-      <c r="I38" s="222"/>
-      <c r="J38" s="222"/>
-      <c r="K38" s="222"/>
-      <c r="L38" s="222"/>
-      <c r="M38" s="222"/>
-      <c r="N38" s="222"/>
-      <c r="O38" s="222"/>
-      <c r="P38" s="222"/>
-      <c r="Q38" s="223"/>
+      <c r="B38" s="215"/>
+      <c r="C38" s="216"/>
+      <c r="D38" s="216"/>
+      <c r="E38" s="216"/>
+      <c r="F38" s="216"/>
+      <c r="G38" s="216"/>
+      <c r="H38" s="216"/>
+      <c r="I38" s="216"/>
+      <c r="J38" s="216"/>
+      <c r="K38" s="216"/>
+      <c r="L38" s="216"/>
+      <c r="M38" s="216"/>
+      <c r="N38" s="216"/>
+      <c r="O38" s="216"/>
+      <c r="P38" s="216"/>
+      <c r="Q38" s="217"/>
       <c r="R38" s="93"/>
-      <c r="S38" s="212"/>
-      <c r="T38" s="208"/>
-      <c r="U38" s="208"/>
-      <c r="V38" s="208"/>
-      <c r="W38" s="208"/>
-      <c r="X38" s="198"/>
-      <c r="Y38" s="198"/>
-      <c r="Z38" s="198"/>
-      <c r="AA38" s="198"/>
-      <c r="AB38" s="198"/>
-      <c r="AC38" s="198"/>
-      <c r="AD38" s="198"/>
-      <c r="AE38" s="199"/>
+      <c r="S38" s="231"/>
+      <c r="T38" s="206"/>
+      <c r="U38" s="206"/>
+      <c r="V38" s="206"/>
+      <c r="W38" s="206"/>
+      <c r="X38" s="196"/>
+      <c r="Y38" s="196"/>
+      <c r="Z38" s="196"/>
+      <c r="AA38" s="196"/>
+      <c r="AB38" s="196"/>
+      <c r="AC38" s="196"/>
+      <c r="AD38" s="196"/>
+      <c r="AE38" s="197"/>
     </row>
     <row r="39" spans="1:32" ht="7.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2"/>
@@ -5531,19 +5575,19 @@
       <c r="P39" s="95"/>
       <c r="Q39" s="95"/>
       <c r="R39" s="96"/>
-      <c r="S39" s="212"/>
-      <c r="T39" s="208"/>
-      <c r="U39" s="208"/>
-      <c r="V39" s="208"/>
-      <c r="W39" s="208"/>
-      <c r="X39" s="198"/>
-      <c r="Y39" s="198"/>
-      <c r="Z39" s="198"/>
-      <c r="AA39" s="198"/>
-      <c r="AB39" s="198"/>
-      <c r="AC39" s="198"/>
-      <c r="AD39" s="198"/>
-      <c r="AE39" s="199"/>
+      <c r="S39" s="231"/>
+      <c r="T39" s="206"/>
+      <c r="U39" s="206"/>
+      <c r="V39" s="206"/>
+      <c r="W39" s="206"/>
+      <c r="X39" s="196"/>
+      <c r="Y39" s="196"/>
+      <c r="Z39" s="196"/>
+      <c r="AA39" s="196"/>
+      <c r="AB39" s="196"/>
+      <c r="AC39" s="196"/>
+      <c r="AD39" s="196"/>
+      <c r="AE39" s="197"/>
     </row>
     <row r="40" spans="1:32" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="2"/>
@@ -5570,38 +5614,38 @@
       <c r="P40" s="103"/>
       <c r="Q40" s="104"/>
       <c r="R40" s="7"/>
-      <c r="S40" s="204">
+      <c r="S40" s="202">
         <v>2</v>
       </c>
-      <c r="T40" s="209" t="s">
+      <c r="T40" s="208" t="s">
         <v>60</v>
       </c>
-      <c r="U40" s="209"/>
-      <c r="V40" s="209"/>
-      <c r="W40" s="209"/>
-      <c r="X40" s="198">
+      <c r="U40" s="208"/>
+      <c r="V40" s="208"/>
+      <c r="W40" s="208"/>
+      <c r="X40" s="196">
         <f>+AM108</f>
         <v>484.09</v>
       </c>
-      <c r="Y40" s="198"/>
-      <c r="Z40" s="198">
+      <c r="Y40" s="196"/>
+      <c r="Z40" s="196">
         <f>+AR108</f>
         <v>96.81</v>
       </c>
-      <c r="AA40" s="198"/>
-      <c r="AB40" s="198">
+      <c r="AA40" s="196"/>
+      <c r="AB40" s="196">
         <f>+AT108</f>
         <v>193.63</v>
       </c>
-      <c r="AC40" s="198">
+      <c r="AC40" s="196">
         <f>+AV108</f>
         <v>96.81</v>
       </c>
-      <c r="AD40" s="198">
+      <c r="AD40" s="196">
         <f>+AX108</f>
         <v>193.63</v>
       </c>
-      <c r="AE40" s="199">
+      <c r="AE40" s="197">
         <f>+AZ108</f>
         <v>242.04</v>
       </c>
@@ -5625,28 +5669,28 @@
       <c r="J41" s="111"/>
       <c r="K41" s="112"/>
       <c r="L41" s="113"/>
-      <c r="M41" s="206">
+      <c r="M41" s="204">
         <f>AE29</f>
-        <v>0</v>
-      </c>
-      <c r="N41" s="206"/>
-      <c r="O41" s="206"/>
-      <c r="P41" s="206"/>
-      <c r="Q41" s="206"/>
+        <v>53.78</v>
+      </c>
+      <c r="N41" s="204"/>
+      <c r="O41" s="204"/>
+      <c r="P41" s="204"/>
+      <c r="Q41" s="204"/>
       <c r="R41" s="7"/>
-      <c r="S41" s="204"/>
-      <c r="T41" s="209"/>
-      <c r="U41" s="209"/>
-      <c r="V41" s="209"/>
-      <c r="W41" s="209"/>
-      <c r="X41" s="198"/>
-      <c r="Y41" s="198"/>
-      <c r="Z41" s="198"/>
-      <c r="AA41" s="198"/>
-      <c r="AB41" s="198"/>
-      <c r="AC41" s="198"/>
-      <c r="AD41" s="198"/>
-      <c r="AE41" s="199"/>
+      <c r="S41" s="202"/>
+      <c r="T41" s="208"/>
+      <c r="U41" s="208"/>
+      <c r="V41" s="208"/>
+      <c r="W41" s="208"/>
+      <c r="X41" s="196"/>
+      <c r="Y41" s="196"/>
+      <c r="Z41" s="196"/>
+      <c r="AA41" s="196"/>
+      <c r="AB41" s="196"/>
+      <c r="AC41" s="196"/>
+      <c r="AD41" s="196"/>
+      <c r="AE41" s="197"/>
     </row>
     <row r="42" spans="1:32" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="2"/>
@@ -5659,32 +5703,32 @@
       <c r="F42" s="108"/>
       <c r="G42" s="109"/>
       <c r="H42" s="109"/>
-      <c r="I42" s="207" t="str">
-        <f>AO77</f>
-        <v>***  ***</v>
-      </c>
-      <c r="J42" s="207"/>
-      <c r="K42" s="207"/>
-      <c r="L42" s="207"/>
-      <c r="M42" s="207"/>
-      <c r="N42" s="207"/>
-      <c r="O42" s="207"/>
-      <c r="P42" s="207"/>
-      <c r="Q42" s="207"/>
+      <c r="I42" s="205" t="str">
+        <f ca="1">AO77</f>
+        <v>*** CINQÜENTA E TRÊS REAIS  E SETENTA E OITO CENTAVOS ***</v>
+      </c>
+      <c r="J42" s="205"/>
+      <c r="K42" s="205"/>
+      <c r="L42" s="205"/>
+      <c r="M42" s="205"/>
+      <c r="N42" s="205"/>
+      <c r="O42" s="205"/>
+      <c r="P42" s="205"/>
+      <c r="Q42" s="205"/>
       <c r="R42" s="7"/>
-      <c r="S42" s="204"/>
-      <c r="T42" s="209"/>
-      <c r="U42" s="209"/>
-      <c r="V42" s="209"/>
-      <c r="W42" s="209"/>
-      <c r="X42" s="198"/>
-      <c r="Y42" s="198"/>
-      <c r="Z42" s="198"/>
-      <c r="AA42" s="198"/>
-      <c r="AB42" s="198"/>
-      <c r="AC42" s="198"/>
-      <c r="AD42" s="198"/>
-      <c r="AE42" s="199"/>
+      <c r="S42" s="202"/>
+      <c r="T42" s="208"/>
+      <c r="U42" s="208"/>
+      <c r="V42" s="208"/>
+      <c r="W42" s="208"/>
+      <c r="X42" s="196"/>
+      <c r="Y42" s="196"/>
+      <c r="Z42" s="196"/>
+      <c r="AA42" s="196"/>
+      <c r="AB42" s="196"/>
+      <c r="AC42" s="196"/>
+      <c r="AD42" s="196"/>
+      <c r="AE42" s="197"/>
     </row>
     <row r="43" spans="1:32" s="20" customFormat="1" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="2"/>
@@ -5697,48 +5741,48 @@
       <c r="F43" s="108"/>
       <c r="G43" s="109"/>
       <c r="H43" s="109"/>
-      <c r="I43" s="207"/>
-      <c r="J43" s="207"/>
-      <c r="K43" s="207"/>
-      <c r="L43" s="207"/>
-      <c r="M43" s="207"/>
-      <c r="N43" s="207"/>
-      <c r="O43" s="207"/>
-      <c r="P43" s="207"/>
-      <c r="Q43" s="207"/>
+      <c r="I43" s="205"/>
+      <c r="J43" s="205"/>
+      <c r="K43" s="205"/>
+      <c r="L43" s="205"/>
+      <c r="M43" s="205"/>
+      <c r="N43" s="205"/>
+      <c r="O43" s="205"/>
+      <c r="P43" s="205"/>
+      <c r="Q43" s="205"/>
       <c r="R43" s="114"/>
-      <c r="S43" s="204">
+      <c r="S43" s="202">
         <v>3</v>
       </c>
-      <c r="T43" s="208" t="s">
+      <c r="T43" s="206" t="s">
         <v>66</v>
       </c>
-      <c r="U43" s="208"/>
-      <c r="V43" s="208"/>
-      <c r="W43" s="208"/>
-      <c r="X43" s="198">
+      <c r="U43" s="206"/>
+      <c r="V43" s="206"/>
+      <c r="W43" s="206"/>
+      <c r="X43" s="196">
         <f>+AM109</f>
         <v>457.19</v>
       </c>
-      <c r="Y43" s="198"/>
-      <c r="Z43" s="198">
+      <c r="Y43" s="196"/>
+      <c r="Z43" s="196">
         <f>+AR109</f>
         <v>91.43</v>
       </c>
-      <c r="AA43" s="198"/>
-      <c r="AB43" s="198">
+      <c r="AA43" s="196"/>
+      <c r="AB43" s="196">
         <f>+AT109</f>
         <v>182.87</v>
       </c>
-      <c r="AC43" s="198">
+      <c r="AC43" s="196">
         <f>+AV109</f>
         <v>91.43</v>
       </c>
-      <c r="AD43" s="198">
+      <c r="AD43" s="196">
         <f>+AX109</f>
         <v>182.87</v>
       </c>
-      <c r="AE43" s="199">
+      <c r="AE43" s="197">
         <f>+AZ109</f>
         <v>228.59</v>
       </c>
@@ -5752,40 +5796,42 @@
       <c r="F44" s="118"/>
       <c r="G44" s="116"/>
       <c r="H44" s="116"/>
-      <c r="I44" s="207"/>
-      <c r="J44" s="207"/>
-      <c r="K44" s="207"/>
-      <c r="L44" s="207"/>
-      <c r="M44" s="207"/>
-      <c r="N44" s="207"/>
-      <c r="O44" s="207"/>
-      <c r="P44" s="207"/>
-      <c r="Q44" s="207"/>
+      <c r="I44" s="205"/>
+      <c r="J44" s="205"/>
+      <c r="K44" s="205"/>
+      <c r="L44" s="205"/>
+      <c r="M44" s="205"/>
+      <c r="N44" s="205"/>
+      <c r="O44" s="205"/>
+      <c r="P44" s="205"/>
+      <c r="Q44" s="205"/>
       <c r="R44" s="7"/>
-      <c r="S44" s="204"/>
-      <c r="T44" s="208"/>
-      <c r="U44" s="208"/>
-      <c r="V44" s="208"/>
-      <c r="W44" s="208"/>
-      <c r="X44" s="198"/>
-      <c r="Y44" s="198"/>
-      <c r="Z44" s="198"/>
-      <c r="AA44" s="198"/>
-      <c r="AB44" s="198"/>
-      <c r="AC44" s="198"/>
-      <c r="AD44" s="198"/>
-      <c r="AE44" s="199"/>
+      <c r="S44" s="202"/>
+      <c r="T44" s="206"/>
+      <c r="U44" s="206"/>
+      <c r="V44" s="206"/>
+      <c r="W44" s="206"/>
+      <c r="X44" s="196"/>
+      <c r="Y44" s="196"/>
+      <c r="Z44" s="196"/>
+      <c r="AA44" s="196"/>
+      <c r="AB44" s="196"/>
+      <c r="AC44" s="196"/>
+      <c r="AD44" s="196"/>
+      <c r="AE44" s="197"/>
     </row>
     <row r="45" spans="1:32" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="2"/>
       <c r="B45" s="115" t="s">
         <v>67</v>
       </c>
-      <c r="C45" s="201">
-        <v>46249</v>
-      </c>
-      <c r="D45" s="201"/>
-      <c r="E45" s="201"/>
+      <c r="C45" s="199" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="D45" s="199"/>
+      <c r="E45" s="199"/>
       <c r="F45" s="118" t="s">
         <v>68</v>
       </c>
@@ -5801,19 +5847,19 @@
       <c r="P45" s="120"/>
       <c r="Q45" s="121"/>
       <c r="R45" s="7"/>
-      <c r="S45" s="204"/>
-      <c r="T45" s="208"/>
-      <c r="U45" s="208"/>
-      <c r="V45" s="208"/>
-      <c r="W45" s="208"/>
-      <c r="X45" s="198"/>
-      <c r="Y45" s="198"/>
-      <c r="Z45" s="198"/>
-      <c r="AA45" s="198"/>
-      <c r="AB45" s="198"/>
-      <c r="AC45" s="198"/>
-      <c r="AD45" s="198"/>
-      <c r="AE45" s="199"/>
+      <c r="S45" s="202"/>
+      <c r="T45" s="206"/>
+      <c r="U45" s="206"/>
+      <c r="V45" s="206"/>
+      <c r="W45" s="206"/>
+      <c r="X45" s="196"/>
+      <c r="Y45" s="196"/>
+      <c r="Z45" s="196"/>
+      <c r="AA45" s="196"/>
+      <c r="AB45" s="196"/>
+      <c r="AC45" s="196"/>
+      <c r="AD45" s="196"/>
+      <c r="AE45" s="197"/>
     </row>
     <row r="46" spans="1:32" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="2"/>
@@ -5821,19 +5867,19 @@
       <c r="C46" s="109"/>
       <c r="D46" s="109"/>
       <c r="E46" s="123"/>
-      <c r="F46" s="202">
+      <c r="F46" s="200">
         <f>C45</f>
         <v>46249</v>
       </c>
-      <c r="G46" s="202"/>
-      <c r="H46" s="202"/>
-      <c r="I46" s="203">
+      <c r="G46" s="200"/>
+      <c r="H46" s="200"/>
+      <c r="I46" s="201">
         <f>+AC8</f>
         <v>46244</v>
       </c>
-      <c r="J46" s="203"/>
-      <c r="K46" s="203"/>
-      <c r="L46" s="203"/>
+      <c r="J46" s="201"/>
+      <c r="K46" s="201"/>
+      <c r="L46" s="201"/>
       <c r="M46" s="119" t="s">
         <v>70</v>
       </c>
@@ -5841,38 +5887,38 @@
       <c r="P46" s="124"/>
       <c r="Q46" s="125"/>
       <c r="R46" s="7"/>
-      <c r="S46" s="204">
+      <c r="S46" s="202">
         <v>4</v>
       </c>
-      <c r="T46" s="205" t="s">
+      <c r="T46" s="203" t="s">
         <v>71</v>
       </c>
-      <c r="U46" s="205"/>
-      <c r="V46" s="205"/>
-      <c r="W46" s="205"/>
-      <c r="X46" s="198">
+      <c r="U46" s="203"/>
+      <c r="V46" s="203"/>
+      <c r="W46" s="203"/>
+      <c r="X46" s="196">
         <f>+AM110</f>
         <v>403.41</v>
       </c>
-      <c r="Y46" s="198"/>
-      <c r="Z46" s="198">
+      <c r="Y46" s="196"/>
+      <c r="Z46" s="196">
         <f>+AR110</f>
         <v>80.680000000000007</v>
       </c>
-      <c r="AA46" s="198"/>
-      <c r="AB46" s="198">
+      <c r="AA46" s="196"/>
+      <c r="AB46" s="196">
         <f>+AT110</f>
         <v>161.36000000000001</v>
       </c>
-      <c r="AC46" s="198">
+      <c r="AC46" s="196">
         <f>+AV110</f>
         <v>80.680000000000007</v>
       </c>
-      <c r="AD46" s="198">
+      <c r="AD46" s="196">
         <f>+AX110</f>
         <v>161.36000000000001</v>
       </c>
-      <c r="AE46" s="199">
+      <c r="AE46" s="197">
         <f>+AZ110</f>
         <v>201.7</v>
       </c>
@@ -5896,19 +5942,19 @@
       <c r="P47" s="120"/>
       <c r="Q47" s="127"/>
       <c r="R47" s="114"/>
-      <c r="S47" s="204"/>
-      <c r="T47" s="205"/>
-      <c r="U47" s="205"/>
-      <c r="V47" s="205"/>
-      <c r="W47" s="205"/>
-      <c r="X47" s="198"/>
-      <c r="Y47" s="198"/>
-      <c r="Z47" s="198"/>
-      <c r="AA47" s="198"/>
-      <c r="AB47" s="198"/>
-      <c r="AC47" s="198"/>
-      <c r="AD47" s="198"/>
-      <c r="AE47" s="199"/>
+      <c r="S47" s="202"/>
+      <c r="T47" s="203"/>
+      <c r="U47" s="203"/>
+      <c r="V47" s="203"/>
+      <c r="W47" s="203"/>
+      <c r="X47" s="196"/>
+      <c r="Y47" s="196"/>
+      <c r="Z47" s="196"/>
+      <c r="AA47" s="196"/>
+      <c r="AB47" s="196"/>
+      <c r="AC47" s="196"/>
+      <c r="AD47" s="196"/>
+      <c r="AE47" s="197"/>
     </row>
     <row r="48" spans="1:32" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="2"/>
@@ -5923,30 +5969,30 @@
         <v>72</v>
       </c>
       <c r="J48" s="111"/>
-      <c r="K48" s="200">
+      <c r="K48" s="198">
         <f>C45</f>
         <v>46249</v>
       </c>
-      <c r="L48" s="200"/>
-      <c r="M48" s="200"/>
+      <c r="L48" s="198"/>
+      <c r="M48" s="198"/>
       <c r="N48" s="128"/>
       <c r="O48" s="120"/>
       <c r="P48" s="120"/>
       <c r="Q48" s="127"/>
       <c r="R48" s="7"/>
-      <c r="S48" s="204"/>
-      <c r="T48" s="205"/>
-      <c r="U48" s="205"/>
-      <c r="V48" s="205"/>
-      <c r="W48" s="205"/>
-      <c r="X48" s="198"/>
-      <c r="Y48" s="198"/>
-      <c r="Z48" s="198"/>
-      <c r="AA48" s="198"/>
-      <c r="AB48" s="198"/>
-      <c r="AC48" s="198"/>
-      <c r="AD48" s="198"/>
-      <c r="AE48" s="199"/>
+      <c r="S48" s="202"/>
+      <c r="T48" s="203"/>
+      <c r="U48" s="203"/>
+      <c r="V48" s="203"/>
+      <c r="W48" s="203"/>
+      <c r="X48" s="196"/>
+      <c r="Y48" s="196"/>
+      <c r="Z48" s="196"/>
+      <c r="AA48" s="196"/>
+      <c r="AB48" s="196"/>
+      <c r="AC48" s="196"/>
+      <c r="AD48" s="196"/>
+      <c r="AE48" s="197"/>
     </row>
     <row r="49" spans="1:62" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="2"/>
@@ -5967,38 +6013,38 @@
       <c r="P49" s="120"/>
       <c r="Q49" s="127"/>
       <c r="R49" s="7"/>
-      <c r="S49" s="196">
+      <c r="S49" s="194">
         <v>5</v>
       </c>
-      <c r="T49" s="197" t="s">
+      <c r="T49" s="195" t="s">
         <v>164</v>
       </c>
-      <c r="U49" s="197"/>
-      <c r="V49" s="197"/>
-      <c r="W49" s="197"/>
-      <c r="X49" s="188">
+      <c r="U49" s="195"/>
+      <c r="V49" s="195"/>
+      <c r="W49" s="195"/>
+      <c r="X49" s="186">
         <f>+AM111</f>
         <v>268.94</v>
       </c>
-      <c r="Y49" s="188"/>
-      <c r="Z49" s="188">
+      <c r="Y49" s="186"/>
+      <c r="Z49" s="186">
         <f>+AR111</f>
         <v>53.78</v>
       </c>
-      <c r="AA49" s="188"/>
-      <c r="AB49" s="188">
+      <c r="AA49" s="186"/>
+      <c r="AB49" s="186">
         <f>+AT111</f>
         <v>107.57</v>
       </c>
-      <c r="AC49" s="188">
+      <c r="AC49" s="186">
         <f>+AV111</f>
         <v>53.78</v>
       </c>
-      <c r="AD49" s="188">
+      <c r="AD49" s="186">
         <f>+AX111</f>
         <v>107.57</v>
       </c>
-      <c r="AE49" s="190">
+      <c r="AE49" s="188">
         <f>+AZ111</f>
         <v>134.47</v>
       </c>
@@ -6022,58 +6068,58 @@
       <c r="P50" s="120"/>
       <c r="Q50" s="127"/>
       <c r="R50" s="7"/>
-      <c r="S50" s="196"/>
-      <c r="T50" s="197"/>
-      <c r="U50" s="197"/>
-      <c r="V50" s="197"/>
-      <c r="W50" s="197"/>
-      <c r="X50" s="188"/>
-      <c r="Y50" s="188"/>
-      <c r="Z50" s="188"/>
-      <c r="AA50" s="188"/>
-      <c r="AB50" s="188"/>
-      <c r="AC50" s="188"/>
-      <c r="AD50" s="188"/>
-      <c r="AE50" s="190"/>
+      <c r="S50" s="194"/>
+      <c r="T50" s="195"/>
+      <c r="U50" s="195"/>
+      <c r="V50" s="195"/>
+      <c r="W50" s="195"/>
+      <c r="X50" s="186"/>
+      <c r="Y50" s="186"/>
+      <c r="Z50" s="186"/>
+      <c r="AA50" s="186"/>
+      <c r="AB50" s="186"/>
+      <c r="AC50" s="186"/>
+      <c r="AD50" s="186"/>
+      <c r="AE50" s="188"/>
     </row>
     <row r="51" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A51" s="2"/>
-      <c r="B51" s="191" t="s">
+      <c r="B51" s="189" t="s">
         <v>74</v>
       </c>
-      <c r="C51" s="191"/>
-      <c r="D51" s="191"/>
-      <c r="E51" s="191"/>
-      <c r="F51" s="192" t="s">
+      <c r="C51" s="189"/>
+      <c r="D51" s="189"/>
+      <c r="E51" s="189"/>
+      <c r="F51" s="190" t="s">
         <v>74</v>
       </c>
-      <c r="G51" s="192"/>
-      <c r="H51" s="192"/>
-      <c r="I51" s="193" t="s">
+      <c r="G51" s="190"/>
+      <c r="H51" s="190"/>
+      <c r="I51" s="191" t="s">
         <v>74</v>
       </c>
-      <c r="J51" s="193"/>
-      <c r="K51" s="193"/>
-      <c r="L51" s="193"/>
-      <c r="M51" s="193"/>
-      <c r="N51" s="193"/>
-      <c r="O51" s="193"/>
-      <c r="P51" s="193"/>
-      <c r="Q51" s="193"/>
+      <c r="J51" s="191"/>
+      <c r="K51" s="191"/>
+      <c r="L51" s="191"/>
+      <c r="M51" s="191"/>
+      <c r="N51" s="191"/>
+      <c r="O51" s="191"/>
+      <c r="P51" s="191"/>
+      <c r="Q51" s="191"/>
       <c r="R51" s="7"/>
-      <c r="S51" s="196"/>
-      <c r="T51" s="197"/>
-      <c r="U51" s="197"/>
-      <c r="V51" s="197"/>
-      <c r="W51" s="197"/>
-      <c r="X51" s="188"/>
-      <c r="Y51" s="188"/>
-      <c r="Z51" s="188"/>
-      <c r="AA51" s="188"/>
-      <c r="AB51" s="188"/>
-      <c r="AC51" s="188"/>
-      <c r="AD51" s="188"/>
-      <c r="AE51" s="190"/>
+      <c r="S51" s="194"/>
+      <c r="T51" s="195"/>
+      <c r="U51" s="195"/>
+      <c r="V51" s="195"/>
+      <c r="W51" s="195"/>
+      <c r="X51" s="186"/>
+      <c r="Y51" s="186"/>
+      <c r="Z51" s="186"/>
+      <c r="AA51" s="186"/>
+      <c r="AB51" s="186"/>
+      <c r="AC51" s="186"/>
+      <c r="AD51" s="186"/>
+      <c r="AE51" s="188"/>
     </row>
     <row r="52" spans="1:62" ht="13.5" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A52" s="2"/>
@@ -6140,11 +6186,11 @@
     <row r="57" spans="1:62" hidden="1" x14ac:dyDescent="0.2">
       <c r="AJ57" s="77">
         <f>AE29</f>
-        <v>0</v>
+        <v>53.78</v>
       </c>
       <c r="AL57" s="77" t="str">
         <f>TEXT(AE29,"0000,00")</f>
-        <v>0000,00</v>
+        <v>0053,78</v>
       </c>
     </row>
     <row r="58" spans="1:62" hidden="1" x14ac:dyDescent="0.2"/>
@@ -6226,19 +6272,19 @@
       </c>
       <c r="AL66" s="1" t="str">
         <f>IF(MID($AL$57,$AL$75-1,1)="1",MID($AL$57,$AL75-1,2),MID($AL$57,$AL$75,1))</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="AM66" s="1" t="str">
         <f ca="1">LOOKUP(VALUE(AL66),$AI$64:$AI$103,$AJ$64:$AJ$8727)</f>
-        <v xml:space="preserve"> </v>
+        <v>oito</v>
       </c>
       <c r="AN66" s="1" t="str">
         <f t="shared" ref="AN66:AN71" si="8">IF(AL66="0","F","T")</f>
-        <v>F</v>
+        <v>T</v>
       </c>
       <c r="AO66" s="1" t="str">
         <f ca="1">IF(AND(AL67="0",AL69="0",AL71="0"),AM70&amp;" e "&amp;AM68&amp;AL77&amp;AM66&amp;AM77,AM67&amp;" e "&amp;AM66&amp;AM77)</f>
-        <v xml:space="preserve">  e   real   centavo </v>
+        <v xml:space="preserve">setenta e oito centavos </v>
       </c>
     </row>
     <row r="67" spans="33:62" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6255,15 +6301,15 @@
       </c>
       <c r="AL67" s="1" t="str">
         <f>IF(MID($AL$57,$AL$75-1,1)&gt;"1",MID($AL$57,$AL$75-1,1),"0")</f>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="AM67" s="1" t="str">
         <f ca="1">LOOKUP(VALUE(AL67)*10,$AI$64:$AI$103,$AJ$64:$AJ$8727)</f>
-        <v xml:space="preserve"> </v>
+        <v>setenta</v>
       </c>
       <c r="AN67" s="1" t="str">
         <f t="shared" si="8"/>
-        <v>F</v>
+        <v>T</v>
       </c>
       <c r="AP67" s="20"/>
       <c r="AQ67" s="20"/>
@@ -6299,15 +6345,15 @@
       </c>
       <c r="AL68" s="1" t="str">
         <f>IF(MID($AL$57,$AL$75-4,1)="1",MID($AL$57,$AL$75-4,2),MID($AL$57,$AL$75-3,1))</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AM68" s="1" t="str">
         <f ca="1">LOOKUP(VALUE(AL68),$AI$64:$AI$103,$AJ$64:$AJ$8727)</f>
-        <v xml:space="preserve"> </v>
+        <v>três</v>
       </c>
       <c r="AN68" s="1" t="str">
         <f t="shared" si="8"/>
-        <v>F</v>
+        <v>T</v>
       </c>
     </row>
     <row r="69" spans="33:62" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6322,15 +6368,15 @@
       </c>
       <c r="AL69" s="1" t="str">
         <f>IF(MID($AL$57,$AL$75-4,1)&gt;"1",MID($AL$57,$AL$75-4,1),"0")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AM69" s="1" t="str">
         <f>LOOKUP(VALUE(AL69)*10,$AI$64:$AI$103,$AJ$64:$AJ$103)</f>
-        <v xml:space="preserve"> </v>
+        <v>cinqüenta</v>
       </c>
       <c r="AN69" s="1" t="str">
         <f t="shared" si="8"/>
-        <v>F</v>
+        <v>T</v>
       </c>
     </row>
     <row r="70" spans="33:62" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6475,15 +6521,15 @@
       </c>
       <c r="AL77" s="1" t="str">
         <f>IF(VALUE(MID($AL$57,$AL$75-5,4))&gt;1," reais "," real ")</f>
-        <v xml:space="preserve"> real </v>
+        <v xml:space="preserve"> reais </v>
       </c>
       <c r="AM77" s="1" t="str">
         <f>IF(VALUE(MID($AL$57,$AL$75-1,2))&gt;1," centavos "," centavo ")</f>
-        <v xml:space="preserve"> centavo </v>
+        <v xml:space="preserve"> centavos </v>
       </c>
       <c r="AO77" s="182" t="str">
-        <f>UPPER("*** "&amp;AM78&amp;AM80&amp;AM79&amp;"***")</f>
-        <v>***  ***</v>
+        <f ca="1">UPPER("*** "&amp;AM78&amp;AM80&amp;AM79&amp;"***")</f>
+        <v>*** CINQÜENTA E TRÊS REAIS  E SETENTA E OITO CENTAVOS ***</v>
       </c>
     </row>
     <row r="78" spans="33:62" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6510,14 +6556,14 @@
       </c>
       <c r="AK79" s="1" t="str">
         <f>AN66&amp;AN67</f>
-        <v>FF</v>
+        <v>TT</v>
       </c>
       <c r="AL79" s="1" t="s">
         <v>100</v>
       </c>
       <c r="AM79" s="1" t="str">
-        <f>IF(AN66&amp;AN67="TT"," e "&amp;AM67&amp;" e "&amp;AM66&amp;AM77,IF(AN66&amp;AN67="FF","",IF(AN66&amp;AN67="TF"," e "&amp;AM66&amp;AM77,IF(AN66&amp;AN67="FT"," e "&amp;AM67&amp;AM77))))</f>
-        <v/>
+        <f ca="1">IF(AN66&amp;AN67="TT"," e "&amp;AM67&amp;" e "&amp;AM66&amp;AM77,IF(AN66&amp;AN67="FF","",IF(AN66&amp;AN67="TF"," e "&amp;AM66&amp;AM77,IF(AN66&amp;AN67="FT"," e "&amp;AM67&amp;AM77))))</f>
+        <v xml:space="preserve"> e setenta e oito centavos </v>
       </c>
     </row>
     <row r="80" spans="33:62" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6529,14 +6575,14 @@
       </c>
       <c r="AK80" s="1" t="str">
         <f>AN68&amp;AN69&amp;AN70</f>
-        <v>FFF</v>
+        <v>TTF</v>
       </c>
       <c r="AL80" s="1" t="s">
         <v>102</v>
       </c>
       <c r="AM80" s="1" t="str">
-        <f>IF(AN68&amp;AN69&amp;AN70="TTT",AM70&amp;" e "&amp;AM69&amp;" e "&amp;AM68&amp;AL77,IF(AN68&amp;AN69&amp;AN70="FTT",AM70&amp;" e "&amp;AM69&amp;AL77,IF(AN68&amp;AN69&amp;AN70="FFT",AM70&amp;AL77,IF(AN68&amp;AN69&amp;AN70="TTF",AM69&amp;" e "&amp;AM68&amp;AL77,IF(AN68&amp;AN69&amp;AN70="TFT",AM70&amp;" e "&amp;AM68&amp;AL77,IF(AN68&amp;AN69&amp;AN70="TFF",AM68&amp;AL77,IF(AN68&amp;AN69&amp;AN70="FFF"," ",IF(AN68&amp;AN69&amp;AN70="FTF",AM69&amp;AL77," "))))))))</f>
-        <v xml:space="preserve"> </v>
+        <f ca="1">IF(AN68&amp;AN69&amp;AN70="TTT",AM70&amp;" e "&amp;AM69&amp;" e "&amp;AM68&amp;AL77,IF(AN68&amp;AN69&amp;AN70="FTT",AM70&amp;" e "&amp;AM69&amp;AL77,IF(AN68&amp;AN69&amp;AN70="FFT",AM70&amp;AL77,IF(AN68&amp;AN69&amp;AN70="TTF",AM69&amp;" e "&amp;AM68&amp;AL77,IF(AN68&amp;AN69&amp;AN70="TFT",AM70&amp;" e "&amp;AM68&amp;AL77,IF(AN68&amp;AN69&amp;AN70="TFF",AM68&amp;AL77,IF(AN68&amp;AN69&amp;AN70="FFF"," ",IF(AN68&amp;AN69&amp;AN70="FTF",AM69&amp;AL77," "))))))))</f>
+        <v xml:space="preserve">cinqüenta e três reais </v>
       </c>
     </row>
     <row r="81" spans="33:75" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6567,7 +6613,7 @@
       </c>
       <c r="AM83" s="1" t="str">
         <f ca="1">AM70&amp;" e "&amp;AM69&amp;" e "&amp;AM68&amp;AL77</f>
-        <v xml:space="preserve">  e   e   real </v>
+        <v xml:space="preserve">  e cinqüenta e três reais </v>
       </c>
       <c r="AO83" s="1" t="s">
         <v>107</v>
@@ -6588,7 +6634,7 @@
       </c>
       <c r="AM84" s="1" t="str">
         <f ca="1">AM70&amp;" e "&amp;AM69&amp;AL77</f>
-        <v xml:space="preserve">  e   real </v>
+        <v xml:space="preserve">  e cinqüenta reais </v>
       </c>
       <c r="AN84" s="1"/>
       <c r="AO84" s="1" t="s">
@@ -6644,7 +6690,7 @@
       </c>
       <c r="AM85" s="1" t="str">
         <f ca="1">AM70&amp;AL77</f>
-        <v xml:space="preserve">  real </v>
+        <v xml:space="preserve">  reais </v>
       </c>
       <c r="AN85" s="1"/>
       <c r="AO85" s="1" t="s">
@@ -6721,7 +6767,7 @@
       </c>
       <c r="AM87" s="1" t="str">
         <f>AM69&amp;AL77</f>
-        <v xml:space="preserve">  real </v>
+        <v xml:space="preserve">cinqüenta reais </v>
       </c>
       <c r="AO87" s="1" t="s">
         <v>118</v>
@@ -6752,7 +6798,7 @@
       </c>
       <c r="AM88" s="1" t="str">
         <f ca="1">AM69&amp;" e "&amp;AM68&amp;AL77</f>
-        <v xml:space="preserve">  e   real </v>
+        <v xml:space="preserve">cinqüenta e três reais </v>
       </c>
       <c r="AO88" s="1" t="s">
         <v>121</v>
@@ -6783,7 +6829,7 @@
       </c>
       <c r="AM89" s="1" t="str">
         <f ca="1">AM70&amp;" e "&amp;AM68&amp;AL77</f>
-        <v xml:space="preserve">  e   real </v>
+        <v xml:space="preserve">  e três reais </v>
       </c>
       <c r="AO89" s="1" t="s">
         <v>124</v>
@@ -6814,7 +6860,7 @@
       </c>
       <c r="AM90" s="1" t="str">
         <f>AM69&amp;AL77</f>
-        <v xml:space="preserve">  real </v>
+        <v xml:space="preserve">cinqüenta reais </v>
       </c>
       <c r="AO90" s="1" t="s">
         <v>118</v>
@@ -6867,7 +6913,7 @@
       </c>
       <c r="AM92" s="1" t="str">
         <f ca="1">AM67&amp;" e "&amp;AM66&amp;AM77</f>
-        <v xml:space="preserve">  e   centavo </v>
+        <v xml:space="preserve">setenta e oito centavos </v>
       </c>
       <c r="AO92" s="1" t="s">
         <v>130</v>
@@ -6898,7 +6944,7 @@
       </c>
       <c r="AM93" s="1" t="str">
         <f ca="1">AM67&amp;AM77</f>
-        <v xml:space="preserve">  centavo </v>
+        <v xml:space="preserve">setenta centavos </v>
       </c>
       <c r="AO93" s="1" t="s">
         <v>133</v>
@@ -6959,7 +7005,7 @@
       </c>
       <c r="AM95" s="1" t="str">
         <f ca="1">AM66&amp;AM77</f>
-        <v xml:space="preserve">  centavo </v>
+        <v xml:space="preserve">oito centavos </v>
       </c>
       <c r="AO95" s="1" t="s">
         <v>139</v>
@@ -7072,22 +7118,22 @@
       <c r="AP104" s="138" t="s">
         <v>29</v>
       </c>
-      <c r="AQ104" s="194" t="s">
+      <c r="AQ104" s="192" t="s">
         <v>30</v>
       </c>
-      <c r="AR104" s="194"/>
-      <c r="AS104" s="194"/>
-      <c r="AT104" s="194"/>
-      <c r="AU104" s="195" t="s">
+      <c r="AR104" s="192"/>
+      <c r="AS104" s="192"/>
+      <c r="AT104" s="192"/>
+      <c r="AU104" s="193" t="s">
         <v>31</v>
       </c>
-      <c r="AV104" s="195"/>
-      <c r="AW104" s="195"/>
-      <c r="AX104" s="195"/>
-      <c r="AY104" s="189" t="s">
+      <c r="AV104" s="193"/>
+      <c r="AW104" s="193"/>
+      <c r="AX104" s="193"/>
+      <c r="AY104" s="187" t="s">
         <v>32</v>
       </c>
-      <c r="AZ104" s="189"/>
+      <c r="AZ104" s="187"/>
       <c r="BA104" s="6"/>
       <c r="BB104" s="6"/>
       <c r="BC104" s="6"/>
@@ -7879,42 +7925,44 @@
     </row>
     <row r="10" spans="1:29" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="15" spans="1:29" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A15" s="186" t="s">
+      <c r="A15" s="271" t="s">
         <v>163</v>
       </c>
-      <c r="B15" s="186"/>
-      <c r="C15" s="186"/>
-      <c r="D15" s="186"/>
-      <c r="E15" s="186"/>
-      <c r="F15" s="186"/>
-      <c r="G15" s="186"/>
-      <c r="H15" s="186"/>
-      <c r="I15" s="186"/>
-      <c r="J15" s="186"/>
-      <c r="K15" s="186"/>
-      <c r="L15" s="186"/>
-      <c r="M15" s="186"/>
-      <c r="N15" s="186"/>
-      <c r="O15" s="186"/>
+      <c r="B15" s="271"/>
+      <c r="C15" s="271"/>
+      <c r="D15" s="271"/>
+      <c r="E15" s="271"/>
+      <c r="F15" s="271"/>
+      <c r="G15" s="271"/>
+      <c r="H15" s="271"/>
+      <c r="I15" s="271"/>
+      <c r="J15" s="271"/>
+      <c r="K15" s="271"/>
+      <c r="L15" s="271"/>
+      <c r="M15" s="271"/>
+      <c r="N15" s="271"/>
+      <c r="O15" s="271"/>
     </row>
     <row r="16" spans="1:29" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A16" s="187" t="s">
-        <v>173</v>
-      </c>
-      <c r="B16" s="187"/>
-      <c r="C16" s="187"/>
-      <c r="D16" s="187"/>
-      <c r="E16" s="187"/>
-      <c r="F16" s="187"/>
-      <c r="G16" s="187"/>
-      <c r="H16" s="187"/>
-      <c r="I16" s="187"/>
-      <c r="J16" s="187"/>
-      <c r="K16" s="187"/>
-      <c r="L16" s="187"/>
-      <c r="M16" s="187"/>
-      <c r="N16" s="187"/>
-      <c r="O16" s="187"/>
+      <c r="A16" s="272" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B16" s="272"/>
+      <c r="C16" s="272"/>
+      <c r="D16" s="272"/>
+      <c r="E16" s="272"/>
+      <c r="F16" s="272"/>
+      <c r="G16" s="272"/>
+      <c r="H16" s="272"/>
+      <c r="I16" s="272"/>
+      <c r="J16" s="272"/>
+      <c r="K16" s="272"/>
+      <c r="L16" s="272"/>
+      <c r="M16" s="272"/>
+      <c r="N16" s="272"/>
+      <c r="O16" s="272"/>
     </row>
     <row r="21" spans="5:8" x14ac:dyDescent="0.2">
       <c r="E21" s="183" t="s">

</xml_diff>

<commit_message>
Implementa melhorias no fluxo de diárias
</commit_message>
<xml_diff>
--- a/modelos/modelo_mapa.xlsx
+++ b/modelos/modelo_mapa.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gustavo\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98ECFAE4-9925-4457-8878-6CC21F0332D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09EF87C2-B1C9-4CB6-8D4F-A3E3C29FB006}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{807D5CED-EEB3-4DB9-8087-ADFB5AE7F696}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{8800D05A-11AB-44C8-952A-A0A169E38BB0}"/>
   </bookViews>
   <sheets>
     <sheet name="Limite 50%" sheetId="1" r:id="rId1"/>
@@ -35,13 +35,11 @@
     <definedName name="Z_FF834EEA_98EE_4D52_930D_AE89D7F4F75B_.wvu.Cols" localSheetId="0" hidden="1">'Limite 50%'!$AF:$AZ</definedName>
     <definedName name="Z_FF834EEA_98EE_4D52_930D_AE89D7F4F75B_.wvu.PrintArea" localSheetId="0" hidden="1">'Limite 50%'!$A$1:$AE$51</definedName>
     <definedName name="Z_FF834EEA_98EE_4D52_930D_AE89D7F4F75B_.wvu.Rows" localSheetId="0" hidden="1">'Limite 50%'!$53:$152</definedName>
-    <definedName name="_SIG_DIARIAS_B34_TEMPLATE_001" hidden="1">"PGlzPjx0PkFzc3VtaXIgbyBQbGFudMOjbyBuYSBDZW50cmFsIGRlIFBvbMOtY2lhIEp1ZGljacOhcmlhIGRlIHt7e2NpZGFkZV9wbGFudGFvfX19LVNQLCBjb25mb3JtZSBkZXRlcm1pbmHDp8OjbyBjb250aWRhIG5hIEVzY2FsYSByZWZlcmVudGUgYSB7e3tkYXRh"</definedName>
-    <definedName name="_SIG_DIARIAS_B34_TEMPLATE_002" hidden="1">"X2lkYX19fTwvdD48L2lzPg=="</definedName>
   </definedNames>
   <calcPr calcId="191029" calcMode="manual" fullPrecision="0"/>
   <customWorkbookViews>
+    <customWorkbookView name="policial - Modo de exibição pessoal" guid="{FF834EEA-98EE-4D52-930D-AE89D7F4F75B}" mergeInterval="0" personalView="1" maximized="1" xWindow="-8" yWindow="-8" windowWidth="1936" windowHeight="1056" tabRatio="500" activeSheetId="1"/>
     <customWorkbookView name=" " guid="{21947858-9CF7-CF4C-8635-4940C68DA20F}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1200" windowHeight="1000" tabRatio="1000" activeSheetId="1"/>
-    <customWorkbookView name="policial - Modo de exibição pessoal" guid="{FF834EEA-98EE-4D52-930D-AE89D7F4F75B}" mergeInterval="0" personalView="1" maximized="1" xWindow="-8" yWindow="-8" windowWidth="1936" windowHeight="1056" tabRatio="500" activeSheetId="1"/>
   </customWorkbookViews>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -60,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="178">
   <si>
     <t xml:space="preserve">SECRETARIA DE ESTADO DOS NEGÓCIOS DA SEGURANÇA PÚBLICA </t>
   </si>
@@ -573,43 +571,52 @@
     <t>Superior a 200.000 habit. e mais de 70 Km</t>
   </si>
   <si>
-    <t>DELPOL TAGUAÍ</t>
-  </si>
-  <si>
     <t>PROTOCOLO "S" DO REQUERIMENTO:</t>
   </si>
   <si>
     <t>Demais Delocamentos</t>
   </si>
   <si>
-    <t>GUSTAVO SILVA ALMEIDA</t>
-  </si>
-  <si>
     <t>45.027.980-7</t>
   </si>
   <si>
-    <t>369.002.488-96</t>
-  </si>
-  <si>
-    <t>001 / 203-8 / 129065-7</t>
-  </si>
-  <si>
-    <t>TAQUARITUBA</t>
-  </si>
-  <si>
     <t>II</t>
   </si>
   <si>
-    <t>AGENTE POLICIAL 2ª CLASSE</t>
-  </si>
-  <si>
-    <t>PARTICULAR</t>
-  </si>
-  <si>
     <t>215626/2026</t>
   </si>
   <si>
     <t>Assumir o Plantão na Central de Polícia Judiciária de {{{cidade_plantao}}}-SP, conforme determinação contida na Escala referente a {{{data_ida}}}</t>
+  </si>
+  <si>
+    <t>data protocoloo</t>
+  </si>
+  <si>
+    <t>delegacia abrev</t>
+  </si>
+  <si>
+    <t>NOME COMPLETO</t>
+  </si>
+  <si>
+    <t>CARGO E CLASSE</t>
+  </si>
+  <si>
+    <t>CIDADE PLANTAO</t>
+  </si>
+  <si>
+    <t>MEIO</t>
+  </si>
+  <si>
+    <t>ida</t>
+  </si>
+  <si>
+    <t>volta</t>
+  </si>
+  <si>
+    <t>001 / 123-4 / 123456-7</t>
+  </si>
+  <si>
+    <t>123.456.789-01</t>
   </si>
 </sst>
 </file>
@@ -2269,276 +2276,6 @@
     <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="14" fontId="44" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
-    <xf numFmtId="4" fontId="25" fillId="0" borderId="31" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="7" borderId="24" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="25" fillId="0" borderId="29" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="32" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="34" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="5" borderId="24" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="6" borderId="24" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="35" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="32" fillId="0" borderId="31" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="25" fillId="0" borderId="24" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="25" fillId="0" borderId="28" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="9" fillId="0" borderId="36" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="9" fillId="2" borderId="37" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="9" fillId="0" borderId="21" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="32" fillId="0" borderId="15" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="38" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="33" fillId="0" borderId="24" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="32" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="33" fillId="0" borderId="26" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="24" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="29" fillId="0" borderId="24" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="25" fillId="2" borderId="11" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="25" fillId="2" borderId="12" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="25" fillId="2" borderId="17" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="25" fillId="2" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="25" fillId="2" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="25" fillId="2" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="25" fillId="2" borderId="6" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="25" fillId="2" borderId="7" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="25" fillId="2" borderId="8" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="39" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="38" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" indent="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="14" fillId="0" borderId="38" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="23" fillId="0" borderId="35" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="40" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="40" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="38" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="24" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="24" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="4" fontId="1" fillId="0" borderId="24" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="24" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="38" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="38" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="41" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="21" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="20" fontId="1" fillId="2" borderId="21" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="4" fontId="1" fillId="0" borderId="22" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="1" fillId="0" borderId="21" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="24" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="41" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="4" fontId="1" fillId="0" borderId="23" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="45" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="46" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="42" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="12" fillId="2" borderId="33" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="43" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="44" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="8" fillId="0" borderId="34" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="31" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="46" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
@@ -2591,6 +2328,276 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="42" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="12" fillId="2" borderId="33" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="43" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="44" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="8" fillId="0" borderId="34" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="31" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="46" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="41" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="21" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="20" fontId="1" fillId="2" borderId="21" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="21" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="16" fillId="0" borderId="24" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="41" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="23" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="45" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="46" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="22" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="25" fillId="2" borderId="11" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="25" fillId="2" borderId="12" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="25" fillId="2" borderId="17" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="25" fillId="2" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="25" fillId="2" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="25" fillId="2" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="25" fillId="2" borderId="6" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="25" fillId="2" borderId="7" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="25" fillId="2" borderId="8" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="39" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="38" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" indent="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="14" fillId="0" borderId="38" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="23" fillId="0" borderId="35" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="40" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="40" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="38" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="24" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="24" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="24" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="24" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="38" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="24" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="25" fillId="0" borderId="24" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="38" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="25" fillId="0" borderId="28" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="38" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="29" fillId="0" borderId="24" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="2" borderId="37" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="0" borderId="21" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="32" fillId="0" borderId="15" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="33" fillId="0" borderId="24" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="32" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="33" fillId="0" borderId="26" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="0" borderId="36" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="25" fillId="0" borderId="31" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="7" borderId="24" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="25" fillId="0" borderId="29" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="32" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="34" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="5" borderId="24" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="6" borderId="24" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="35" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="32" fillId="0" borderId="31" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
     <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2599,10 +2606,10 @@
     </xf>
   </cellXfs>
   <cellStyles count="4">
-    <cellStyle name="Moeda_Diárias preenchimento automatico" xfId="1" xr:uid="{4EFC2F0A-E1D9-4C19-9421-D20B2169BAB5}"/>
+    <cellStyle name="Moeda_Diárias preenchimento automatico" xfId="1" xr:uid="{1EC7ED33-6D83-4595-BE0F-8B24B74AC603}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="2" xr:uid="{4BBE053E-E067-4F02-AF69-813D4B940E9B}"/>
-    <cellStyle name="Normal_Diárias preenchimento automatico" xfId="3" xr:uid="{1FF71112-5CB7-4A98-B10E-709A81FD206D}"/>
+    <cellStyle name="Normal 2" xfId="2" xr:uid="{DF7B6CB9-227F-45B5-9A5D-8273C2EE5A25}"/>
+    <cellStyle name="Normal_Diárias preenchimento automatico" xfId="3" xr:uid="{270F79C4-AC18-4C80-ACEB-DA6E69250766}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2701,7 +2708,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-FAC0-4B9B-89D3-57B495829754}"/>
+              <c16:uniqueId val="{00000000-F3D2-4C01-90D0-C67202EFBE81}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2739,7 +2746,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-FAC0-4B9B-89D3-57B495829754}"/>
+              <c16:uniqueId val="{00000001-F3D2-4C01-90D0-C67202EFBE81}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2753,11 +2760,11 @@
         </c:dLbls>
         <c:gapWidth val="219"/>
         <c:overlap val="-27"/>
-        <c:axId val="60590048"/>
+        <c:axId val="684523216"/>
         <c:axId val="1"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="60590048"/>
+        <c:axId val="684523216"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2857,7 +2864,7 @@
             <a:endParaRPr lang="pt-BR"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="60590048"/>
+        <c:crossAx val="684523216"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2931,7 +2938,7 @@
 </file>
 
 <file path=xl/chartsheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartsheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" xr:uid="{5D68B3C3-510E-4842-99A1-0405E79F7CCA}">
+<chartsheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" xr:uid="{AE5DA71E-D794-4D28-84DD-62DD38AC5A8D}">
   <sheetPr/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <drawing r:id="rId1"/>
@@ -2958,7 +2965,7 @@
         <xdr:cNvPr id="1659" name="Figura 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{65DD0E9C-D7A2-092F-F56F-804CCA121EBF}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EA692938-C4D3-BF42-91DA-E6C045C78477}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3032,7 +3039,7 @@
         <xdr:cNvPr id="2" name="Gráfico 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D97F29A0-3D4C-FBE2-E128-D0C7ED346593}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{15F1E7FB-7DAC-DCE9-109F-75857AE6600E}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3075,7 +3082,7 @@
         <xdr:cNvPr id="2" name="CaixaDeTexto 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D5B537E6-AC1D-FAB6-EE74-27045A1BD245}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BFDE0E35-93A7-9866-B8F8-C17C4B790770}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3607,7 +3614,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54209629-9520-46AB-8FE2-C44B2C6AE994}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7F51C20-4C5F-4DF2-A904-9C67A6C7D8E0}">
   <sheetPr codeName="Plan1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -3698,33 +3705,33 @@
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
-      <c r="F2" s="264" t="s">
-        <v>0</v>
-      </c>
-      <c r="G2" s="264"/>
-      <c r="H2" s="264"/>
-      <c r="I2" s="264"/>
-      <c r="J2" s="264"/>
-      <c r="K2" s="264"/>
-      <c r="L2" s="264"/>
-      <c r="M2" s="264"/>
-      <c r="N2" s="264"/>
-      <c r="O2" s="264"/>
-      <c r="P2" s="264"/>
-      <c r="Q2" s="264"/>
-      <c r="R2" s="264"/>
-      <c r="S2" s="264"/>
-      <c r="T2" s="264"/>
-      <c r="U2" s="264"/>
-      <c r="V2" s="264"/>
-      <c r="W2" s="264"/>
-      <c r="X2" s="264"/>
-      <c r="Y2" s="264"/>
-      <c r="Z2" s="264"/>
-      <c r="AA2" s="264"/>
-      <c r="AB2" s="264"/>
-      <c r="AC2" s="264"/>
-      <c r="AD2" s="264"/>
+      <c r="F2" s="196" t="s">
+        <v>0</v>
+      </c>
+      <c r="G2" s="196"/>
+      <c r="H2" s="196"/>
+      <c r="I2" s="196"/>
+      <c r="J2" s="196"/>
+      <c r="K2" s="196"/>
+      <c r="L2" s="196"/>
+      <c r="M2" s="196"/>
+      <c r="N2" s="196"/>
+      <c r="O2" s="196"/>
+      <c r="P2" s="196"/>
+      <c r="Q2" s="196"/>
+      <c r="R2" s="196"/>
+      <c r="S2" s="196"/>
+      <c r="T2" s="196"/>
+      <c r="U2" s="196"/>
+      <c r="V2" s="196"/>
+      <c r="W2" s="196"/>
+      <c r="X2" s="196"/>
+      <c r="Y2" s="196"/>
+      <c r="Z2" s="196"/>
+      <c r="AA2" s="196"/>
+      <c r="AB2" s="196"/>
+      <c r="AC2" s="196"/>
+      <c r="AD2" s="196"/>
       <c r="AE2" s="5"/>
       <c r="AF2" s="6"/>
       <c r="AG2" s="6"/>
@@ -3732,33 +3739,33 @@
     <row r="3" spans="1:38" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2"/>
       <c r="B3" s="7"/>
-      <c r="F3" s="265" t="s">
+      <c r="F3" s="197" t="s">
         <v>1</v>
       </c>
-      <c r="G3" s="265"/>
-      <c r="H3" s="265"/>
-      <c r="I3" s="265"/>
-      <c r="J3" s="265"/>
-      <c r="K3" s="265"/>
-      <c r="L3" s="265"/>
-      <c r="M3" s="265"/>
-      <c r="N3" s="265"/>
-      <c r="O3" s="265"/>
-      <c r="P3" s="265"/>
-      <c r="Q3" s="265"/>
-      <c r="R3" s="265"/>
-      <c r="S3" s="265"/>
-      <c r="T3" s="265"/>
-      <c r="U3" s="265"/>
-      <c r="V3" s="265"/>
-      <c r="W3" s="265"/>
-      <c r="X3" s="265"/>
-      <c r="Y3" s="265"/>
-      <c r="Z3" s="265"/>
-      <c r="AA3" s="265"/>
-      <c r="AB3" s="265"/>
-      <c r="AC3" s="265"/>
-      <c r="AD3" s="265"/>
+      <c r="G3" s="197"/>
+      <c r="H3" s="197"/>
+      <c r="I3" s="197"/>
+      <c r="J3" s="197"/>
+      <c r="K3" s="197"/>
+      <c r="L3" s="197"/>
+      <c r="M3" s="197"/>
+      <c r="N3" s="197"/>
+      <c r="O3" s="197"/>
+      <c r="P3" s="197"/>
+      <c r="Q3" s="197"/>
+      <c r="R3" s="197"/>
+      <c r="S3" s="197"/>
+      <c r="T3" s="197"/>
+      <c r="U3" s="197"/>
+      <c r="V3" s="197"/>
+      <c r="W3" s="197"/>
+      <c r="X3" s="197"/>
+      <c r="Y3" s="197"/>
+      <c r="Z3" s="197"/>
+      <c r="AA3" s="197"/>
+      <c r="AB3" s="197"/>
+      <c r="AC3" s="197"/>
+      <c r="AD3" s="197"/>
       <c r="AE3" s="8"/>
       <c r="AF3" s="6"/>
       <c r="AG3" s="6"/>
@@ -3766,33 +3773,33 @@
     <row r="4" spans="1:38" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2"/>
       <c r="B4" s="7"/>
-      <c r="F4" s="265" t="s">
+      <c r="F4" s="197" t="s">
         <v>2</v>
       </c>
-      <c r="G4" s="265"/>
-      <c r="H4" s="265"/>
-      <c r="I4" s="265"/>
-      <c r="J4" s="265"/>
-      <c r="K4" s="265"/>
-      <c r="L4" s="265"/>
-      <c r="M4" s="265"/>
-      <c r="N4" s="265"/>
-      <c r="O4" s="265"/>
-      <c r="P4" s="265"/>
-      <c r="Q4" s="265"/>
-      <c r="R4" s="265"/>
-      <c r="S4" s="265"/>
-      <c r="T4" s="265"/>
-      <c r="U4" s="265"/>
-      <c r="V4" s="265"/>
-      <c r="W4" s="265"/>
-      <c r="X4" s="265"/>
-      <c r="Y4" s="265"/>
-      <c r="Z4" s="265"/>
-      <c r="AA4" s="265"/>
-      <c r="AB4" s="265"/>
-      <c r="AC4" s="265"/>
-      <c r="AD4" s="265"/>
+      <c r="G4" s="197"/>
+      <c r="H4" s="197"/>
+      <c r="I4" s="197"/>
+      <c r="J4" s="197"/>
+      <c r="K4" s="197"/>
+      <c r="L4" s="197"/>
+      <c r="M4" s="197"/>
+      <c r="N4" s="197"/>
+      <c r="O4" s="197"/>
+      <c r="P4" s="197"/>
+      <c r="Q4" s="197"/>
+      <c r="R4" s="197"/>
+      <c r="S4" s="197"/>
+      <c r="T4" s="197"/>
+      <c r="U4" s="197"/>
+      <c r="V4" s="197"/>
+      <c r="W4" s="197"/>
+      <c r="X4" s="197"/>
+      <c r="Y4" s="197"/>
+      <c r="Z4" s="197"/>
+      <c r="AA4" s="197"/>
+      <c r="AB4" s="197"/>
+      <c r="AC4" s="197"/>
+      <c r="AD4" s="197"/>
       <c r="AE4" s="8"/>
       <c r="AF4" s="6"/>
       <c r="AG4" s="6"/>
@@ -3803,33 +3810,33 @@
       <c r="C5" s="10"/>
       <c r="D5" s="10"/>
       <c r="E5" s="10"/>
-      <c r="F5" s="266" t="s">
+      <c r="F5" s="198" t="s">
         <v>3</v>
       </c>
-      <c r="G5" s="266"/>
-      <c r="H5" s="266"/>
-      <c r="I5" s="266"/>
-      <c r="J5" s="266"/>
-      <c r="K5" s="266"/>
-      <c r="L5" s="266"/>
-      <c r="M5" s="266"/>
-      <c r="N5" s="266"/>
-      <c r="O5" s="266"/>
-      <c r="P5" s="266"/>
-      <c r="Q5" s="266"/>
-      <c r="R5" s="266"/>
-      <c r="S5" s="266"/>
-      <c r="T5" s="266"/>
-      <c r="U5" s="266"/>
-      <c r="V5" s="266"/>
-      <c r="W5" s="266"/>
-      <c r="X5" s="266"/>
-      <c r="Y5" s="266"/>
-      <c r="Z5" s="266"/>
-      <c r="AA5" s="266"/>
-      <c r="AB5" s="266"/>
-      <c r="AC5" s="266"/>
-      <c r="AD5" s="266"/>
+      <c r="G5" s="198"/>
+      <c r="H5" s="198"/>
+      <c r="I5" s="198"/>
+      <c r="J5" s="198"/>
+      <c r="K5" s="198"/>
+      <c r="L5" s="198"/>
+      <c r="M5" s="198"/>
+      <c r="N5" s="198"/>
+      <c r="O5" s="198"/>
+      <c r="P5" s="198"/>
+      <c r="Q5" s="198"/>
+      <c r="R5" s="198"/>
+      <c r="S5" s="198"/>
+      <c r="T5" s="198"/>
+      <c r="U5" s="198"/>
+      <c r="V5" s="198"/>
+      <c r="W5" s="198"/>
+      <c r="X5" s="198"/>
+      <c r="Y5" s="198"/>
+      <c r="Z5" s="198"/>
+      <c r="AA5" s="198"/>
+      <c r="AB5" s="198"/>
+      <c r="AC5" s="198"/>
+      <c r="AD5" s="198"/>
       <c r="AE5" s="11"/>
       <c r="AF5" s="6"/>
       <c r="AG5" s="6"/>
@@ -3839,7 +3846,7 @@
       <c r="AF6" s="6"/>
       <c r="AG6" s="6"/>
     </row>
-    <row r="7" spans="1:38" s="20" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:38" s="20" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2"/>
       <c r="B7" s="12" t="s">
         <v>4</v>
@@ -3884,52 +3891,44 @@
     </row>
     <row r="8" spans="1:38" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2"/>
-      <c r="B8" s="267" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="C8" s="267"/>
-      <c r="D8" s="267"/>
-      <c r="E8" s="267"/>
-      <c r="F8" s="267"/>
-      <c r="G8" s="267"/>
-      <c r="H8" s="267"/>
-      <c r="I8" s="267"/>
-      <c r="J8" s="267"/>
-      <c r="K8" s="267"/>
-      <c r="L8" s="267"/>
-      <c r="M8" s="267"/>
-      <c r="N8" s="268" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="O8" s="268"/>
-      <c r="P8" s="268"/>
-      <c r="Q8" s="268"/>
-      <c r="R8" s="268"/>
-      <c r="S8" s="268"/>
-      <c r="T8" s="269" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="U8" s="269"/>
-      <c r="V8" s="269"/>
-      <c r="W8" s="269"/>
-      <c r="X8" s="269"/>
-      <c r="Y8" s="269"/>
-      <c r="Z8" s="269"/>
-      <c r="AA8" s="269"/>
-      <c r="AB8" s="269"/>
-      <c r="AC8" s="270" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="AD8" s="270"/>
-      <c r="AE8" s="270"/>
+      <c r="B8" s="199" t="s">
+        <v>170</v>
+      </c>
+      <c r="C8" s="199"/>
+      <c r="D8" s="199"/>
+      <c r="E8" s="199"/>
+      <c r="F8" s="199"/>
+      <c r="G8" s="199"/>
+      <c r="H8" s="199"/>
+      <c r="I8" s="199"/>
+      <c r="J8" s="199"/>
+      <c r="K8" s="199"/>
+      <c r="L8" s="199"/>
+      <c r="M8" s="199"/>
+      <c r="N8" s="200" t="s">
+        <v>164</v>
+      </c>
+      <c r="O8" s="200"/>
+      <c r="P8" s="200"/>
+      <c r="Q8" s="200"/>
+      <c r="R8" s="200"/>
+      <c r="S8" s="200"/>
+      <c r="T8" s="201" t="s">
+        <v>169</v>
+      </c>
+      <c r="U8" s="201"/>
+      <c r="V8" s="201"/>
+      <c r="W8" s="201"/>
+      <c r="X8" s="201"/>
+      <c r="Y8" s="201"/>
+      <c r="Z8" s="201"/>
+      <c r="AA8" s="201"/>
+      <c r="AB8" s="201"/>
+      <c r="AC8" s="202" t="s">
+        <v>168</v>
+      </c>
+      <c r="AD8" s="202"/>
+      <c r="AE8" s="202"/>
       <c r="AF8" s="6"/>
       <c r="AG8" s="6"/>
       <c r="AH8" s="21"/>
@@ -3961,11 +3960,11 @@
       <c r="P9" s="29"/>
       <c r="Q9" s="29"/>
       <c r="R9" s="26"/>
-      <c r="S9" s="254" t="s">
+      <c r="S9" s="186" t="s">
         <v>12</v>
       </c>
-      <c r="T9" s="254"/>
-      <c r="U9" s="254"/>
+      <c r="T9" s="186"/>
+      <c r="U9" s="186"/>
       <c r="V9" s="30" t="s">
         <v>13</v>
       </c>
@@ -3985,105 +3984,95 @@
     </row>
     <row r="10" spans="1:38" s="20" customFormat="1" ht="8.4499999999999993" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
-      <c r="B10" s="255" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="C10" s="255"/>
-      <c r="D10" s="255"/>
-      <c r="E10" s="256" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="F10" s="256"/>
-      <c r="G10" s="256"/>
-      <c r="H10" s="256"/>
-      <c r="I10" s="256"/>
-      <c r="J10" s="256"/>
-      <c r="K10" s="257" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="L10" s="258"/>
-      <c r="M10" s="259"/>
-      <c r="N10" s="263">
+      <c r="B10" s="187" t="s">
+        <v>165</v>
+      </c>
+      <c r="C10" s="187"/>
+      <c r="D10" s="187"/>
+      <c r="E10" s="188" t="s">
+        <v>171</v>
+      </c>
+      <c r="F10" s="188"/>
+      <c r="G10" s="188"/>
+      <c r="H10" s="188"/>
+      <c r="I10" s="188"/>
+      <c r="J10" s="188"/>
+      <c r="K10" s="189">
+        <v>1234.56</v>
+      </c>
+      <c r="L10" s="190"/>
+      <c r="M10" s="191"/>
+      <c r="N10" s="195">
         <f>+K10/2</f>
-        <v>3790.74</v>
-      </c>
-      <c r="O10" s="263"/>
-      <c r="P10" s="263"/>
-      <c r="Q10" s="263"/>
-      <c r="R10" s="263"/>
+        <v>617.28</v>
+      </c>
+      <c r="O10" s="195"/>
+      <c r="P10" s="195"/>
+      <c r="Q10" s="195"/>
+      <c r="R10" s="195"/>
       <c r="S10" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="T10" s="254" t="s">
+      <c r="T10" s="186" t="s">
         <v>17</v>
       </c>
-      <c r="U10" s="254"/>
-      <c r="V10" s="248" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="W10" s="248"/>
-      <c r="X10" s="248"/>
-      <c r="Y10" s="248"/>
-      <c r="Z10" s="249" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="AA10" s="250" t="s">
+      <c r="U10" s="186"/>
+      <c r="V10" s="206">
+        <v>12.34</v>
+      </c>
+      <c r="W10" s="206"/>
+      <c r="X10" s="206"/>
+      <c r="Y10" s="206"/>
+      <c r="Z10" s="207">
+        <v>7</v>
+      </c>
+      <c r="AA10" s="208" t="s">
         <v>18</v>
       </c>
-      <c r="AB10" s="250"/>
-      <c r="AC10" s="251">
+      <c r="AB10" s="208"/>
+      <c r="AC10" s="209">
         <f>+Z10*V10</f>
-        <v>268.94</v>
-      </c>
-      <c r="AD10" s="251"/>
-      <c r="AE10" s="251"/>
+        <v>86.38</v>
+      </c>
+      <c r="AD10" s="209"/>
+      <c r="AE10" s="209"/>
       <c r="AF10" s="6"/>
       <c r="AG10" s="6"/>
     </row>
     <row r="11" spans="1:38" ht="11.1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
-      <c r="B11" s="255"/>
-      <c r="C11" s="255"/>
-      <c r="D11" s="255"/>
-      <c r="E11" s="256"/>
-      <c r="F11" s="256"/>
-      <c r="G11" s="256"/>
-      <c r="H11" s="256"/>
-      <c r="I11" s="256"/>
-      <c r="J11" s="256"/>
-      <c r="K11" s="260"/>
-      <c r="L11" s="261"/>
-      <c r="M11" s="262"/>
-      <c r="N11" s="263"/>
-      <c r="O11" s="263"/>
-      <c r="P11" s="263"/>
-      <c r="Q11" s="263"/>
-      <c r="R11" s="263"/>
+      <c r="B11" s="187"/>
+      <c r="C11" s="187"/>
+      <c r="D11" s="187"/>
+      <c r="E11" s="188"/>
+      <c r="F11" s="188"/>
+      <c r="G11" s="188"/>
+      <c r="H11" s="188"/>
+      <c r="I11" s="188"/>
+      <c r="J11" s="188"/>
+      <c r="K11" s="192"/>
+      <c r="L11" s="193"/>
+      <c r="M11" s="194"/>
+      <c r="N11" s="195"/>
+      <c r="O11" s="195"/>
+      <c r="P11" s="195"/>
+      <c r="Q11" s="195"/>
+      <c r="R11" s="195"/>
       <c r="S11" s="35"/>
-      <c r="T11" s="252" t="s">
+      <c r="T11" s="210" t="s">
         <v>19</v>
       </c>
-      <c r="U11" s="252"/>
-      <c r="V11" s="248"/>
-      <c r="W11" s="248"/>
-      <c r="X11" s="248"/>
-      <c r="Y11" s="248"/>
-      <c r="Z11" s="249"/>
-      <c r="AA11" s="250"/>
-      <c r="AB11" s="250"/>
-      <c r="AC11" s="251"/>
-      <c r="AD11" s="251"/>
-      <c r="AE11" s="251"/>
+      <c r="U11" s="210"/>
+      <c r="V11" s="206"/>
+      <c r="W11" s="206"/>
+      <c r="X11" s="206"/>
+      <c r="Y11" s="206"/>
+      <c r="Z11" s="207"/>
+      <c r="AA11" s="208"/>
+      <c r="AB11" s="208"/>
+      <c r="AC11" s="209"/>
+      <c r="AD11" s="209"/>
+      <c r="AE11" s="209"/>
       <c r="AF11" s="6"/>
       <c r="AG11" s="6"/>
     </row>
@@ -4125,48 +4114,48 @@
     </row>
     <row r="13" spans="1:38" s="45" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="2"/>
-      <c r="B13" s="242" t="s">
+      <c r="B13" s="220" t="s">
         <v>20</v>
       </c>
-      <c r="C13" s="242"/>
-      <c r="D13" s="242"/>
-      <c r="E13" s="242"/>
+      <c r="C13" s="220"/>
+      <c r="D13" s="220"/>
+      <c r="E13" s="220"/>
       <c r="F13" s="43" t="s">
         <v>21</v>
       </c>
-      <c r="G13" s="243" t="s">
+      <c r="G13" s="221" t="s">
         <v>22</v>
       </c>
-      <c r="H13" s="243"/>
-      <c r="I13" s="243"/>
-      <c r="J13" s="244" t="s">
+      <c r="H13" s="221"/>
+      <c r="I13" s="221"/>
+      <c r="J13" s="222" t="s">
         <v>23</v>
       </c>
-      <c r="K13" s="244"/>
-      <c r="L13" s="244" t="s">
+      <c r="K13" s="222"/>
+      <c r="L13" s="222" t="s">
         <v>24</v>
       </c>
-      <c r="M13" s="244"/>
-      <c r="N13" s="244"/>
-      <c r="O13" s="244"/>
-      <c r="P13" s="253" t="s">
+      <c r="M13" s="222"/>
+      <c r="N13" s="222"/>
+      <c r="O13" s="222"/>
+      <c r="P13" s="211" t="s">
         <v>25</v>
       </c>
-      <c r="Q13" s="253"/>
-      <c r="R13" s="253"/>
-      <c r="S13" s="253"/>
-      <c r="T13" s="253"/>
-      <c r="U13" s="253"/>
-      <c r="V13" s="253"/>
-      <c r="W13" s="253"/>
-      <c r="X13" s="253"/>
-      <c r="Y13" s="253"/>
-      <c r="Z13" s="253"/>
-      <c r="AA13" s="253"/>
-      <c r="AB13" s="253"/>
-      <c r="AC13" s="253"/>
-      <c r="AD13" s="253"/>
-      <c r="AE13" s="245" t="s">
+      <c r="Q13" s="211"/>
+      <c r="R13" s="211"/>
+      <c r="S13" s="211"/>
+      <c r="T13" s="211"/>
+      <c r="U13" s="211"/>
+      <c r="V13" s="211"/>
+      <c r="W13" s="211"/>
+      <c r="X13" s="211"/>
+      <c r="Y13" s="211"/>
+      <c r="Z13" s="211"/>
+      <c r="AA13" s="211"/>
+      <c r="AB13" s="211"/>
+      <c r="AC13" s="211"/>
+      <c r="AD13" s="211"/>
+      <c r="AE13" s="203" t="s">
         <v>26</v>
       </c>
       <c r="AF13" s="6"/>
@@ -4175,66 +4164,66 @@
     </row>
     <row r="14" spans="1:38" s="45" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="2"/>
-      <c r="B14" s="242"/>
-      <c r="C14" s="242"/>
-      <c r="D14" s="242"/>
-      <c r="E14" s="242"/>
+      <c r="B14" s="220"/>
+      <c r="C14" s="220"/>
+      <c r="D14" s="220"/>
+      <c r="E14" s="220"/>
       <c r="F14" s="46" t="s">
         <v>27</v>
       </c>
-      <c r="G14" s="243"/>
-      <c r="H14" s="243"/>
-      <c r="I14" s="243"/>
-      <c r="J14" s="244"/>
-      <c r="K14" s="244"/>
-      <c r="L14" s="244"/>
-      <c r="M14" s="244"/>
-      <c r="N14" s="244"/>
-      <c r="O14" s="244"/>
-      <c r="P14" s="246" t="s">
+      <c r="G14" s="221"/>
+      <c r="H14" s="221"/>
+      <c r="I14" s="221"/>
+      <c r="J14" s="222"/>
+      <c r="K14" s="222"/>
+      <c r="L14" s="222"/>
+      <c r="M14" s="222"/>
+      <c r="N14" s="222"/>
+      <c r="O14" s="222"/>
+      <c r="P14" s="204" t="s">
         <v>28</v>
       </c>
-      <c r="Q14" s="246" t="s">
+      <c r="Q14" s="204" t="s">
         <v>29</v>
       </c>
-      <c r="R14" s="246" t="s">
+      <c r="R14" s="204" t="s">
         <v>30</v>
       </c>
-      <c r="S14" s="246"/>
-      <c r="T14" s="246"/>
-      <c r="U14" s="246"/>
-      <c r="V14" s="246"/>
-      <c r="W14" s="246" t="s">
+      <c r="S14" s="204"/>
+      <c r="T14" s="204"/>
+      <c r="U14" s="204"/>
+      <c r="V14" s="204"/>
+      <c r="W14" s="204" t="s">
         <v>31</v>
       </c>
-      <c r="X14" s="246"/>
-      <c r="Y14" s="246"/>
-      <c r="Z14" s="246"/>
-      <c r="AA14" s="246"/>
-      <c r="AB14" s="246"/>
-      <c r="AC14" s="246" t="s">
+      <c r="X14" s="204"/>
+      <c r="Y14" s="204"/>
+      <c r="Z14" s="204"/>
+      <c r="AA14" s="204"/>
+      <c r="AB14" s="204"/>
+      <c r="AC14" s="204" t="s">
         <v>28</v>
       </c>
-      <c r="AD14" s="247" t="s">
+      <c r="AD14" s="205" t="s">
         <v>32</v>
       </c>
-      <c r="AE14" s="245"/>
+      <c r="AE14" s="203"/>
       <c r="AF14" s="6"/>
       <c r="AG14" s="6"/>
       <c r="AH14" s="47"/>
     </row>
     <row r="15" spans="1:38" s="57" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="48"/>
-      <c r="B15" s="242"/>
-      <c r="C15" s="242"/>
-      <c r="D15" s="242"/>
-      <c r="E15" s="242"/>
+      <c r="B15" s="220"/>
+      <c r="C15" s="220"/>
+      <c r="D15" s="220"/>
+      <c r="E15" s="220"/>
       <c r="F15" s="49" t="s">
         <v>31</v>
       </c>
-      <c r="G15" s="243"/>
-      <c r="H15" s="243"/>
-      <c r="I15" s="243"/>
+      <c r="G15" s="221"/>
+      <c r="H15" s="221"/>
+      <c r="I15" s="221"/>
       <c r="J15" s="52" t="s">
         <v>33</v>
       </c>
@@ -4244,13 +4233,13 @@
       <c r="L15" s="51" t="s">
         <v>33</v>
       </c>
-      <c r="M15" s="238" t="s">
+      <c r="M15" s="216" t="s">
         <v>34</v>
       </c>
-      <c r="N15" s="238"/>
-      <c r="O15" s="238"/>
-      <c r="P15" s="246"/>
-      <c r="Q15" s="246"/>
+      <c r="N15" s="216"/>
+      <c r="O15" s="216"/>
+      <c r="P15" s="204"/>
+      <c r="Q15" s="204"/>
       <c r="R15" s="52" t="s">
         <v>28</v>
       </c>
@@ -4260,27 +4249,27 @@
       <c r="T15" s="52" t="s">
         <v>28</v>
       </c>
-      <c r="U15" s="238" t="s">
+      <c r="U15" s="216" t="s">
         <v>36</v>
       </c>
-      <c r="V15" s="238"/>
+      <c r="V15" s="216"/>
       <c r="W15" s="52" t="s">
         <v>28</v>
       </c>
-      <c r="X15" s="238" t="s">
+      <c r="X15" s="216" t="s">
         <v>37</v>
       </c>
-      <c r="Y15" s="238"/>
+      <c r="Y15" s="216"/>
       <c r="Z15" s="52" t="s">
         <v>28</v>
       </c>
-      <c r="AA15" s="238" t="s">
+      <c r="AA15" s="216" t="s">
         <v>38</v>
       </c>
-      <c r="AB15" s="238"/>
-      <c r="AC15" s="246"/>
-      <c r="AD15" s="247"/>
-      <c r="AE15" s="245"/>
+      <c r="AB15" s="216"/>
+      <c r="AC15" s="204"/>
+      <c r="AD15" s="205"/>
+      <c r="AE15" s="203"/>
       <c r="AF15" s="53"/>
       <c r="AG15" s="53"/>
       <c r="AH15" s="54"/>
@@ -4291,46 +4280,34 @@
     </row>
     <row r="16" spans="1:38" s="38" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A16" s="2"/>
-      <c r="B16" s="239" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="C16" s="239"/>
-      <c r="D16" s="239"/>
-      <c r="E16" s="239"/>
+      <c r="B16" s="217" t="s">
+        <v>172</v>
+      </c>
+      <c r="C16" s="217"/>
+      <c r="D16" s="217"/>
+      <c r="E16" s="217"/>
       <c r="F16" s="58">
         <v>5</v>
       </c>
-      <c r="G16" s="240" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="H16" s="240"/>
-      <c r="I16" s="240"/>
-      <c r="J16" s="59" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="K16" s="60" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="L16" s="61" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="M16" s="235" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="N16" s="235"/>
-      <c r="O16" s="235"/>
+      <c r="G16" s="218" t="s">
+        <v>173</v>
+      </c>
+      <c r="H16" s="218"/>
+      <c r="I16" s="218"/>
+      <c r="J16" s="59" t="s">
+        <v>174</v>
+      </c>
+      <c r="K16" s="60">
+        <v>5.8159722222222203E-2</v>
+      </c>
+      <c r="L16" s="61" t="s">
+        <v>175</v>
+      </c>
+      <c r="M16" s="214">
+        <v>0.52425925925925898</v>
+      </c>
+      <c r="N16" s="214"/>
+      <c r="O16" s="214"/>
       <c r="P16" s="62"/>
       <c r="Q16" s="63">
         <f t="shared" ref="Q16:Q27" si="0">IF(P16="",0,VLOOKUP(F16,AN$107:AZ$111,3,FALSE)*P16)</f>
@@ -4342,34 +4319,28 @@
         <v>0</v>
       </c>
       <c r="T16" s="61"/>
-      <c r="U16" s="241">
+      <c r="U16" s="219">
         <f t="shared" ref="U16:U27" si="2">IF(T16="",0,VLOOKUP(F16,AN$107:AZ$111,7,FALSE)*T16)</f>
         <v>0</v>
       </c>
-      <c r="V16" s="241" t="e">
+      <c r="V16" s="219" t="e">
         <f t="shared" ref="V16:V27" si="3">IF(U16="",0,VLOOKUP(J$16,AT$107:AV$111,3,FALSE)*U16)</f>
         <v>#N/A</v>
       </c>
-      <c r="W16" s="61" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="X16" s="241">
+      <c r="W16" s="61">
+        <v>1</v>
+      </c>
+      <c r="X16" s="219">
         <f>IF(W16="",0,VLOOKUP(F16,AN$107:AZ$111,9,FALSE)*W16)</f>
-        <v>53.78</v>
-      </c>
-      <c r="Y16" s="241"/>
-      <c r="Z16" s="61" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="AA16" s="237">
+        <v>17.27</v>
+      </c>
+      <c r="Y16" s="219"/>
+      <c r="Z16" s="61"/>
+      <c r="AA16" s="215">
         <f>IF(Z16="",0,VLOOKUP(F16,AN$107:AZ$111,11,FALSE)*Z16)</f>
         <v>0</v>
       </c>
-      <c r="AB16" s="237"/>
+      <c r="AB16" s="215"/>
       <c r="AC16" s="59"/>
       <c r="AD16" s="63">
         <f t="shared" ref="AD16:AD27" si="4">IF(AC16="",0,VLOOKUP(F16,AN$107:AZ$111,13,FALSE)*AC16)</f>
@@ -4377,7 +4348,7 @@
       </c>
       <c r="AE16" s="64">
         <f t="shared" ref="AE16:AE27" si="5">+Q16+S16+U16+X16+AA16+AD16</f>
-        <v>53.78</v>
+        <v>17.27</v>
       </c>
       <c r="AF16" s="6"/>
       <c r="AG16" s="6"/>
@@ -4389,20 +4360,20 @@
     </row>
     <row r="17" spans="1:38" s="38" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A17" s="2"/>
-      <c r="B17" s="233"/>
-      <c r="C17" s="233"/>
-      <c r="D17" s="233"/>
-      <c r="E17" s="233"/>
+      <c r="B17" s="212"/>
+      <c r="C17" s="212"/>
+      <c r="D17" s="212"/>
+      <c r="E17" s="212"/>
       <c r="F17" s="58"/>
-      <c r="G17" s="234"/>
-      <c r="H17" s="234"/>
-      <c r="I17" s="234"/>
+      <c r="G17" s="213"/>
+      <c r="H17" s="213"/>
+      <c r="I17" s="213"/>
       <c r="J17" s="69"/>
       <c r="K17" s="60"/>
       <c r="L17" s="70"/>
-      <c r="M17" s="235"/>
-      <c r="N17" s="235"/>
-      <c r="O17" s="235"/>
+      <c r="M17" s="214"/>
+      <c r="N17" s="214"/>
+      <c r="O17" s="214"/>
       <c r="P17" s="70"/>
       <c r="Q17" s="71">
         <f t="shared" si="0"/>
@@ -4414,26 +4385,26 @@
         <v>0</v>
       </c>
       <c r="T17" s="70"/>
-      <c r="U17" s="237">
+      <c r="U17" s="215">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="V17" s="237" t="e">
+      <c r="V17" s="215" t="e">
         <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="W17" s="70"/>
-      <c r="X17" s="237">
+      <c r="X17" s="215">
         <f t="shared" ref="X17:X27" si="6">IF(W17="",0,VLOOKUP(F17,AN$107:AZ$111,9,FALSE)*W17)</f>
         <v>0</v>
       </c>
-      <c r="Y17" s="237"/>
+      <c r="Y17" s="215"/>
       <c r="Z17" s="70"/>
-      <c r="AA17" s="237">
+      <c r="AA17" s="215">
         <f t="shared" ref="AA17:AA27" si="7">IF(Z17="",0,VLOOKUP(F17,AN$107:AZ$111,11,FALSE)*Z17)</f>
         <v>0</v>
       </c>
-      <c r="AB17" s="237"/>
+      <c r="AB17" s="215"/>
       <c r="AC17" s="70"/>
       <c r="AD17" s="71">
         <f t="shared" si="4"/>
@@ -4453,20 +4424,20 @@
     </row>
     <row r="18" spans="1:38" s="38" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A18" s="2"/>
-      <c r="B18" s="233"/>
-      <c r="C18" s="233"/>
-      <c r="D18" s="233"/>
-      <c r="E18" s="233"/>
+      <c r="B18" s="212"/>
+      <c r="C18" s="212"/>
+      <c r="D18" s="212"/>
+      <c r="E18" s="212"/>
       <c r="F18" s="58"/>
-      <c r="G18" s="234"/>
-      <c r="H18" s="234"/>
-      <c r="I18" s="234"/>
+      <c r="G18" s="213"/>
+      <c r="H18" s="213"/>
+      <c r="I18" s="213"/>
       <c r="J18" s="69"/>
       <c r="K18" s="60"/>
       <c r="L18" s="70"/>
-      <c r="M18" s="235"/>
-      <c r="N18" s="235"/>
-      <c r="O18" s="235"/>
+      <c r="M18" s="214"/>
+      <c r="N18" s="214"/>
+      <c r="O18" s="214"/>
       <c r="P18" s="70"/>
       <c r="Q18" s="71">
         <f t="shared" si="0"/>
@@ -4478,26 +4449,26 @@
         <v>0</v>
       </c>
       <c r="T18" s="70"/>
-      <c r="U18" s="237">
+      <c r="U18" s="215">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="V18" s="237" t="e">
+      <c r="V18" s="215" t="e">
         <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="W18" s="70"/>
-      <c r="X18" s="237">
+      <c r="X18" s="215">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="Y18" s="237"/>
+      <c r="Y18" s="215"/>
       <c r="Z18" s="70"/>
-      <c r="AA18" s="237">
+      <c r="AA18" s="215">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="AB18" s="237"/>
+      <c r="AB18" s="215"/>
       <c r="AC18" s="70"/>
       <c r="AD18" s="71">
         <f t="shared" si="4"/>
@@ -4517,20 +4488,20 @@
     </row>
     <row r="19" spans="1:38" s="38" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A19" s="2"/>
-      <c r="B19" s="233"/>
-      <c r="C19" s="233"/>
-      <c r="D19" s="233"/>
-      <c r="E19" s="233"/>
+      <c r="B19" s="212"/>
+      <c r="C19" s="212"/>
+      <c r="D19" s="212"/>
+      <c r="E19" s="212"/>
       <c r="F19" s="58"/>
-      <c r="G19" s="234"/>
-      <c r="H19" s="234"/>
-      <c r="I19" s="234"/>
+      <c r="G19" s="213"/>
+      <c r="H19" s="213"/>
+      <c r="I19" s="213"/>
       <c r="J19" s="69"/>
       <c r="K19" s="60"/>
       <c r="L19" s="70"/>
-      <c r="M19" s="235"/>
-      <c r="N19" s="235"/>
-      <c r="O19" s="235"/>
+      <c r="M19" s="214"/>
+      <c r="N19" s="214"/>
+      <c r="O19" s="214"/>
       <c r="P19" s="70"/>
       <c r="Q19" s="71">
         <f t="shared" si="0"/>
@@ -4542,26 +4513,26 @@
         <v>0</v>
       </c>
       <c r="T19" s="70"/>
-      <c r="U19" s="237">
+      <c r="U19" s="215">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="V19" s="237" t="e">
+      <c r="V19" s="215" t="e">
         <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="W19" s="70"/>
-      <c r="X19" s="237">
+      <c r="X19" s="215">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="Y19" s="237"/>
+      <c r="Y19" s="215"/>
       <c r="Z19" s="70"/>
-      <c r="AA19" s="237">
+      <c r="AA19" s="215">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="AB19" s="237"/>
+      <c r="AB19" s="215"/>
       <c r="AC19" s="70"/>
       <c r="AD19" s="71">
         <f t="shared" si="4"/>
@@ -4581,20 +4552,20 @@
     </row>
     <row r="20" spans="1:38" s="38" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A20" s="2"/>
-      <c r="B20" s="233"/>
-      <c r="C20" s="233"/>
-      <c r="D20" s="233"/>
-      <c r="E20" s="233"/>
+      <c r="B20" s="212"/>
+      <c r="C20" s="212"/>
+      <c r="D20" s="212"/>
+      <c r="E20" s="212"/>
       <c r="F20" s="58"/>
-      <c r="G20" s="234"/>
-      <c r="H20" s="234"/>
-      <c r="I20" s="234"/>
+      <c r="G20" s="213"/>
+      <c r="H20" s="213"/>
+      <c r="I20" s="213"/>
       <c r="J20" s="70"/>
       <c r="K20" s="60"/>
       <c r="L20" s="70"/>
-      <c r="M20" s="235"/>
-      <c r="N20" s="235"/>
-      <c r="O20" s="235"/>
+      <c r="M20" s="214"/>
+      <c r="N20" s="214"/>
+      <c r="O20" s="214"/>
       <c r="P20" s="70"/>
       <c r="Q20" s="71">
         <f t="shared" si="0"/>
@@ -4606,26 +4577,26 @@
         <v>0</v>
       </c>
       <c r="T20" s="70"/>
-      <c r="U20" s="237">
+      <c r="U20" s="215">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="V20" s="237" t="e">
+      <c r="V20" s="215" t="e">
         <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="W20" s="70"/>
-      <c r="X20" s="237">
+      <c r="X20" s="215">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="Y20" s="237"/>
+      <c r="Y20" s="215"/>
       <c r="Z20" s="70"/>
-      <c r="AA20" s="237">
+      <c r="AA20" s="215">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="AB20" s="237"/>
+      <c r="AB20" s="215"/>
       <c r="AC20" s="70"/>
       <c r="AD20" s="71">
         <f t="shared" si="4"/>
@@ -4645,20 +4616,20 @@
     </row>
     <row r="21" spans="1:38" s="38" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A21" s="2"/>
-      <c r="B21" s="233"/>
-      <c r="C21" s="233"/>
-      <c r="D21" s="233"/>
-      <c r="E21" s="233"/>
+      <c r="B21" s="212"/>
+      <c r="C21" s="212"/>
+      <c r="D21" s="212"/>
+      <c r="E21" s="212"/>
       <c r="F21" s="58"/>
-      <c r="G21" s="234"/>
-      <c r="H21" s="234"/>
-      <c r="I21" s="234"/>
+      <c r="G21" s="213"/>
+      <c r="H21" s="213"/>
+      <c r="I21" s="213"/>
       <c r="J21" s="70"/>
       <c r="K21" s="60"/>
       <c r="L21" s="70"/>
-      <c r="M21" s="235"/>
-      <c r="N21" s="235"/>
-      <c r="O21" s="235"/>
+      <c r="M21" s="214"/>
+      <c r="N21" s="214"/>
+      <c r="O21" s="214"/>
       <c r="P21" s="70"/>
       <c r="Q21" s="71">
         <f t="shared" si="0"/>
@@ -4670,26 +4641,26 @@
         <v>0</v>
       </c>
       <c r="T21" s="70"/>
-      <c r="U21" s="237">
+      <c r="U21" s="215">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="V21" s="237" t="e">
+      <c r="V21" s="215" t="e">
         <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="W21" s="70"/>
-      <c r="X21" s="237">
+      <c r="X21" s="215">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="Y21" s="237"/>
+      <c r="Y21" s="215"/>
       <c r="Z21" s="70"/>
-      <c r="AA21" s="237">
+      <c r="AA21" s="215">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="AB21" s="237"/>
+      <c r="AB21" s="215"/>
       <c r="AC21" s="70"/>
       <c r="AD21" s="71">
         <f t="shared" si="4"/>
@@ -4709,20 +4680,20 @@
     </row>
     <row r="22" spans="1:38" s="38" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A22" s="2"/>
-      <c r="B22" s="233"/>
-      <c r="C22" s="233"/>
-      <c r="D22" s="233"/>
-      <c r="E22" s="233"/>
+      <c r="B22" s="212"/>
+      <c r="C22" s="212"/>
+      <c r="D22" s="212"/>
+      <c r="E22" s="212"/>
       <c r="F22" s="58"/>
-      <c r="G22" s="234"/>
-      <c r="H22" s="234"/>
-      <c r="I22" s="234"/>
+      <c r="G22" s="213"/>
+      <c r="H22" s="213"/>
+      <c r="I22" s="213"/>
       <c r="J22" s="70"/>
       <c r="K22" s="60"/>
       <c r="L22" s="70"/>
-      <c r="M22" s="235"/>
-      <c r="N22" s="235"/>
-      <c r="O22" s="235"/>
+      <c r="M22" s="214"/>
+      <c r="N22" s="214"/>
+      <c r="O22" s="214"/>
       <c r="P22" s="70"/>
       <c r="Q22" s="71">
         <f t="shared" si="0"/>
@@ -4734,26 +4705,26 @@
         <v>0</v>
       </c>
       <c r="T22" s="70"/>
-      <c r="U22" s="237">
+      <c r="U22" s="215">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="V22" s="237" t="e">
+      <c r="V22" s="215" t="e">
         <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="W22" s="70"/>
-      <c r="X22" s="237">
+      <c r="X22" s="215">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="Y22" s="237"/>
+      <c r="Y22" s="215"/>
       <c r="Z22" s="70"/>
-      <c r="AA22" s="237">
+      <c r="AA22" s="215">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="AB22" s="237"/>
+      <c r="AB22" s="215"/>
       <c r="AC22" s="69"/>
       <c r="AD22" s="71">
         <f t="shared" si="4"/>
@@ -4773,20 +4744,20 @@
     </row>
     <row r="23" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A23" s="2"/>
-      <c r="B23" s="233"/>
-      <c r="C23" s="233"/>
-      <c r="D23" s="233"/>
-      <c r="E23" s="233"/>
+      <c r="B23" s="212"/>
+      <c r="C23" s="212"/>
+      <c r="D23" s="212"/>
+      <c r="E23" s="212"/>
       <c r="F23" s="58"/>
-      <c r="G23" s="234"/>
-      <c r="H23" s="234"/>
-      <c r="I23" s="234"/>
+      <c r="G23" s="213"/>
+      <c r="H23" s="213"/>
+      <c r="I23" s="213"/>
       <c r="J23" s="75"/>
       <c r="K23" s="60"/>
       <c r="L23" s="70"/>
-      <c r="M23" s="235"/>
-      <c r="N23" s="235"/>
-      <c r="O23" s="235"/>
+      <c r="M23" s="214"/>
+      <c r="N23" s="214"/>
+      <c r="O23" s="214"/>
       <c r="P23" s="70"/>
       <c r="Q23" s="71">
         <f t="shared" si="0"/>
@@ -4798,26 +4769,26 @@
         <v>0</v>
       </c>
       <c r="T23" s="75"/>
-      <c r="U23" s="237">
+      <c r="U23" s="215">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="V23" s="237" t="e">
+      <c r="V23" s="215" t="e">
         <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="W23" s="75"/>
-      <c r="X23" s="237">
+      <c r="X23" s="215">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="Y23" s="237"/>
+      <c r="Y23" s="215"/>
       <c r="Z23" s="75"/>
-      <c r="AA23" s="237">
+      <c r="AA23" s="215">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="AB23" s="237"/>
+      <c r="AB23" s="215"/>
       <c r="AC23" s="76"/>
       <c r="AD23" s="71">
         <f t="shared" si="4"/>
@@ -4835,20 +4806,20 @@
     </row>
     <row r="24" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A24" s="2"/>
-      <c r="B24" s="233"/>
-      <c r="C24" s="233"/>
-      <c r="D24" s="233"/>
-      <c r="E24" s="233"/>
+      <c r="B24" s="212"/>
+      <c r="C24" s="212"/>
+      <c r="D24" s="212"/>
+      <c r="E24" s="212"/>
       <c r="F24" s="58"/>
-      <c r="G24" s="234"/>
-      <c r="H24" s="234"/>
-      <c r="I24" s="234"/>
+      <c r="G24" s="213"/>
+      <c r="H24" s="213"/>
+      <c r="I24" s="213"/>
       <c r="J24" s="75"/>
       <c r="K24" s="60"/>
       <c r="L24" s="70"/>
-      <c r="M24" s="235"/>
-      <c r="N24" s="235"/>
-      <c r="O24" s="235"/>
+      <c r="M24" s="214"/>
+      <c r="N24" s="214"/>
+      <c r="O24" s="214"/>
       <c r="P24" s="70"/>
       <c r="Q24" s="71">
         <f t="shared" si="0"/>
@@ -4860,26 +4831,26 @@
         <v>0</v>
       </c>
       <c r="T24" s="75"/>
-      <c r="U24" s="237">
+      <c r="U24" s="215">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="V24" s="237" t="e">
+      <c r="V24" s="215" t="e">
         <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="W24" s="75"/>
-      <c r="X24" s="237">
+      <c r="X24" s="215">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="Y24" s="237"/>
+      <c r="Y24" s="215"/>
       <c r="Z24" s="75"/>
-      <c r="AA24" s="237">
+      <c r="AA24" s="215">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="AB24" s="237"/>
+      <c r="AB24" s="215"/>
       <c r="AC24" s="76"/>
       <c r="AD24" s="71">
         <f t="shared" si="4"/>
@@ -4897,20 +4868,20 @@
     </row>
     <row r="25" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A25" s="2"/>
-      <c r="B25" s="233"/>
-      <c r="C25" s="233"/>
-      <c r="D25" s="233"/>
-      <c r="E25" s="233"/>
+      <c r="B25" s="212"/>
+      <c r="C25" s="212"/>
+      <c r="D25" s="212"/>
+      <c r="E25" s="212"/>
       <c r="F25" s="58"/>
-      <c r="G25" s="234"/>
-      <c r="H25" s="234"/>
-      <c r="I25" s="234"/>
+      <c r="G25" s="213"/>
+      <c r="H25" s="213"/>
+      <c r="I25" s="213"/>
       <c r="J25" s="75"/>
       <c r="K25" s="60"/>
       <c r="L25" s="70"/>
-      <c r="M25" s="235"/>
-      <c r="N25" s="235"/>
-      <c r="O25" s="235"/>
+      <c r="M25" s="214"/>
+      <c r="N25" s="214"/>
+      <c r="O25" s="214"/>
       <c r="P25" s="70"/>
       <c r="Q25" s="71">
         <f t="shared" si="0"/>
@@ -4922,26 +4893,26 @@
         <v>0</v>
       </c>
       <c r="T25" s="75"/>
-      <c r="U25" s="237">
+      <c r="U25" s="215">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="V25" s="237" t="e">
+      <c r="V25" s="215" t="e">
         <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="W25" s="75"/>
-      <c r="X25" s="237">
+      <c r="X25" s="215">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="Y25" s="237"/>
+      <c r="Y25" s="215"/>
       <c r="Z25" s="75"/>
-      <c r="AA25" s="237">
+      <c r="AA25" s="215">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="AB25" s="237"/>
+      <c r="AB25" s="215"/>
       <c r="AC25" s="76"/>
       <c r="AD25" s="71">
         <f t="shared" si="4"/>
@@ -4959,20 +4930,20 @@
     </row>
     <row r="26" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A26" s="2"/>
-      <c r="B26" s="233"/>
-      <c r="C26" s="233"/>
-      <c r="D26" s="233"/>
-      <c r="E26" s="233"/>
+      <c r="B26" s="212"/>
+      <c r="C26" s="212"/>
+      <c r="D26" s="212"/>
+      <c r="E26" s="212"/>
       <c r="F26" s="58"/>
-      <c r="G26" s="234"/>
-      <c r="H26" s="234"/>
-      <c r="I26" s="234"/>
+      <c r="G26" s="213"/>
+      <c r="H26" s="213"/>
+      <c r="I26" s="213"/>
       <c r="J26" s="75"/>
       <c r="K26" s="60"/>
       <c r="L26" s="70"/>
-      <c r="M26" s="235"/>
-      <c r="N26" s="235"/>
-      <c r="O26" s="235"/>
+      <c r="M26" s="214"/>
+      <c r="N26" s="214"/>
+      <c r="O26" s="214"/>
       <c r="P26" s="70"/>
       <c r="Q26" s="71">
         <f t="shared" si="0"/>
@@ -4984,26 +4955,26 @@
         <v>0</v>
       </c>
       <c r="T26" s="75"/>
-      <c r="U26" s="237">
+      <c r="U26" s="215">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="V26" s="237" t="e">
+      <c r="V26" s="215" t="e">
         <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="W26" s="75"/>
-      <c r="X26" s="237">
+      <c r="X26" s="215">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="Y26" s="237"/>
+      <c r="Y26" s="215"/>
       <c r="Z26" s="75"/>
-      <c r="AA26" s="237">
+      <c r="AA26" s="215">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="AB26" s="237"/>
+      <c r="AB26" s="215"/>
       <c r="AC26" s="76"/>
       <c r="AD26" s="71">
         <f t="shared" si="4"/>
@@ -5021,20 +4992,20 @@
     </row>
     <row r="27" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A27" s="2"/>
-      <c r="B27" s="233"/>
-      <c r="C27" s="233"/>
-      <c r="D27" s="233"/>
-      <c r="E27" s="233"/>
+      <c r="B27" s="212"/>
+      <c r="C27" s="212"/>
+      <c r="D27" s="212"/>
+      <c r="E27" s="212"/>
       <c r="F27" s="58"/>
-      <c r="G27" s="234"/>
-      <c r="H27" s="234"/>
-      <c r="I27" s="234"/>
+      <c r="G27" s="213"/>
+      <c r="H27" s="213"/>
+      <c r="I27" s="213"/>
       <c r="J27" s="75"/>
       <c r="K27" s="60"/>
       <c r="L27" s="70"/>
-      <c r="M27" s="235"/>
-      <c r="N27" s="235"/>
-      <c r="O27" s="235"/>
+      <c r="M27" s="214"/>
+      <c r="N27" s="214"/>
+      <c r="O27" s="214"/>
       <c r="P27" s="70"/>
       <c r="Q27" s="80">
         <f t="shared" si="0"/>
@@ -5046,26 +5017,26 @@
         <v>0</v>
       </c>
       <c r="T27" s="81"/>
-      <c r="U27" s="236">
+      <c r="U27" s="223">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="V27" s="236" t="e">
+      <c r="V27" s="223" t="e">
         <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
       <c r="W27" s="81"/>
-      <c r="X27" s="236">
+      <c r="X27" s="223">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="Y27" s="236"/>
+      <c r="Y27" s="223"/>
       <c r="Z27" s="81"/>
-      <c r="AA27" s="236">
+      <c r="AA27" s="223">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="AB27" s="236"/>
+      <c r="AB27" s="223"/>
       <c r="AC27" s="82"/>
       <c r="AD27" s="80">
         <f t="shared" si="4"/>
@@ -5083,51 +5054,47 @@
     </row>
     <row r="28" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A28" s="2"/>
-      <c r="B28" s="224" t="s">
+      <c r="B28" s="239" t="s">
         <v>39</v>
       </c>
-      <c r="C28" s="224"/>
-      <c r="D28" s="224"/>
-      <c r="E28" s="224"/>
-      <c r="F28" s="224"/>
-      <c r="G28" s="224"/>
-      <c r="H28" s="225" t="s">
+      <c r="C28" s="239"/>
+      <c r="D28" s="239"/>
+      <c r="E28" s="239"/>
+      <c r="F28" s="239"/>
+      <c r="G28" s="239"/>
+      <c r="H28" s="240" t="s">
         <v>40</v>
       </c>
-      <c r="I28" s="225"/>
-      <c r="J28" s="226" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="K28" s="226"/>
-      <c r="L28" s="226"/>
-      <c r="M28" s="225" t="s">
+      <c r="I28" s="240"/>
+      <c r="J28" s="241" t="s">
+        <v>177</v>
+      </c>
+      <c r="K28" s="241"/>
+      <c r="L28" s="241"/>
+      <c r="M28" s="240" t="s">
         <v>41</v>
       </c>
-      <c r="N28" s="225"/>
-      <c r="O28" s="225"/>
-      <c r="P28" s="225"/>
-      <c r="Q28" s="225"/>
-      <c r="R28" s="225"/>
-      <c r="S28" s="225"/>
-      <c r="T28" s="227" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="U28" s="227"/>
-      <c r="V28" s="227"/>
-      <c r="W28" s="227"/>
-      <c r="X28" s="227"/>
-      <c r="Y28" s="227"/>
-      <c r="Z28" s="227"/>
-      <c r="AA28" s="228" t="s">
+      <c r="N28" s="240"/>
+      <c r="O28" s="240"/>
+      <c r="P28" s="240"/>
+      <c r="Q28" s="240"/>
+      <c r="R28" s="240"/>
+      <c r="S28" s="240"/>
+      <c r="T28" s="242" t="s">
+        <v>176</v>
+      </c>
+      <c r="U28" s="242"/>
+      <c r="V28" s="242"/>
+      <c r="W28" s="242"/>
+      <c r="X28" s="242"/>
+      <c r="Y28" s="242"/>
+      <c r="Z28" s="242"/>
+      <c r="AA28" s="243" t="s">
         <v>42</v>
       </c>
-      <c r="AB28" s="228"/>
-      <c r="AC28" s="228"/>
-      <c r="AD28" s="228"/>
+      <c r="AB28" s="243"/>
+      <c r="AC28" s="243"/>
+      <c r="AD28" s="243"/>
       <c r="AE28" s="83">
         <f>IF(AH29&gt;N10,-N10+AH29,0)</f>
         <v>0</v>
@@ -5142,84 +5109,84 @@
     </row>
     <row r="29" spans="1:38" ht="13.7" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="2"/>
-      <c r="B29" s="218" t="s">
+      <c r="B29" s="233" t="s">
         <v>44</v>
       </c>
-      <c r="C29" s="218"/>
-      <c r="D29" s="218"/>
-      <c r="E29" s="218"/>
-      <c r="F29" s="218"/>
-      <c r="G29" s="218"/>
-      <c r="H29" s="218"/>
-      <c r="I29" s="218"/>
-      <c r="J29" s="218"/>
-      <c r="K29" s="218"/>
-      <c r="L29" s="218"/>
-      <c r="M29" s="218"/>
-      <c r="N29" s="218"/>
-      <c r="O29" s="218"/>
-      <c r="P29" s="218"/>
-      <c r="Q29" s="218"/>
-      <c r="R29" s="218"/>
-      <c r="S29" s="218"/>
-      <c r="T29" s="218"/>
-      <c r="U29" s="219" t="s">
+      <c r="C29" s="233"/>
+      <c r="D29" s="233"/>
+      <c r="E29" s="233"/>
+      <c r="F29" s="233"/>
+      <c r="G29" s="233"/>
+      <c r="H29" s="233"/>
+      <c r="I29" s="233"/>
+      <c r="J29" s="233"/>
+      <c r="K29" s="233"/>
+      <c r="L29" s="233"/>
+      <c r="M29" s="233"/>
+      <c r="N29" s="233"/>
+      <c r="O29" s="233"/>
+      <c r="P29" s="233"/>
+      <c r="Q29" s="233"/>
+      <c r="R29" s="233"/>
+      <c r="S29" s="233"/>
+      <c r="T29" s="233"/>
+      <c r="U29" s="234" t="s">
         <v>45</v>
       </c>
-      <c r="V29" s="219"/>
-      <c r="W29" s="219"/>
-      <c r="X29" s="219"/>
-      <c r="Y29" s="219"/>
-      <c r="Z29" s="219"/>
-      <c r="AA29" s="219"/>
-      <c r="AB29" s="219"/>
-      <c r="AC29" s="219"/>
-      <c r="AD29" s="219"/>
+      <c r="V29" s="234"/>
+      <c r="W29" s="234"/>
+      <c r="X29" s="234"/>
+      <c r="Y29" s="234"/>
+      <c r="Z29" s="234"/>
+      <c r="AA29" s="234"/>
+      <c r="AB29" s="234"/>
+      <c r="AC29" s="234"/>
+      <c r="AD29" s="234"/>
       <c r="AE29" s="84">
         <f>+AH29-AE28</f>
-        <v>53.78</v>
+        <v>17.27</v>
       </c>
       <c r="AF29" s="6"/>
       <c r="AG29" s="6"/>
       <c r="AH29" s="85">
         <f>SUM(AE16:AE27)</f>
-        <v>53.78</v>
+        <v>17.27</v>
       </c>
       <c r="AJ29" s="78"/>
     </row>
     <row r="30" spans="1:38" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="2"/>
-      <c r="B30" s="218"/>
-      <c r="C30" s="218"/>
-      <c r="D30" s="218"/>
-      <c r="E30" s="218"/>
-      <c r="F30" s="218"/>
-      <c r="G30" s="218"/>
-      <c r="H30" s="218"/>
-      <c r="I30" s="218"/>
-      <c r="J30" s="218"/>
-      <c r="K30" s="218"/>
-      <c r="L30" s="218"/>
-      <c r="M30" s="218"/>
-      <c r="N30" s="218"/>
-      <c r="O30" s="218"/>
-      <c r="P30" s="218"/>
-      <c r="Q30" s="218"/>
-      <c r="R30" s="218"/>
-      <c r="S30" s="218"/>
-      <c r="T30" s="218"/>
-      <c r="U30" s="220" t="s">
+      <c r="B30" s="233"/>
+      <c r="C30" s="233"/>
+      <c r="D30" s="233"/>
+      <c r="E30" s="233"/>
+      <c r="F30" s="233"/>
+      <c r="G30" s="233"/>
+      <c r="H30" s="233"/>
+      <c r="I30" s="233"/>
+      <c r="J30" s="233"/>
+      <c r="K30" s="233"/>
+      <c r="L30" s="233"/>
+      <c r="M30" s="233"/>
+      <c r="N30" s="233"/>
+      <c r="O30" s="233"/>
+      <c r="P30" s="233"/>
+      <c r="Q30" s="233"/>
+      <c r="R30" s="233"/>
+      <c r="S30" s="233"/>
+      <c r="T30" s="233"/>
+      <c r="U30" s="235" t="s">
         <v>46</v>
       </c>
-      <c r="V30" s="220"/>
-      <c r="W30" s="220"/>
-      <c r="X30" s="220"/>
-      <c r="Y30" s="220"/>
-      <c r="Z30" s="220"/>
-      <c r="AA30" s="220"/>
-      <c r="AB30" s="220"/>
-      <c r="AC30" s="220"/>
-      <c r="AD30" s="220"/>
+      <c r="V30" s="235"/>
+      <c r="W30" s="235"/>
+      <c r="X30" s="235"/>
+      <c r="Y30" s="235"/>
+      <c r="Z30" s="235"/>
+      <c r="AA30" s="235"/>
+      <c r="AB30" s="235"/>
+      <c r="AC30" s="235"/>
+      <c r="AD30" s="235"/>
       <c r="AE30" s="86"/>
       <c r="AF30" s="6"/>
       <c r="AG30" s="6"/>
@@ -5228,40 +5195,40 @@
     </row>
     <row r="31" spans="1:38" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="2"/>
-      <c r="B31" s="218"/>
-      <c r="C31" s="218"/>
-      <c r="D31" s="218"/>
-      <c r="E31" s="218"/>
-      <c r="F31" s="218"/>
-      <c r="G31" s="218"/>
-      <c r="H31" s="218"/>
-      <c r="I31" s="218"/>
-      <c r="J31" s="218"/>
-      <c r="K31" s="218"/>
-      <c r="L31" s="218"/>
-      <c r="M31" s="218"/>
-      <c r="N31" s="218"/>
-      <c r="O31" s="218"/>
-      <c r="P31" s="218"/>
-      <c r="Q31" s="218"/>
-      <c r="R31" s="218"/>
-      <c r="S31" s="218"/>
-      <c r="T31" s="218"/>
-      <c r="U31" s="221" t="s">
+      <c r="B31" s="233"/>
+      <c r="C31" s="233"/>
+      <c r="D31" s="233"/>
+      <c r="E31" s="233"/>
+      <c r="F31" s="233"/>
+      <c r="G31" s="233"/>
+      <c r="H31" s="233"/>
+      <c r="I31" s="233"/>
+      <c r="J31" s="233"/>
+      <c r="K31" s="233"/>
+      <c r="L31" s="233"/>
+      <c r="M31" s="233"/>
+      <c r="N31" s="233"/>
+      <c r="O31" s="233"/>
+      <c r="P31" s="233"/>
+      <c r="Q31" s="233"/>
+      <c r="R31" s="233"/>
+      <c r="S31" s="233"/>
+      <c r="T31" s="233"/>
+      <c r="U31" s="236" t="s">
         <v>47</v>
       </c>
-      <c r="V31" s="221"/>
-      <c r="W31" s="221"/>
-      <c r="X31" s="221"/>
-      <c r="Y31" s="221"/>
-      <c r="Z31" s="221"/>
-      <c r="AA31" s="221"/>
-      <c r="AB31" s="221"/>
-      <c r="AC31" s="221"/>
-      <c r="AD31" s="221"/>
+      <c r="V31" s="236"/>
+      <c r="W31" s="236"/>
+      <c r="X31" s="236"/>
+      <c r="Y31" s="236"/>
+      <c r="Z31" s="236"/>
+      <c r="AA31" s="236"/>
+      <c r="AB31" s="236"/>
+      <c r="AC31" s="236"/>
+      <c r="AD31" s="236"/>
       <c r="AE31" s="87">
         <f>+AE29-AE30</f>
-        <v>53.78</v>
+        <v>17.27</v>
       </c>
       <c r="AF31" s="6"/>
       <c r="AG31" s="6"/>
@@ -5307,156 +5274,154 @@
     </row>
     <row r="33" spans="1:32" ht="9.9499999999999993" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2"/>
-      <c r="B33" s="222" t="s">
+      <c r="B33" s="237" t="s">
         <v>48</v>
       </c>
-      <c r="C33" s="222"/>
-      <c r="D33" s="222"/>
-      <c r="E33" s="222"/>
-      <c r="F33" s="222"/>
-      <c r="G33" s="222"/>
-      <c r="H33" s="222"/>
-      <c r="I33" s="222"/>
-      <c r="J33" s="222"/>
-      <c r="K33" s="222"/>
-      <c r="L33" s="222"/>
-      <c r="M33" s="222"/>
-      <c r="N33" s="222"/>
-      <c r="O33" s="222"/>
-      <c r="P33" s="222"/>
-      <c r="Q33" s="222"/>
+      <c r="C33" s="237"/>
+      <c r="D33" s="237"/>
+      <c r="E33" s="237"/>
+      <c r="F33" s="237"/>
+      <c r="G33" s="237"/>
+      <c r="H33" s="237"/>
+      <c r="I33" s="237"/>
+      <c r="J33" s="237"/>
+      <c r="K33" s="237"/>
+      <c r="L33" s="237"/>
+      <c r="M33" s="237"/>
+      <c r="N33" s="237"/>
+      <c r="O33" s="237"/>
+      <c r="P33" s="237"/>
+      <c r="Q33" s="237"/>
       <c r="R33" s="91"/>
-      <c r="S33" s="223" t="s">
+      <c r="S33" s="238" t="s">
         <v>49</v>
       </c>
-      <c r="T33" s="223"/>
-      <c r="U33" s="223"/>
-      <c r="V33" s="223"/>
-      <c r="W33" s="223"/>
-      <c r="X33" s="223"/>
-      <c r="Y33" s="223"/>
-      <c r="Z33" s="223"/>
-      <c r="AA33" s="223"/>
-      <c r="AB33" s="223"/>
-      <c r="AC33" s="223"/>
-      <c r="AD33" s="223"/>
-      <c r="AE33" s="223"/>
+      <c r="T33" s="238"/>
+      <c r="U33" s="238"/>
+      <c r="V33" s="238"/>
+      <c r="W33" s="238"/>
+      <c r="X33" s="238"/>
+      <c r="Y33" s="238"/>
+      <c r="Z33" s="238"/>
+      <c r="AA33" s="238"/>
+      <c r="AB33" s="238"/>
+      <c r="AC33" s="238"/>
+      <c r="AD33" s="238"/>
+      <c r="AE33" s="238"/>
       <c r="AF33" s="6"/>
     </row>
     <row r="34" spans="1:32" ht="12.6" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A34" s="2"/>
-      <c r="B34" s="209" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="C34" s="210"/>
-      <c r="D34" s="210"/>
-      <c r="E34" s="210"/>
-      <c r="F34" s="210"/>
-      <c r="G34" s="210"/>
-      <c r="H34" s="210"/>
-      <c r="I34" s="210"/>
-      <c r="J34" s="210"/>
-      <c r="K34" s="210"/>
-      <c r="L34" s="210"/>
-      <c r="M34" s="210"/>
-      <c r="N34" s="210"/>
-      <c r="O34" s="210"/>
-      <c r="P34" s="210"/>
-      <c r="Q34" s="211"/>
+      <c r="B34" s="224" t="s">
+        <v>167</v>
+      </c>
+      <c r="C34" s="225"/>
+      <c r="D34" s="225"/>
+      <c r="E34" s="225"/>
+      <c r="F34" s="225"/>
+      <c r="G34" s="225"/>
+      <c r="H34" s="225"/>
+      <c r="I34" s="225"/>
+      <c r="J34" s="225"/>
+      <c r="K34" s="225"/>
+      <c r="L34" s="225"/>
+      <c r="M34" s="225"/>
+      <c r="N34" s="225"/>
+      <c r="O34" s="225"/>
+      <c r="P34" s="225"/>
+      <c r="Q34" s="226"/>
       <c r="R34" s="92"/>
-      <c r="S34" s="223"/>
-      <c r="T34" s="223"/>
-      <c r="U34" s="223"/>
-      <c r="V34" s="223"/>
-      <c r="W34" s="223"/>
-      <c r="X34" s="223"/>
-      <c r="Y34" s="223"/>
-      <c r="Z34" s="223"/>
-      <c r="AA34" s="223"/>
-      <c r="AB34" s="223"/>
-      <c r="AC34" s="223"/>
-      <c r="AD34" s="223"/>
-      <c r="AE34" s="223"/>
+      <c r="S34" s="238"/>
+      <c r="T34" s="238"/>
+      <c r="U34" s="238"/>
+      <c r="V34" s="238"/>
+      <c r="W34" s="238"/>
+      <c r="X34" s="238"/>
+      <c r="Y34" s="238"/>
+      <c r="Z34" s="238"/>
+      <c r="AA34" s="238"/>
+      <c r="AB34" s="238"/>
+      <c r="AC34" s="238"/>
+      <c r="AD34" s="238"/>
+      <c r="AE34" s="238"/>
       <c r="AF34" s="6"/>
     </row>
     <row r="35" spans="1:32" ht="12.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="2"/>
-      <c r="B35" s="212"/>
-      <c r="C35" s="213"/>
-      <c r="D35" s="213"/>
-      <c r="E35" s="213"/>
-      <c r="F35" s="213"/>
-      <c r="G35" s="213"/>
-      <c r="H35" s="213"/>
-      <c r="I35" s="213"/>
-      <c r="J35" s="213"/>
-      <c r="K35" s="213"/>
-      <c r="L35" s="213"/>
-      <c r="M35" s="213"/>
-      <c r="N35" s="213"/>
-      <c r="O35" s="213"/>
-      <c r="P35" s="213"/>
-      <c r="Q35" s="214"/>
+      <c r="B35" s="227"/>
+      <c r="C35" s="228"/>
+      <c r="D35" s="228"/>
+      <c r="E35" s="228"/>
+      <c r="F35" s="228"/>
+      <c r="G35" s="228"/>
+      <c r="H35" s="228"/>
+      <c r="I35" s="228"/>
+      <c r="J35" s="228"/>
+      <c r="K35" s="228"/>
+      <c r="L35" s="228"/>
+      <c r="M35" s="228"/>
+      <c r="N35" s="228"/>
+      <c r="O35" s="228"/>
+      <c r="P35" s="228"/>
+      <c r="Q35" s="229"/>
       <c r="R35" s="93"/>
-      <c r="S35" s="232" t="s">
+      <c r="S35" s="249" t="s">
         <v>21</v>
       </c>
-      <c r="T35" s="230" t="s">
+      <c r="T35" s="245" t="s">
         <v>51</v>
       </c>
-      <c r="U35" s="230"/>
-      <c r="V35" s="230"/>
-      <c r="W35" s="230"/>
-      <c r="X35" s="207" t="s">
+      <c r="U35" s="245"/>
+      <c r="V35" s="245"/>
+      <c r="W35" s="245"/>
+      <c r="X35" s="250" t="s">
         <v>29</v>
       </c>
-      <c r="Y35" s="207"/>
-      <c r="Z35" s="207" t="s">
+      <c r="Y35" s="250"/>
+      <c r="Z35" s="250" t="s">
         <v>30</v>
       </c>
-      <c r="AA35" s="207"/>
-      <c r="AB35" s="207"/>
-      <c r="AC35" s="207" t="s">
+      <c r="AA35" s="250"/>
+      <c r="AB35" s="250"/>
+      <c r="AC35" s="250" t="s">
         <v>31</v>
       </c>
-      <c r="AD35" s="207"/>
-      <c r="AE35" s="229" t="s">
+      <c r="AD35" s="250"/>
+      <c r="AE35" s="244" t="s">
         <v>32</v>
       </c>
       <c r="AF35" s="6"/>
     </row>
     <row r="36" spans="1:32" ht="12.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="2"/>
-      <c r="B36" s="212"/>
-      <c r="C36" s="213"/>
-      <c r="D36" s="213"/>
-      <c r="E36" s="213"/>
-      <c r="F36" s="213"/>
-      <c r="G36" s="213"/>
-      <c r="H36" s="213"/>
-      <c r="I36" s="213"/>
-      <c r="J36" s="213"/>
-      <c r="K36" s="213"/>
-      <c r="L36" s="213"/>
-      <c r="M36" s="213"/>
-      <c r="N36" s="213"/>
-      <c r="O36" s="213"/>
-      <c r="P36" s="213"/>
-      <c r="Q36" s="214"/>
+      <c r="B36" s="227"/>
+      <c r="C36" s="228"/>
+      <c r="D36" s="228"/>
+      <c r="E36" s="228"/>
+      <c r="F36" s="228"/>
+      <c r="G36" s="228"/>
+      <c r="H36" s="228"/>
+      <c r="I36" s="228"/>
+      <c r="J36" s="228"/>
+      <c r="K36" s="228"/>
+      <c r="L36" s="228"/>
+      <c r="M36" s="228"/>
+      <c r="N36" s="228"/>
+      <c r="O36" s="228"/>
+      <c r="P36" s="228"/>
+      <c r="Q36" s="229"/>
       <c r="R36" s="93"/>
-      <c r="S36" s="232"/>
-      <c r="T36" s="230"/>
-      <c r="U36" s="230"/>
-      <c r="V36" s="230"/>
-      <c r="W36" s="230"/>
-      <c r="X36" s="207"/>
-      <c r="Y36" s="207"/>
-      <c r="Z36" s="230" t="s">
+      <c r="S36" s="249"/>
+      <c r="T36" s="245"/>
+      <c r="U36" s="245"/>
+      <c r="V36" s="245"/>
+      <c r="W36" s="245"/>
+      <c r="X36" s="250"/>
+      <c r="Y36" s="250"/>
+      <c r="Z36" s="245" t="s">
         <v>52</v>
       </c>
-      <c r="AA36" s="230"/>
+      <c r="AA36" s="245"/>
       <c r="AB36" s="94" t="s">
         <v>53</v>
       </c>
@@ -5466,95 +5431,95 @@
       <c r="AD36" s="94" t="s">
         <v>55</v>
       </c>
-      <c r="AE36" s="229"/>
+      <c r="AE36" s="244"/>
     </row>
     <row r="37" spans="1:32" ht="12.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="2"/>
-      <c r="B37" s="212"/>
-      <c r="C37" s="213"/>
-      <c r="D37" s="213"/>
-      <c r="E37" s="213"/>
-      <c r="F37" s="213"/>
-      <c r="G37" s="213"/>
-      <c r="H37" s="213"/>
-      <c r="I37" s="213"/>
-      <c r="J37" s="213"/>
-      <c r="K37" s="213"/>
-      <c r="L37" s="213"/>
-      <c r="M37" s="213"/>
-      <c r="N37" s="213"/>
-      <c r="O37" s="213"/>
-      <c r="P37" s="213"/>
-      <c r="Q37" s="214"/>
+      <c r="B37" s="227"/>
+      <c r="C37" s="228"/>
+      <c r="D37" s="228"/>
+      <c r="E37" s="228"/>
+      <c r="F37" s="228"/>
+      <c r="G37" s="228"/>
+      <c r="H37" s="228"/>
+      <c r="I37" s="228"/>
+      <c r="J37" s="228"/>
+      <c r="K37" s="228"/>
+      <c r="L37" s="228"/>
+      <c r="M37" s="228"/>
+      <c r="N37" s="228"/>
+      <c r="O37" s="228"/>
+      <c r="P37" s="228"/>
+      <c r="Q37" s="229"/>
       <c r="R37" s="93"/>
-      <c r="S37" s="231">
+      <c r="S37" s="246">
         <v>1</v>
       </c>
-      <c r="T37" s="206" t="s">
+      <c r="T37" s="247" t="s">
         <v>56</v>
       </c>
-      <c r="U37" s="206"/>
-      <c r="V37" s="206"/>
-      <c r="W37" s="206"/>
-      <c r="X37" s="196">
+      <c r="U37" s="247"/>
+      <c r="V37" s="247"/>
+      <c r="W37" s="247"/>
+      <c r="X37" s="248">
         <f>+AM107</f>
-        <v>537.88</v>
-      </c>
-      <c r="Y37" s="196"/>
-      <c r="Z37" s="196">
+        <v>172.76</v>
+      </c>
+      <c r="Y37" s="248"/>
+      <c r="Z37" s="248">
         <f>+AR107</f>
-        <v>107.57</v>
-      </c>
-      <c r="AA37" s="196"/>
-      <c r="AB37" s="196">
+        <v>34.549999999999997</v>
+      </c>
+      <c r="AA37" s="248"/>
+      <c r="AB37" s="248">
         <f>+AT107</f>
-        <v>215.15</v>
-      </c>
-      <c r="AC37" s="196">
+        <v>69.099999999999994</v>
+      </c>
+      <c r="AC37" s="248">
         <f>+AV107</f>
-        <v>107.57</v>
-      </c>
-      <c r="AD37" s="196">
+        <v>34.549999999999997</v>
+      </c>
+      <c r="AD37" s="248">
         <f>+AX107</f>
-        <v>215.15</v>
-      </c>
-      <c r="AE37" s="197">
+        <v>69.099999999999994</v>
+      </c>
+      <c r="AE37" s="251">
         <f>+AZ107</f>
-        <v>268.94</v>
+        <v>86.38</v>
       </c>
     </row>
     <row r="38" spans="1:32" ht="12.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2"/>
-      <c r="B38" s="215"/>
-      <c r="C38" s="216"/>
-      <c r="D38" s="216"/>
-      <c r="E38" s="216"/>
-      <c r="F38" s="216"/>
-      <c r="G38" s="216"/>
-      <c r="H38" s="216"/>
-      <c r="I38" s="216"/>
-      <c r="J38" s="216"/>
-      <c r="K38" s="216"/>
-      <c r="L38" s="216"/>
-      <c r="M38" s="216"/>
-      <c r="N38" s="216"/>
-      <c r="O38" s="216"/>
-      <c r="P38" s="216"/>
-      <c r="Q38" s="217"/>
+      <c r="B38" s="230"/>
+      <c r="C38" s="231"/>
+      <c r="D38" s="231"/>
+      <c r="E38" s="231"/>
+      <c r="F38" s="231"/>
+      <c r="G38" s="231"/>
+      <c r="H38" s="231"/>
+      <c r="I38" s="231"/>
+      <c r="J38" s="231"/>
+      <c r="K38" s="231"/>
+      <c r="L38" s="231"/>
+      <c r="M38" s="231"/>
+      <c r="N38" s="231"/>
+      <c r="O38" s="231"/>
+      <c r="P38" s="231"/>
+      <c r="Q38" s="232"/>
       <c r="R38" s="93"/>
-      <c r="S38" s="231"/>
-      <c r="T38" s="206"/>
-      <c r="U38" s="206"/>
-      <c r="V38" s="206"/>
-      <c r="W38" s="206"/>
-      <c r="X38" s="196"/>
-      <c r="Y38" s="196"/>
-      <c r="Z38" s="196"/>
-      <c r="AA38" s="196"/>
-      <c r="AB38" s="196"/>
-      <c r="AC38" s="196"/>
-      <c r="AD38" s="196"/>
-      <c r="AE38" s="197"/>
+      <c r="S38" s="246"/>
+      <c r="T38" s="247"/>
+      <c r="U38" s="247"/>
+      <c r="V38" s="247"/>
+      <c r="W38" s="247"/>
+      <c r="X38" s="248"/>
+      <c r="Y38" s="248"/>
+      <c r="Z38" s="248"/>
+      <c r="AA38" s="248"/>
+      <c r="AB38" s="248"/>
+      <c r="AC38" s="248"/>
+      <c r="AD38" s="248"/>
+      <c r="AE38" s="251"/>
     </row>
     <row r="39" spans="1:32" ht="7.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2"/>
@@ -5575,19 +5540,19 @@
       <c r="P39" s="95"/>
       <c r="Q39" s="95"/>
       <c r="R39" s="96"/>
-      <c r="S39" s="231"/>
-      <c r="T39" s="206"/>
-      <c r="U39" s="206"/>
-      <c r="V39" s="206"/>
-      <c r="W39" s="206"/>
-      <c r="X39" s="196"/>
-      <c r="Y39" s="196"/>
-      <c r="Z39" s="196"/>
-      <c r="AA39" s="196"/>
-      <c r="AB39" s="196"/>
-      <c r="AC39" s="196"/>
-      <c r="AD39" s="196"/>
-      <c r="AE39" s="197"/>
+      <c r="S39" s="246"/>
+      <c r="T39" s="247"/>
+      <c r="U39" s="247"/>
+      <c r="V39" s="247"/>
+      <c r="W39" s="247"/>
+      <c r="X39" s="248"/>
+      <c r="Y39" s="248"/>
+      <c r="Z39" s="248"/>
+      <c r="AA39" s="248"/>
+      <c r="AB39" s="248"/>
+      <c r="AC39" s="248"/>
+      <c r="AD39" s="248"/>
+      <c r="AE39" s="251"/>
     </row>
     <row r="40" spans="1:32" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="2"/>
@@ -5614,40 +5579,40 @@
       <c r="P40" s="103"/>
       <c r="Q40" s="104"/>
       <c r="R40" s="7"/>
-      <c r="S40" s="202">
+      <c r="S40" s="252">
         <v>2</v>
       </c>
-      <c r="T40" s="208" t="s">
+      <c r="T40" s="253" t="s">
         <v>60</v>
       </c>
-      <c r="U40" s="208"/>
-      <c r="V40" s="208"/>
-      <c r="W40" s="208"/>
-      <c r="X40" s="196">
+      <c r="U40" s="253"/>
+      <c r="V40" s="253"/>
+      <c r="W40" s="253"/>
+      <c r="X40" s="248">
         <f>+AM108</f>
-        <v>484.09</v>
-      </c>
-      <c r="Y40" s="196"/>
-      <c r="Z40" s="196">
+        <v>155.47999999999999</v>
+      </c>
+      <c r="Y40" s="248"/>
+      <c r="Z40" s="248">
         <f>+AR108</f>
-        <v>96.81</v>
-      </c>
-      <c r="AA40" s="196"/>
-      <c r="AB40" s="196">
+        <v>31.09</v>
+      </c>
+      <c r="AA40" s="248"/>
+      <c r="AB40" s="248">
         <f>+AT108</f>
-        <v>193.63</v>
-      </c>
-      <c r="AC40" s="196">
+        <v>62.19</v>
+      </c>
+      <c r="AC40" s="248">
         <f>+AV108</f>
-        <v>96.81</v>
-      </c>
-      <c r="AD40" s="196">
+        <v>31.09</v>
+      </c>
+      <c r="AD40" s="248">
         <f>+AX108</f>
-        <v>193.63</v>
-      </c>
-      <c r="AE40" s="197">
+        <v>62.19</v>
+      </c>
+      <c r="AE40" s="251">
         <f>+AZ108</f>
-        <v>242.04</v>
+        <v>77.739999999999995</v>
       </c>
     </row>
     <row r="41" spans="1:32" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -5669,28 +5634,28 @@
       <c r="J41" s="111"/>
       <c r="K41" s="112"/>
       <c r="L41" s="113"/>
-      <c r="M41" s="204">
+      <c r="M41" s="258">
         <f>AE29</f>
-        <v>53.78</v>
-      </c>
-      <c r="N41" s="204"/>
-      <c r="O41" s="204"/>
-      <c r="P41" s="204"/>
-      <c r="Q41" s="204"/>
+        <v>17.27</v>
+      </c>
+      <c r="N41" s="258"/>
+      <c r="O41" s="258"/>
+      <c r="P41" s="258"/>
+      <c r="Q41" s="258"/>
       <c r="R41" s="7"/>
-      <c r="S41" s="202"/>
-      <c r="T41" s="208"/>
-      <c r="U41" s="208"/>
-      <c r="V41" s="208"/>
-      <c r="W41" s="208"/>
-      <c r="X41" s="196"/>
-      <c r="Y41" s="196"/>
-      <c r="Z41" s="196"/>
-      <c r="AA41" s="196"/>
-      <c r="AB41" s="196"/>
-      <c r="AC41" s="196"/>
-      <c r="AD41" s="196"/>
-      <c r="AE41" s="197"/>
+      <c r="S41" s="252"/>
+      <c r="T41" s="253"/>
+      <c r="U41" s="253"/>
+      <c r="V41" s="253"/>
+      <c r="W41" s="253"/>
+      <c r="X41" s="248"/>
+      <c r="Y41" s="248"/>
+      <c r="Z41" s="248"/>
+      <c r="AA41" s="248"/>
+      <c r="AB41" s="248"/>
+      <c r="AC41" s="248"/>
+      <c r="AD41" s="248"/>
+      <c r="AE41" s="251"/>
     </row>
     <row r="42" spans="1:32" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="2"/>
@@ -5703,32 +5668,32 @@
       <c r="F42" s="108"/>
       <c r="G42" s="109"/>
       <c r="H42" s="109"/>
-      <c r="I42" s="205" t="str">
+      <c r="I42" s="259" t="str">
         <f ca="1">AO77</f>
-        <v>*** CINQÜENTA E TRÊS REAIS  E SETENTA E OITO CENTAVOS ***</v>
-      </c>
-      <c r="J42" s="205"/>
-      <c r="K42" s="205"/>
-      <c r="L42" s="205"/>
-      <c r="M42" s="205"/>
-      <c r="N42" s="205"/>
-      <c r="O42" s="205"/>
-      <c r="P42" s="205"/>
-      <c r="Q42" s="205"/>
+        <v>*** DEZESSETE REAIS  E VINTE E SETE CENTAVOS ***</v>
+      </c>
+      <c r="J42" s="259"/>
+      <c r="K42" s="259"/>
+      <c r="L42" s="259"/>
+      <c r="M42" s="259"/>
+      <c r="N42" s="259"/>
+      <c r="O42" s="259"/>
+      <c r="P42" s="259"/>
+      <c r="Q42" s="259"/>
       <c r="R42" s="7"/>
-      <c r="S42" s="202"/>
-      <c r="T42" s="208"/>
-      <c r="U42" s="208"/>
-      <c r="V42" s="208"/>
-      <c r="W42" s="208"/>
-      <c r="X42" s="196"/>
-      <c r="Y42" s="196"/>
-      <c r="Z42" s="196"/>
-      <c r="AA42" s="196"/>
-      <c r="AB42" s="196"/>
-      <c r="AC42" s="196"/>
-      <c r="AD42" s="196"/>
-      <c r="AE42" s="197"/>
+      <c r="S42" s="252"/>
+      <c r="T42" s="253"/>
+      <c r="U42" s="253"/>
+      <c r="V42" s="253"/>
+      <c r="W42" s="253"/>
+      <c r="X42" s="248"/>
+      <c r="Y42" s="248"/>
+      <c r="Z42" s="248"/>
+      <c r="AA42" s="248"/>
+      <c r="AB42" s="248"/>
+      <c r="AC42" s="248"/>
+      <c r="AD42" s="248"/>
+      <c r="AE42" s="251"/>
     </row>
     <row r="43" spans="1:32" s="20" customFormat="1" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="2"/>
@@ -5741,50 +5706,50 @@
       <c r="F43" s="108"/>
       <c r="G43" s="109"/>
       <c r="H43" s="109"/>
-      <c r="I43" s="205"/>
-      <c r="J43" s="205"/>
-      <c r="K43" s="205"/>
-      <c r="L43" s="205"/>
-      <c r="M43" s="205"/>
-      <c r="N43" s="205"/>
-      <c r="O43" s="205"/>
-      <c r="P43" s="205"/>
-      <c r="Q43" s="205"/>
+      <c r="I43" s="259"/>
+      <c r="J43" s="259"/>
+      <c r="K43" s="259"/>
+      <c r="L43" s="259"/>
+      <c r="M43" s="259"/>
+      <c r="N43" s="259"/>
+      <c r="O43" s="259"/>
+      <c r="P43" s="259"/>
+      <c r="Q43" s="259"/>
       <c r="R43" s="114"/>
-      <c r="S43" s="202">
+      <c r="S43" s="252">
         <v>3</v>
       </c>
-      <c r="T43" s="206" t="s">
+      <c r="T43" s="247" t="s">
         <v>66</v>
       </c>
-      <c r="U43" s="206"/>
-      <c r="V43" s="206"/>
-      <c r="W43" s="206"/>
-      <c r="X43" s="196">
+      <c r="U43" s="247"/>
+      <c r="V43" s="247"/>
+      <c r="W43" s="247"/>
+      <c r="X43" s="248">
         <f>+AM109</f>
-        <v>457.19</v>
-      </c>
-      <c r="Y43" s="196"/>
-      <c r="Z43" s="196">
+        <v>146.84</v>
+      </c>
+      <c r="Y43" s="248"/>
+      <c r="Z43" s="248">
         <f>+AR109</f>
-        <v>91.43</v>
-      </c>
-      <c r="AA43" s="196"/>
-      <c r="AB43" s="196">
+        <v>29.36</v>
+      </c>
+      <c r="AA43" s="248"/>
+      <c r="AB43" s="248">
         <f>+AT109</f>
-        <v>182.87</v>
-      </c>
-      <c r="AC43" s="196">
+        <v>58.73</v>
+      </c>
+      <c r="AC43" s="248">
         <f>+AV109</f>
-        <v>91.43</v>
-      </c>
-      <c r="AD43" s="196">
+        <v>29.36</v>
+      </c>
+      <c r="AD43" s="248">
         <f>+AX109</f>
-        <v>182.87</v>
-      </c>
-      <c r="AE43" s="197">
+        <v>58.73</v>
+      </c>
+      <c r="AE43" s="251">
         <f>+AZ109</f>
-        <v>228.59</v>
+        <v>73.42</v>
       </c>
     </row>
     <row r="44" spans="1:32" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -5796,42 +5761,40 @@
       <c r="F44" s="118"/>
       <c r="G44" s="116"/>
       <c r="H44" s="116"/>
-      <c r="I44" s="205"/>
-      <c r="J44" s="205"/>
-      <c r="K44" s="205"/>
-      <c r="L44" s="205"/>
-      <c r="M44" s="205"/>
-      <c r="N44" s="205"/>
-      <c r="O44" s="205"/>
-      <c r="P44" s="205"/>
-      <c r="Q44" s="205"/>
+      <c r="I44" s="259"/>
+      <c r="J44" s="259"/>
+      <c r="K44" s="259"/>
+      <c r="L44" s="259"/>
+      <c r="M44" s="259"/>
+      <c r="N44" s="259"/>
+      <c r="O44" s="259"/>
+      <c r="P44" s="259"/>
+      <c r="Q44" s="259"/>
       <c r="R44" s="7"/>
-      <c r="S44" s="202"/>
-      <c r="T44" s="206"/>
-      <c r="U44" s="206"/>
-      <c r="V44" s="206"/>
-      <c r="W44" s="206"/>
-      <c r="X44" s="196"/>
-      <c r="Y44" s="196"/>
-      <c r="Z44" s="196"/>
-      <c r="AA44" s="196"/>
-      <c r="AB44" s="196"/>
-      <c r="AC44" s="196"/>
-      <c r="AD44" s="196"/>
-      <c r="AE44" s="197"/>
+      <c r="S44" s="252"/>
+      <c r="T44" s="247"/>
+      <c r="U44" s="247"/>
+      <c r="V44" s="247"/>
+      <c r="W44" s="247"/>
+      <c r="X44" s="248"/>
+      <c r="Y44" s="248"/>
+      <c r="Z44" s="248"/>
+      <c r="AA44" s="248"/>
+      <c r="AB44" s="248"/>
+      <c r="AC44" s="248"/>
+      <c r="AD44" s="248"/>
+      <c r="AE44" s="251"/>
     </row>
     <row r="45" spans="1:32" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="2"/>
       <c r="B45" s="115" t="s">
         <v>67</v>
       </c>
-      <c r="C45" s="199" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="D45" s="199"/>
-      <c r="E45" s="199"/>
+      <c r="C45" s="254">
+        <v>46249</v>
+      </c>
+      <c r="D45" s="254"/>
+      <c r="E45" s="254"/>
       <c r="F45" s="118" t="s">
         <v>68</v>
       </c>
@@ -5847,19 +5810,19 @@
       <c r="P45" s="120"/>
       <c r="Q45" s="121"/>
       <c r="R45" s="7"/>
-      <c r="S45" s="202"/>
-      <c r="T45" s="206"/>
-      <c r="U45" s="206"/>
-      <c r="V45" s="206"/>
-      <c r="W45" s="206"/>
-      <c r="X45" s="196"/>
-      <c r="Y45" s="196"/>
-      <c r="Z45" s="196"/>
-      <c r="AA45" s="196"/>
-      <c r="AB45" s="196"/>
-      <c r="AC45" s="196"/>
-      <c r="AD45" s="196"/>
-      <c r="AE45" s="197"/>
+      <c r="S45" s="252"/>
+      <c r="T45" s="247"/>
+      <c r="U45" s="247"/>
+      <c r="V45" s="247"/>
+      <c r="W45" s="247"/>
+      <c r="X45" s="248"/>
+      <c r="Y45" s="248"/>
+      <c r="Z45" s="248"/>
+      <c r="AA45" s="248"/>
+      <c r="AB45" s="248"/>
+      <c r="AC45" s="248"/>
+      <c r="AD45" s="248"/>
+      <c r="AE45" s="251"/>
     </row>
     <row r="46" spans="1:32" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="2"/>
@@ -5867,19 +5830,19 @@
       <c r="C46" s="109"/>
       <c r="D46" s="109"/>
       <c r="E46" s="123"/>
-      <c r="F46" s="200">
+      <c r="F46" s="255">
         <f>C45</f>
         <v>46249</v>
       </c>
-      <c r="G46" s="200"/>
-      <c r="H46" s="200"/>
-      <c r="I46" s="201">
+      <c r="G46" s="255"/>
+      <c r="H46" s="255"/>
+      <c r="I46" s="256" t="str">
         <f>+AC8</f>
-        <v>46244</v>
-      </c>
-      <c r="J46" s="201"/>
-      <c r="K46" s="201"/>
-      <c r="L46" s="201"/>
+        <v>data protocoloo</v>
+      </c>
+      <c r="J46" s="256"/>
+      <c r="K46" s="256"/>
+      <c r="L46" s="256"/>
       <c r="M46" s="119" t="s">
         <v>70</v>
       </c>
@@ -5887,40 +5850,40 @@
       <c r="P46" s="124"/>
       <c r="Q46" s="125"/>
       <c r="R46" s="7"/>
-      <c r="S46" s="202">
+      <c r="S46" s="252">
         <v>4</v>
       </c>
-      <c r="T46" s="203" t="s">
+      <c r="T46" s="257" t="s">
         <v>71</v>
       </c>
-      <c r="U46" s="203"/>
-      <c r="V46" s="203"/>
-      <c r="W46" s="203"/>
-      <c r="X46" s="196">
+      <c r="U46" s="257"/>
+      <c r="V46" s="257"/>
+      <c r="W46" s="257"/>
+      <c r="X46" s="248">
         <f>+AM110</f>
-        <v>403.41</v>
-      </c>
-      <c r="Y46" s="196"/>
-      <c r="Z46" s="196">
+        <v>129.57</v>
+      </c>
+      <c r="Y46" s="248"/>
+      <c r="Z46" s="248">
         <f>+AR110</f>
-        <v>80.680000000000007</v>
-      </c>
-      <c r="AA46" s="196"/>
-      <c r="AB46" s="196">
+        <v>25.91</v>
+      </c>
+      <c r="AA46" s="248"/>
+      <c r="AB46" s="248">
         <f>+AT110</f>
-        <v>161.36000000000001</v>
-      </c>
-      <c r="AC46" s="196">
+        <v>51.82</v>
+      </c>
+      <c r="AC46" s="248">
         <f>+AV110</f>
-        <v>80.680000000000007</v>
-      </c>
-      <c r="AD46" s="196">
+        <v>25.91</v>
+      </c>
+      <c r="AD46" s="248">
         <f>+AX110</f>
-        <v>161.36000000000001</v>
-      </c>
-      <c r="AE46" s="197">
+        <v>51.82</v>
+      </c>
+      <c r="AE46" s="251">
         <f>+AZ110</f>
-        <v>201.7</v>
+        <v>64.78</v>
       </c>
     </row>
     <row r="47" spans="1:32" s="20" customFormat="1" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -5942,19 +5905,19 @@
       <c r="P47" s="120"/>
       <c r="Q47" s="127"/>
       <c r="R47" s="114"/>
-      <c r="S47" s="202"/>
-      <c r="T47" s="203"/>
-      <c r="U47" s="203"/>
-      <c r="V47" s="203"/>
-      <c r="W47" s="203"/>
-      <c r="X47" s="196"/>
-      <c r="Y47" s="196"/>
-      <c r="Z47" s="196"/>
-      <c r="AA47" s="196"/>
-      <c r="AB47" s="196"/>
-      <c r="AC47" s="196"/>
-      <c r="AD47" s="196"/>
-      <c r="AE47" s="197"/>
+      <c r="S47" s="252"/>
+      <c r="T47" s="257"/>
+      <c r="U47" s="257"/>
+      <c r="V47" s="257"/>
+      <c r="W47" s="257"/>
+      <c r="X47" s="248"/>
+      <c r="Y47" s="248"/>
+      <c r="Z47" s="248"/>
+      <c r="AA47" s="248"/>
+      <c r="AB47" s="248"/>
+      <c r="AC47" s="248"/>
+      <c r="AD47" s="248"/>
+      <c r="AE47" s="251"/>
     </row>
     <row r="48" spans="1:32" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="2"/>
@@ -5969,30 +5932,30 @@
         <v>72</v>
       </c>
       <c r="J48" s="111"/>
-      <c r="K48" s="198">
+      <c r="K48" s="260">
         <f>C45</f>
         <v>46249</v>
       </c>
-      <c r="L48" s="198"/>
-      <c r="M48" s="198"/>
+      <c r="L48" s="260"/>
+      <c r="M48" s="260"/>
       <c r="N48" s="128"/>
       <c r="O48" s="120"/>
       <c r="P48" s="120"/>
       <c r="Q48" s="127"/>
       <c r="R48" s="7"/>
-      <c r="S48" s="202"/>
-      <c r="T48" s="203"/>
-      <c r="U48" s="203"/>
-      <c r="V48" s="203"/>
-      <c r="W48" s="203"/>
-      <c r="X48" s="196"/>
-      <c r="Y48" s="196"/>
-      <c r="Z48" s="196"/>
-      <c r="AA48" s="196"/>
-      <c r="AB48" s="196"/>
-      <c r="AC48" s="196"/>
-      <c r="AD48" s="196"/>
-      <c r="AE48" s="197"/>
+      <c r="S48" s="252"/>
+      <c r="T48" s="257"/>
+      <c r="U48" s="257"/>
+      <c r="V48" s="257"/>
+      <c r="W48" s="257"/>
+      <c r="X48" s="248"/>
+      <c r="Y48" s="248"/>
+      <c r="Z48" s="248"/>
+      <c r="AA48" s="248"/>
+      <c r="AB48" s="248"/>
+      <c r="AC48" s="248"/>
+      <c r="AD48" s="248"/>
+      <c r="AE48" s="251"/>
     </row>
     <row r="49" spans="1:62" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="2"/>
@@ -6013,40 +5976,40 @@
       <c r="P49" s="120"/>
       <c r="Q49" s="127"/>
       <c r="R49" s="7"/>
-      <c r="S49" s="194">
+      <c r="S49" s="269">
         <v>5</v>
       </c>
-      <c r="T49" s="195" t="s">
-        <v>164</v>
-      </c>
-      <c r="U49" s="195"/>
-      <c r="V49" s="195"/>
-      <c r="W49" s="195"/>
-      <c r="X49" s="186">
+      <c r="T49" s="270" t="s">
+        <v>163</v>
+      </c>
+      <c r="U49" s="270"/>
+      <c r="V49" s="270"/>
+      <c r="W49" s="270"/>
+      <c r="X49" s="261">
         <f>+AM111</f>
-        <v>268.94</v>
-      </c>
-      <c r="Y49" s="186"/>
-      <c r="Z49" s="186">
+        <v>86.38</v>
+      </c>
+      <c r="Y49" s="261"/>
+      <c r="Z49" s="261">
         <f>+AR111</f>
-        <v>53.78</v>
-      </c>
-      <c r="AA49" s="186"/>
-      <c r="AB49" s="186">
+        <v>17.27</v>
+      </c>
+      <c r="AA49" s="261"/>
+      <c r="AB49" s="261">
         <f>+AT111</f>
-        <v>107.57</v>
-      </c>
-      <c r="AC49" s="186">
+        <v>34.549999999999997</v>
+      </c>
+      <c r="AC49" s="261">
         <f>+AV111</f>
-        <v>53.78</v>
-      </c>
-      <c r="AD49" s="186">
+        <v>17.27</v>
+      </c>
+      <c r="AD49" s="261">
         <f>+AX111</f>
-        <v>107.57</v>
-      </c>
-      <c r="AE49" s="188">
+        <v>34.549999999999997</v>
+      </c>
+      <c r="AE49" s="263">
         <f>+AZ111</f>
-        <v>134.47</v>
+        <v>43.19</v>
       </c>
     </row>
     <row r="50" spans="1:62" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -6068,58 +6031,58 @@
       <c r="P50" s="120"/>
       <c r="Q50" s="127"/>
       <c r="R50" s="7"/>
-      <c r="S50" s="194"/>
-      <c r="T50" s="195"/>
-      <c r="U50" s="195"/>
-      <c r="V50" s="195"/>
-      <c r="W50" s="195"/>
-      <c r="X50" s="186"/>
-      <c r="Y50" s="186"/>
-      <c r="Z50" s="186"/>
-      <c r="AA50" s="186"/>
-      <c r="AB50" s="186"/>
-      <c r="AC50" s="186"/>
-      <c r="AD50" s="186"/>
-      <c r="AE50" s="188"/>
+      <c r="S50" s="269"/>
+      <c r="T50" s="270"/>
+      <c r="U50" s="270"/>
+      <c r="V50" s="270"/>
+      <c r="W50" s="270"/>
+      <c r="X50" s="261"/>
+      <c r="Y50" s="261"/>
+      <c r="Z50" s="261"/>
+      <c r="AA50" s="261"/>
+      <c r="AB50" s="261"/>
+      <c r="AC50" s="261"/>
+      <c r="AD50" s="261"/>
+      <c r="AE50" s="263"/>
     </row>
     <row r="51" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A51" s="2"/>
-      <c r="B51" s="189" t="s">
+      <c r="B51" s="264" t="s">
         <v>74</v>
       </c>
-      <c r="C51" s="189"/>
-      <c r="D51" s="189"/>
-      <c r="E51" s="189"/>
-      <c r="F51" s="190" t="s">
+      <c r="C51" s="264"/>
+      <c r="D51" s="264"/>
+      <c r="E51" s="264"/>
+      <c r="F51" s="265" t="s">
         <v>74</v>
       </c>
-      <c r="G51" s="190"/>
-      <c r="H51" s="190"/>
-      <c r="I51" s="191" t="s">
+      <c r="G51" s="265"/>
+      <c r="H51" s="265"/>
+      <c r="I51" s="266" t="s">
         <v>74</v>
       </c>
-      <c r="J51" s="191"/>
-      <c r="K51" s="191"/>
-      <c r="L51" s="191"/>
-      <c r="M51" s="191"/>
-      <c r="N51" s="191"/>
-      <c r="O51" s="191"/>
-      <c r="P51" s="191"/>
-      <c r="Q51" s="191"/>
+      <c r="J51" s="266"/>
+      <c r="K51" s="266"/>
+      <c r="L51" s="266"/>
+      <c r="M51" s="266"/>
+      <c r="N51" s="266"/>
+      <c r="O51" s="266"/>
+      <c r="P51" s="266"/>
+      <c r="Q51" s="266"/>
       <c r="R51" s="7"/>
-      <c r="S51" s="194"/>
-      <c r="T51" s="195"/>
-      <c r="U51" s="195"/>
-      <c r="V51" s="195"/>
-      <c r="W51" s="195"/>
-      <c r="X51" s="186"/>
-      <c r="Y51" s="186"/>
-      <c r="Z51" s="186"/>
-      <c r="AA51" s="186"/>
-      <c r="AB51" s="186"/>
-      <c r="AC51" s="186"/>
-      <c r="AD51" s="186"/>
-      <c r="AE51" s="188"/>
+      <c r="S51" s="269"/>
+      <c r="T51" s="270"/>
+      <c r="U51" s="270"/>
+      <c r="V51" s="270"/>
+      <c r="W51" s="270"/>
+      <c r="X51" s="261"/>
+      <c r="Y51" s="261"/>
+      <c r="Z51" s="261"/>
+      <c r="AA51" s="261"/>
+      <c r="AB51" s="261"/>
+      <c r="AC51" s="261"/>
+      <c r="AD51" s="261"/>
+      <c r="AE51" s="263"/>
     </row>
     <row r="52" spans="1:62" ht="13.5" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A52" s="2"/>
@@ -6186,11 +6149,11 @@
     <row r="57" spans="1:62" hidden="1" x14ac:dyDescent="0.2">
       <c r="AJ57" s="77">
         <f>AE29</f>
-        <v>53.78</v>
+        <v>17.27</v>
       </c>
       <c r="AL57" s="77" t="str">
         <f>TEXT(AE29,"0000,00")</f>
-        <v>0053,78</v>
+        <v>0017,27</v>
       </c>
     </row>
     <row r="58" spans="1:62" hidden="1" x14ac:dyDescent="0.2"/>
@@ -6272,11 +6235,11 @@
       </c>
       <c r="AL66" s="1" t="str">
         <f>IF(MID($AL$57,$AL$75-1,1)="1",MID($AL$57,$AL75-1,2),MID($AL$57,$AL$75,1))</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AM66" s="1" t="str">
         <f ca="1">LOOKUP(VALUE(AL66),$AI$64:$AI$103,$AJ$64:$AJ$8727)</f>
-        <v>oito</v>
+        <v>sete</v>
       </c>
       <c r="AN66" s="1" t="str">
         <f t="shared" ref="AN66:AN71" si="8">IF(AL66="0","F","T")</f>
@@ -6284,7 +6247,7 @@
       </c>
       <c r="AO66" s="1" t="str">
         <f ca="1">IF(AND(AL67="0",AL69="0",AL71="0"),AM70&amp;" e "&amp;AM68&amp;AL77&amp;AM66&amp;AM77,AM67&amp;" e "&amp;AM66&amp;AM77)</f>
-        <v xml:space="preserve">setenta e oito centavos </v>
+        <v xml:space="preserve">vinte e sete centavos </v>
       </c>
     </row>
     <row r="67" spans="33:62" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6301,11 +6264,11 @@
       </c>
       <c r="AL67" s="1" t="str">
         <f>IF(MID($AL$57,$AL$75-1,1)&gt;"1",MID($AL$57,$AL$75-1,1),"0")</f>
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="AM67" s="1" t="str">
         <f ca="1">LOOKUP(VALUE(AL67)*10,$AI$64:$AI$103,$AJ$64:$AJ$8727)</f>
-        <v>setenta</v>
+        <v>vinte</v>
       </c>
       <c r="AN67" s="1" t="str">
         <f t="shared" si="8"/>
@@ -6345,11 +6308,11 @@
       </c>
       <c r="AL68" s="1" t="str">
         <f>IF(MID($AL$57,$AL$75-4,1)="1",MID($AL$57,$AL$75-4,2),MID($AL$57,$AL$75-3,1))</f>
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="AM68" s="1" t="str">
         <f ca="1">LOOKUP(VALUE(AL68),$AI$64:$AI$103,$AJ$64:$AJ$8727)</f>
-        <v>três</v>
+        <v>dezessete</v>
       </c>
       <c r="AN68" s="1" t="str">
         <f t="shared" si="8"/>
@@ -6368,15 +6331,15 @@
       </c>
       <c r="AL69" s="1" t="str">
         <f>IF(MID($AL$57,$AL$75-4,1)&gt;"1",MID($AL$57,$AL$75-4,1),"0")</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AM69" s="1" t="str">
         <f>LOOKUP(VALUE(AL69)*10,$AI$64:$AI$103,$AJ$64:$AJ$103)</f>
-        <v>cinqüenta</v>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="AN69" s="1" t="str">
         <f t="shared" si="8"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="70" spans="33:62" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6529,7 +6492,7 @@
       </c>
       <c r="AO77" s="182" t="str">
         <f ca="1">UPPER("*** "&amp;AM78&amp;AM80&amp;AM79&amp;"***")</f>
-        <v>*** CINQÜENTA E TRÊS REAIS  E SETENTA E OITO CENTAVOS ***</v>
+        <v>*** DEZESSETE REAIS  E VINTE E SETE CENTAVOS ***</v>
       </c>
     </row>
     <row r="78" spans="33:62" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6563,7 +6526,7 @@
       </c>
       <c r="AM79" s="1" t="str">
         <f ca="1">IF(AN66&amp;AN67="TT"," e "&amp;AM67&amp;" e "&amp;AM66&amp;AM77,IF(AN66&amp;AN67="FF","",IF(AN66&amp;AN67="TF"," e "&amp;AM66&amp;AM77,IF(AN66&amp;AN67="FT"," e "&amp;AM67&amp;AM77))))</f>
-        <v xml:space="preserve"> e setenta e oito centavos </v>
+        <v xml:space="preserve"> e vinte e sete centavos </v>
       </c>
     </row>
     <row r="80" spans="33:62" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6575,14 +6538,14 @@
       </c>
       <c r="AK80" s="1" t="str">
         <f>AN68&amp;AN69&amp;AN70</f>
-        <v>TTF</v>
+        <v>TFF</v>
       </c>
       <c r="AL80" s="1" t="s">
         <v>102</v>
       </c>
       <c r="AM80" s="1" t="str">
         <f ca="1">IF(AN68&amp;AN69&amp;AN70="TTT",AM70&amp;" e "&amp;AM69&amp;" e "&amp;AM68&amp;AL77,IF(AN68&amp;AN69&amp;AN70="FTT",AM70&amp;" e "&amp;AM69&amp;AL77,IF(AN68&amp;AN69&amp;AN70="FFT",AM70&amp;AL77,IF(AN68&amp;AN69&amp;AN70="TTF",AM69&amp;" e "&amp;AM68&amp;AL77,IF(AN68&amp;AN69&amp;AN70="TFT",AM70&amp;" e "&amp;AM68&amp;AL77,IF(AN68&amp;AN69&amp;AN70="TFF",AM68&amp;AL77,IF(AN68&amp;AN69&amp;AN70="FFF"," ",IF(AN68&amp;AN69&amp;AN70="FTF",AM69&amp;AL77," "))))))))</f>
-        <v xml:space="preserve">cinqüenta e três reais </v>
+        <v xml:space="preserve">dezessete reais </v>
       </c>
     </row>
     <row r="81" spans="33:75" ht="9.9499999999999993" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
@@ -6613,7 +6576,7 @@
       </c>
       <c r="AM83" s="1" t="str">
         <f ca="1">AM70&amp;" e "&amp;AM69&amp;" e "&amp;AM68&amp;AL77</f>
-        <v xml:space="preserve">  e cinqüenta e três reais </v>
+        <v xml:space="preserve">  e   e dezessete reais </v>
       </c>
       <c r="AO83" s="1" t="s">
         <v>107</v>
@@ -6634,7 +6597,7 @@
       </c>
       <c r="AM84" s="1" t="str">
         <f ca="1">AM70&amp;" e "&amp;AM69&amp;AL77</f>
-        <v xml:space="preserve">  e cinqüenta reais </v>
+        <v xml:space="preserve">  e   reais </v>
       </c>
       <c r="AN84" s="1"/>
       <c r="AO84" s="1" t="s">
@@ -6767,7 +6730,7 @@
       </c>
       <c r="AM87" s="1" t="str">
         <f>AM69&amp;AL77</f>
-        <v xml:space="preserve">cinqüenta reais </v>
+        <v xml:space="preserve">  reais </v>
       </c>
       <c r="AO87" s="1" t="s">
         <v>118</v>
@@ -6798,7 +6761,7 @@
       </c>
       <c r="AM88" s="1" t="str">
         <f ca="1">AM69&amp;" e "&amp;AM68&amp;AL77</f>
-        <v xml:space="preserve">cinqüenta e três reais </v>
+        <v xml:space="preserve">  e dezessete reais </v>
       </c>
       <c r="AO88" s="1" t="s">
         <v>121</v>
@@ -6829,7 +6792,7 @@
       </c>
       <c r="AM89" s="1" t="str">
         <f ca="1">AM70&amp;" e "&amp;AM68&amp;AL77</f>
-        <v xml:space="preserve">  e três reais </v>
+        <v xml:space="preserve">  e dezessete reais </v>
       </c>
       <c r="AO89" s="1" t="s">
         <v>124</v>
@@ -6860,7 +6823,7 @@
       </c>
       <c r="AM90" s="1" t="str">
         <f>AM69&amp;AL77</f>
-        <v xml:space="preserve">cinqüenta reais </v>
+        <v xml:space="preserve">  reais </v>
       </c>
       <c r="AO90" s="1" t="s">
         <v>118</v>
@@ -6913,7 +6876,7 @@
       </c>
       <c r="AM92" s="1" t="str">
         <f ca="1">AM67&amp;" e "&amp;AM66&amp;AM77</f>
-        <v xml:space="preserve">setenta e oito centavos </v>
+        <v xml:space="preserve">vinte e sete centavos </v>
       </c>
       <c r="AO92" s="1" t="s">
         <v>130</v>
@@ -6944,7 +6907,7 @@
       </c>
       <c r="AM93" s="1" t="str">
         <f ca="1">AM67&amp;AM77</f>
-        <v xml:space="preserve">setenta centavos </v>
+        <v xml:space="preserve">vinte centavos </v>
       </c>
       <c r="AO93" s="1" t="s">
         <v>133</v>
@@ -7005,7 +6968,7 @@
       </c>
       <c r="AM95" s="1" t="str">
         <f ca="1">AM66&amp;AM77</f>
-        <v xml:space="preserve">oito centavos </v>
+        <v xml:space="preserve">sete centavos </v>
       </c>
       <c r="AO95" s="1" t="s">
         <v>139</v>
@@ -7118,22 +7081,22 @@
       <c r="AP104" s="138" t="s">
         <v>29</v>
       </c>
-      <c r="AQ104" s="192" t="s">
+      <c r="AQ104" s="267" t="s">
         <v>30</v>
       </c>
-      <c r="AR104" s="192"/>
-      <c r="AS104" s="192"/>
-      <c r="AT104" s="192"/>
-      <c r="AU104" s="193" t="s">
+      <c r="AR104" s="267"/>
+      <c r="AS104" s="267"/>
+      <c r="AT104" s="267"/>
+      <c r="AU104" s="268" t="s">
         <v>31</v>
       </c>
-      <c r="AV104" s="193"/>
-      <c r="AW104" s="193"/>
-      <c r="AX104" s="193"/>
-      <c r="AY104" s="187" t="s">
+      <c r="AV104" s="268"/>
+      <c r="AW104" s="268"/>
+      <c r="AX104" s="268"/>
+      <c r="AY104" s="262" t="s">
         <v>32</v>
       </c>
-      <c r="AZ104" s="187"/>
+      <c r="AZ104" s="262"/>
       <c r="BA104" s="6"/>
       <c r="BB104" s="6"/>
       <c r="BC104" s="6"/>
@@ -7268,11 +7231,11 @@
       </c>
       <c r="AL107" s="161">
         <f>+(AC10*AK107)+AC10</f>
-        <v>537.88</v>
+        <v>172.76</v>
       </c>
       <c r="AM107" s="162">
         <f>ROUNDDOWN(AL107,2)</f>
-        <v>537.88</v>
+        <v>172.76</v>
       </c>
       <c r="AN107" s="163">
         <v>1</v>
@@ -7282,47 +7245,47 @@
       </c>
       <c r="AP107" s="165">
         <f>+AM107</f>
-        <v>537.88</v>
+        <v>172.76</v>
       </c>
       <c r="AQ107" s="166">
         <f>+AQ105*AM107</f>
-        <v>107.57599999999999</v>
+        <v>34.552</v>
       </c>
       <c r="AR107" s="167">
         <f>+ROUNDDOWN(AQ107,2)</f>
-        <v>107.57</v>
+        <v>34.549999999999997</v>
       </c>
       <c r="AS107" s="166">
         <f>+AS$105*AM107</f>
-        <v>215.15199999999999</v>
+        <v>69.103999999999999</v>
       </c>
       <c r="AT107" s="167">
         <f>ROUNDDOWN(AS107,2)</f>
-        <v>215.15</v>
+        <v>69.099999999999994</v>
       </c>
       <c r="AU107" s="168">
         <f>+AU$105*AM107</f>
-        <v>107.57599999999999</v>
+        <v>34.552</v>
       </c>
       <c r="AV107" s="169">
         <f>ROUNDDOWN(AU107,2)</f>
-        <v>107.57</v>
+        <v>34.549999999999997</v>
       </c>
       <c r="AW107" s="168">
         <f>+AW$105*AM107</f>
-        <v>215.15199999999999</v>
+        <v>69.103999999999999</v>
       </c>
       <c r="AX107" s="169">
         <f>ROUNDDOWN(AW107,2)</f>
-        <v>215.15</v>
+        <v>69.099999999999994</v>
       </c>
       <c r="AY107" s="170">
         <f>+AY105*AM107</f>
-        <v>268.94</v>
+        <v>86.38</v>
       </c>
       <c r="AZ107" s="171">
         <f>ROUNDDOWN(AY107,2)</f>
-        <v>268.94</v>
+        <v>86.38</v>
       </c>
       <c r="BA107" s="6"/>
       <c r="BB107" s="6"/>
@@ -7343,11 +7306,11 @@
       </c>
       <c r="AL108" s="161">
         <f>+(AC10*AK108)+AC10</f>
-        <v>484.09199999999998</v>
+        <v>155.48400000000001</v>
       </c>
       <c r="AM108" s="162">
         <f>ROUNDDOWN(AL108,2)</f>
-        <v>484.09</v>
+        <v>155.47999999999999</v>
       </c>
       <c r="AN108" s="172">
         <v>2</v>
@@ -7357,47 +7320,47 @@
       </c>
       <c r="AP108" s="165">
         <f>+AM108</f>
-        <v>484.09</v>
+        <v>155.47999999999999</v>
       </c>
       <c r="AQ108" s="166">
         <f>+AQ105*AM108</f>
-        <v>96.817999999999998</v>
+        <v>31.096</v>
       </c>
       <c r="AR108" s="167">
         <f>+ROUNDDOWN(AQ108,2)</f>
-        <v>96.81</v>
+        <v>31.09</v>
       </c>
       <c r="AS108" s="166">
         <f>+AS$105*AM108</f>
-        <v>193.636</v>
+        <v>62.192</v>
       </c>
       <c r="AT108" s="167">
         <f>ROUNDDOWN(AS108,2)</f>
-        <v>193.63</v>
+        <v>62.19</v>
       </c>
       <c r="AU108" s="168">
         <f>+AU$105*AM108</f>
-        <v>96.817999999999998</v>
+        <v>31.096</v>
       </c>
       <c r="AV108" s="169">
         <f>ROUNDDOWN(AU108,2)</f>
-        <v>96.81</v>
+        <v>31.09</v>
       </c>
       <c r="AW108" s="168">
         <f>+AW$105*AM108</f>
-        <v>193.636</v>
+        <v>62.192</v>
       </c>
       <c r="AX108" s="169">
         <f>ROUNDDOWN(AW108,2)</f>
-        <v>193.63</v>
+        <v>62.19</v>
       </c>
       <c r="AY108" s="170">
         <f>+AY105*AM108</f>
-        <v>242.04499999999999</v>
+        <v>77.739999999999995</v>
       </c>
       <c r="AZ108" s="171">
         <f>ROUNDDOWN(AY108,2)</f>
-        <v>242.04</v>
+        <v>77.739999999999995</v>
       </c>
       <c r="BA108" s="6"/>
       <c r="BB108" s="6"/>
@@ -7418,11 +7381,11 @@
       </c>
       <c r="AL109" s="161">
         <f>+(AC10*AK109)+AC10</f>
-        <v>457.19799999999998</v>
+        <v>146.846</v>
       </c>
       <c r="AM109" s="162">
         <f>ROUNDDOWN(AL109,2)</f>
-        <v>457.19</v>
+        <v>146.84</v>
       </c>
       <c r="AN109" s="163">
         <v>3</v>
@@ -7432,47 +7395,47 @@
       </c>
       <c r="AP109" s="165">
         <f>+AM109</f>
-        <v>457.19</v>
+        <v>146.84</v>
       </c>
       <c r="AQ109" s="166">
         <f>+AQ105*AM109</f>
-        <v>91.438000000000002</v>
+        <v>29.367999999999999</v>
       </c>
       <c r="AR109" s="167">
         <f>+ROUNDDOWN(AQ109,2)</f>
-        <v>91.43</v>
+        <v>29.36</v>
       </c>
       <c r="AS109" s="166">
         <f>+AS$105*AM109</f>
-        <v>182.876</v>
+        <v>58.735999999999997</v>
       </c>
       <c r="AT109" s="167">
         <f>ROUNDDOWN(AS109,2)</f>
-        <v>182.87</v>
+        <v>58.73</v>
       </c>
       <c r="AU109" s="168">
         <f>+AU$105*AM109</f>
-        <v>91.438000000000002</v>
+        <v>29.367999999999999</v>
       </c>
       <c r="AV109" s="169">
         <f>ROUNDDOWN(AU109,2)</f>
-        <v>91.43</v>
+        <v>29.36</v>
       </c>
       <c r="AW109" s="168">
         <f>+AW$105*AM109</f>
-        <v>182.876</v>
+        <v>58.735999999999997</v>
       </c>
       <c r="AX109" s="169">
         <f>ROUNDDOWN(AW109,2)</f>
-        <v>182.87</v>
+        <v>58.73</v>
       </c>
       <c r="AY109" s="170">
         <f>+AY105*AM109</f>
-        <v>228.595</v>
+        <v>73.42</v>
       </c>
       <c r="AZ109" s="171">
         <f>ROUNDDOWN(AY109,2)</f>
-        <v>228.59</v>
+        <v>73.42</v>
       </c>
       <c r="BA109" s="6"/>
       <c r="BB109" s="6"/>
@@ -7493,11 +7456,11 @@
       </c>
       <c r="AL110" s="175">
         <f>+(AC10*AK110)+AC10</f>
-        <v>403.41</v>
+        <v>129.57</v>
       </c>
       <c r="AM110" s="176">
         <f>ROUNDDOWN(AL110,2)</f>
-        <v>403.41</v>
+        <v>129.57</v>
       </c>
       <c r="AN110" s="177">
         <v>4</v>
@@ -7507,47 +7470,47 @@
       </c>
       <c r="AP110" s="178">
         <f>+AM110</f>
-        <v>403.41</v>
+        <v>129.57</v>
       </c>
       <c r="AQ110" s="179">
         <f>+AQ105*AM110</f>
-        <v>80.682000000000002</v>
+        <v>25.914000000000001</v>
       </c>
       <c r="AR110" s="167">
         <f>+ROUNDDOWN(AQ110,2)</f>
-        <v>80.680000000000007</v>
+        <v>25.91</v>
       </c>
       <c r="AS110" s="166">
         <f>+AS$105*AM110</f>
-        <v>161.364</v>
+        <v>51.828000000000003</v>
       </c>
       <c r="AT110" s="167">
         <f>ROUNDDOWN(AS110,2)</f>
-        <v>161.36000000000001</v>
+        <v>51.82</v>
       </c>
       <c r="AU110" s="168">
         <f>+AU$105*AM110</f>
-        <v>80.682000000000002</v>
+        <v>25.914000000000001</v>
       </c>
       <c r="AV110" s="169">
         <f>ROUNDDOWN(AU110,2)</f>
-        <v>80.680000000000007</v>
+        <v>25.91</v>
       </c>
       <c r="AW110" s="168">
         <f>+AW$105*AM110</f>
-        <v>161.364</v>
+        <v>51.828000000000003</v>
       </c>
       <c r="AX110" s="169">
         <f>ROUNDDOWN(AW110,2)</f>
-        <v>161.36000000000001</v>
+        <v>51.82</v>
       </c>
       <c r="AY110" s="180">
         <f>+AY105*AM110</f>
-        <v>201.70500000000001</v>
+        <v>64.784999999999997</v>
       </c>
       <c r="AZ110" s="171">
         <f>ROUNDDOWN(AY110,2)</f>
-        <v>201.7</v>
+        <v>64.78</v>
       </c>
       <c r="BA110" s="6"/>
       <c r="BB110" s="6"/>
@@ -7568,11 +7531,11 @@
       </c>
       <c r="AL111" s="175">
         <f>+AC10</f>
-        <v>268.94</v>
+        <v>86.38</v>
       </c>
       <c r="AM111" s="176">
         <f>ROUNDDOWN(AL111,2)</f>
-        <v>268.94</v>
+        <v>86.38</v>
       </c>
       <c r="AN111" s="177">
         <v>5</v>
@@ -7582,47 +7545,47 @@
       </c>
       <c r="AP111" s="178">
         <f>+AM111</f>
-        <v>268.94</v>
+        <v>86.38</v>
       </c>
       <c r="AQ111" s="179">
         <f>+AQ105*AM111</f>
-        <v>53.787999999999997</v>
+        <v>17.276</v>
       </c>
       <c r="AR111" s="167">
         <f>+ROUNDDOWN(AQ111,2)</f>
-        <v>53.78</v>
+        <v>17.27</v>
       </c>
       <c r="AS111" s="166">
         <f>+AS$105*AM111</f>
-        <v>107.57599999999999</v>
+        <v>34.552</v>
       </c>
       <c r="AT111" s="167">
         <f>ROUNDDOWN(AS111,2)</f>
-        <v>107.57</v>
+        <v>34.549999999999997</v>
       </c>
       <c r="AU111" s="168">
         <f>+AU$105*AM111</f>
-        <v>53.787999999999997</v>
+        <v>17.276</v>
       </c>
       <c r="AV111" s="169">
         <f>ROUNDDOWN(AU111,2)</f>
-        <v>53.78</v>
+        <v>17.27</v>
       </c>
       <c r="AW111" s="168">
         <f>+AW$105*AM111</f>
-        <v>107.57599999999999</v>
+        <v>34.552</v>
       </c>
       <c r="AX111" s="169">
         <f>ROUNDDOWN(AW111,2)</f>
-        <v>107.57</v>
+        <v>34.549999999999997</v>
       </c>
       <c r="AY111" s="180">
         <f>+AY105*AM111</f>
-        <v>134.47</v>
+        <v>43.19</v>
       </c>
       <c r="AZ111" s="171">
         <f>ROUNDDOWN(AY111,2)</f>
-        <v>134.47</v>
+        <v>43.19</v>
       </c>
       <c r="BA111" s="6"/>
       <c r="BB111" s="6"/>
@@ -7691,9 +7654,6 @@
     <row r="152" hidden="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <customSheetViews>
-    <customSheetView guid="{21947858-9CF7-CF4C-8635-4940C68DA20F}" showRuler="0">
-      <pageMargins left="0.78740157499999996" right="0.78740157499999996" top="0.984251969" bottom="0.984251969" header="0.4921259845" footer="0.4921259845"/>
-    </customSheetView>
     <customSheetView guid="{FF834EEA-98EE-4D52-930D-AE89D7F4F75B}" colorId="8" showGridLines="0" zeroValues="0" hiddenRows="1" hiddenColumns="1" topLeftCell="A7">
       <selection activeCell="BE46" sqref="BE46"/>
       <pageMargins left="0.78749999999999998" right="0.39374999999999999" top="0.6694444444444444" bottom="0.39374999999999999" header="0.51180555555555551" footer="0.51180555555555551"/>
@@ -7701,115 +7661,59 @@
       <pageSetup paperSize="9" scale="80" firstPageNumber="0" orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
       <headerFooter alignWithMargins="0"/>
     </customSheetView>
+    <customSheetView guid="{21947858-9CF7-CF4C-8635-4940C68DA20F}" showRuler="0">
+      <pageMargins left="0.78740157499999996" right="0.78740157499999996" top="0.984251969" bottom="0.984251969" header="0.4921259845" footer="0.4921259845"/>
+    </customSheetView>
   </customSheetViews>
   <mergeCells count="179">
-    <mergeCell ref="S9:U9"/>
-    <mergeCell ref="B10:D11"/>
-    <mergeCell ref="E10:J11"/>
-    <mergeCell ref="K10:M11"/>
-    <mergeCell ref="N10:R11"/>
-    <mergeCell ref="T10:U10"/>
-    <mergeCell ref="F2:AD2"/>
-    <mergeCell ref="F3:AD3"/>
-    <mergeCell ref="F4:AD4"/>
-    <mergeCell ref="F5:AD5"/>
-    <mergeCell ref="B8:M8"/>
-    <mergeCell ref="N8:S8"/>
-    <mergeCell ref="T8:AB8"/>
-    <mergeCell ref="AC8:AE8"/>
-    <mergeCell ref="AE13:AE15"/>
-    <mergeCell ref="P14:P15"/>
-    <mergeCell ref="Q14:Q15"/>
-    <mergeCell ref="R14:V14"/>
-    <mergeCell ref="W14:AB14"/>
-    <mergeCell ref="AC14:AC15"/>
-    <mergeCell ref="AD14:AD15"/>
-    <mergeCell ref="V10:Y11"/>
-    <mergeCell ref="Z10:Z11"/>
-    <mergeCell ref="AA10:AB11"/>
-    <mergeCell ref="AC10:AE11"/>
-    <mergeCell ref="T11:U11"/>
-    <mergeCell ref="P13:AD13"/>
-    <mergeCell ref="B17:E17"/>
-    <mergeCell ref="G17:I17"/>
-    <mergeCell ref="M17:O17"/>
-    <mergeCell ref="U17:V17"/>
-    <mergeCell ref="X17:Y17"/>
-    <mergeCell ref="AA17:AB17"/>
-    <mergeCell ref="M15:O15"/>
-    <mergeCell ref="U15:V15"/>
-    <mergeCell ref="X15:Y15"/>
-    <mergeCell ref="AA15:AB15"/>
-    <mergeCell ref="B16:E16"/>
-    <mergeCell ref="G16:I16"/>
-    <mergeCell ref="M16:O16"/>
-    <mergeCell ref="U16:V16"/>
-    <mergeCell ref="X16:Y16"/>
-    <mergeCell ref="AA16:AB16"/>
-    <mergeCell ref="B13:E15"/>
-    <mergeCell ref="G13:I15"/>
-    <mergeCell ref="J13:K14"/>
-    <mergeCell ref="L13:O14"/>
-    <mergeCell ref="B19:E19"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="M19:O19"/>
-    <mergeCell ref="U19:V19"/>
-    <mergeCell ref="X19:Y19"/>
-    <mergeCell ref="AA19:AB19"/>
-    <mergeCell ref="B18:E18"/>
-    <mergeCell ref="G18:I18"/>
-    <mergeCell ref="M18:O18"/>
-    <mergeCell ref="U18:V18"/>
-    <mergeCell ref="X18:Y18"/>
-    <mergeCell ref="AA18:AB18"/>
-    <mergeCell ref="B21:E21"/>
-    <mergeCell ref="G21:I21"/>
-    <mergeCell ref="M21:O21"/>
-    <mergeCell ref="U21:V21"/>
-    <mergeCell ref="X21:Y21"/>
-    <mergeCell ref="AA21:AB21"/>
-    <mergeCell ref="B20:E20"/>
-    <mergeCell ref="G20:I20"/>
-    <mergeCell ref="M20:O20"/>
-    <mergeCell ref="U20:V20"/>
-    <mergeCell ref="X20:Y20"/>
-    <mergeCell ref="AA20:AB20"/>
-    <mergeCell ref="B23:E23"/>
-    <mergeCell ref="G23:I23"/>
-    <mergeCell ref="M23:O23"/>
-    <mergeCell ref="U23:V23"/>
-    <mergeCell ref="X23:Y23"/>
-    <mergeCell ref="AA23:AB23"/>
-    <mergeCell ref="B22:E22"/>
-    <mergeCell ref="G22:I22"/>
-    <mergeCell ref="M22:O22"/>
-    <mergeCell ref="U22:V22"/>
-    <mergeCell ref="X22:Y22"/>
-    <mergeCell ref="AA22:AB22"/>
-    <mergeCell ref="B25:E25"/>
-    <mergeCell ref="G25:I25"/>
-    <mergeCell ref="M25:O25"/>
-    <mergeCell ref="U25:V25"/>
-    <mergeCell ref="X25:Y25"/>
-    <mergeCell ref="AA25:AB25"/>
-    <mergeCell ref="B24:E24"/>
-    <mergeCell ref="G24:I24"/>
-    <mergeCell ref="M24:O24"/>
-    <mergeCell ref="U24:V24"/>
-    <mergeCell ref="X24:Y24"/>
-    <mergeCell ref="AA24:AB24"/>
-    <mergeCell ref="B27:E27"/>
-    <mergeCell ref="G27:I27"/>
-    <mergeCell ref="M27:O27"/>
-    <mergeCell ref="U27:V27"/>
-    <mergeCell ref="X27:Y27"/>
-    <mergeCell ref="AA27:AB27"/>
-    <mergeCell ref="B26:E26"/>
-    <mergeCell ref="G26:I26"/>
-    <mergeCell ref="M26:O26"/>
-    <mergeCell ref="U26:V26"/>
-    <mergeCell ref="X26:Y26"/>
-    <mergeCell ref="AA26:AB26"/>
+    <mergeCell ref="AD49:AD51"/>
+    <mergeCell ref="AY104:AZ104"/>
+    <mergeCell ref="AE49:AE51"/>
+    <mergeCell ref="B51:E51"/>
+    <mergeCell ref="F51:H51"/>
+    <mergeCell ref="I51:Q51"/>
+    <mergeCell ref="AQ104:AT104"/>
+    <mergeCell ref="AU104:AX104"/>
+    <mergeCell ref="S49:S51"/>
+    <mergeCell ref="T49:W51"/>
+    <mergeCell ref="X49:Y51"/>
+    <mergeCell ref="Z49:AA51"/>
+    <mergeCell ref="AB49:AB51"/>
+    <mergeCell ref="AC49:AC51"/>
+    <mergeCell ref="Z46:AA48"/>
+    <mergeCell ref="AB46:AB48"/>
+    <mergeCell ref="AC46:AC48"/>
+    <mergeCell ref="AD46:AD48"/>
+    <mergeCell ref="AE46:AE48"/>
+    <mergeCell ref="K48:M48"/>
+    <mergeCell ref="AB43:AB45"/>
+    <mergeCell ref="AC43:AC45"/>
+    <mergeCell ref="AD43:AD45"/>
+    <mergeCell ref="AE43:AE45"/>
+    <mergeCell ref="Z43:AA45"/>
+    <mergeCell ref="C45:E45"/>
+    <mergeCell ref="F46:H46"/>
+    <mergeCell ref="I46:L46"/>
+    <mergeCell ref="S46:S48"/>
+    <mergeCell ref="T46:W48"/>
+    <mergeCell ref="X46:Y48"/>
+    <mergeCell ref="M41:Q41"/>
+    <mergeCell ref="I42:Q44"/>
+    <mergeCell ref="S43:S45"/>
+    <mergeCell ref="T43:W45"/>
+    <mergeCell ref="X43:Y45"/>
+    <mergeCell ref="Z35:AB35"/>
+    <mergeCell ref="AC35:AD35"/>
+    <mergeCell ref="AD37:AD39"/>
+    <mergeCell ref="AE37:AE39"/>
+    <mergeCell ref="S40:S42"/>
+    <mergeCell ref="T40:W42"/>
+    <mergeCell ref="X40:Y42"/>
+    <mergeCell ref="Z40:AA42"/>
+    <mergeCell ref="AB40:AB42"/>
+    <mergeCell ref="AC40:AC42"/>
+    <mergeCell ref="AD40:AD42"/>
+    <mergeCell ref="AE40:AE42"/>
     <mergeCell ref="B34:Q38"/>
     <mergeCell ref="B29:T31"/>
     <mergeCell ref="U29:AD29"/>
@@ -7834,69 +7738,128 @@
     <mergeCell ref="S35:S36"/>
     <mergeCell ref="T35:W36"/>
     <mergeCell ref="X35:Y36"/>
-    <mergeCell ref="Z35:AB35"/>
-    <mergeCell ref="AC35:AD35"/>
-    <mergeCell ref="AD37:AD39"/>
-    <mergeCell ref="AE37:AE39"/>
-    <mergeCell ref="S40:S42"/>
-    <mergeCell ref="T40:W42"/>
-    <mergeCell ref="X40:Y42"/>
-    <mergeCell ref="Z40:AA42"/>
-    <mergeCell ref="AB40:AB42"/>
-    <mergeCell ref="AC40:AC42"/>
-    <mergeCell ref="AD40:AD42"/>
-    <mergeCell ref="AE40:AE42"/>
-    <mergeCell ref="C45:E45"/>
-    <mergeCell ref="F46:H46"/>
-    <mergeCell ref="I46:L46"/>
-    <mergeCell ref="S46:S48"/>
-    <mergeCell ref="T46:W48"/>
-    <mergeCell ref="X46:Y48"/>
-    <mergeCell ref="M41:Q41"/>
-    <mergeCell ref="I42:Q44"/>
-    <mergeCell ref="S43:S45"/>
-    <mergeCell ref="T43:W45"/>
-    <mergeCell ref="X43:Y45"/>
-    <mergeCell ref="Z46:AA48"/>
-    <mergeCell ref="AB46:AB48"/>
-    <mergeCell ref="AC46:AC48"/>
-    <mergeCell ref="AD46:AD48"/>
-    <mergeCell ref="AE46:AE48"/>
-    <mergeCell ref="K48:M48"/>
-    <mergeCell ref="AB43:AB45"/>
-    <mergeCell ref="AC43:AC45"/>
-    <mergeCell ref="AD43:AD45"/>
-    <mergeCell ref="AE43:AE45"/>
-    <mergeCell ref="Z43:AA45"/>
-    <mergeCell ref="AD49:AD51"/>
-    <mergeCell ref="AY104:AZ104"/>
-    <mergeCell ref="AE49:AE51"/>
-    <mergeCell ref="B51:E51"/>
-    <mergeCell ref="F51:H51"/>
-    <mergeCell ref="I51:Q51"/>
-    <mergeCell ref="AQ104:AT104"/>
-    <mergeCell ref="AU104:AX104"/>
-    <mergeCell ref="S49:S51"/>
-    <mergeCell ref="T49:W51"/>
-    <mergeCell ref="X49:Y51"/>
-    <mergeCell ref="Z49:AA51"/>
-    <mergeCell ref="AB49:AB51"/>
-    <mergeCell ref="AC49:AC51"/>
+    <mergeCell ref="B27:E27"/>
+    <mergeCell ref="G27:I27"/>
+    <mergeCell ref="M27:O27"/>
+    <mergeCell ref="U27:V27"/>
+    <mergeCell ref="X27:Y27"/>
+    <mergeCell ref="AA27:AB27"/>
+    <mergeCell ref="B26:E26"/>
+    <mergeCell ref="G26:I26"/>
+    <mergeCell ref="M26:O26"/>
+    <mergeCell ref="U26:V26"/>
+    <mergeCell ref="X26:Y26"/>
+    <mergeCell ref="AA26:AB26"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="G25:I25"/>
+    <mergeCell ref="M25:O25"/>
+    <mergeCell ref="U25:V25"/>
+    <mergeCell ref="X25:Y25"/>
+    <mergeCell ref="AA25:AB25"/>
+    <mergeCell ref="B24:E24"/>
+    <mergeCell ref="G24:I24"/>
+    <mergeCell ref="M24:O24"/>
+    <mergeCell ref="U24:V24"/>
+    <mergeCell ref="X24:Y24"/>
+    <mergeCell ref="AA24:AB24"/>
+    <mergeCell ref="B23:E23"/>
+    <mergeCell ref="G23:I23"/>
+    <mergeCell ref="M23:O23"/>
+    <mergeCell ref="U23:V23"/>
+    <mergeCell ref="X23:Y23"/>
+    <mergeCell ref="AA23:AB23"/>
+    <mergeCell ref="B22:E22"/>
+    <mergeCell ref="G22:I22"/>
+    <mergeCell ref="M22:O22"/>
+    <mergeCell ref="U22:V22"/>
+    <mergeCell ref="X22:Y22"/>
+    <mergeCell ref="AA22:AB22"/>
+    <mergeCell ref="B21:E21"/>
+    <mergeCell ref="G21:I21"/>
+    <mergeCell ref="M21:O21"/>
+    <mergeCell ref="U21:V21"/>
+    <mergeCell ref="X21:Y21"/>
+    <mergeCell ref="AA21:AB21"/>
+    <mergeCell ref="B20:E20"/>
+    <mergeCell ref="G20:I20"/>
+    <mergeCell ref="M20:O20"/>
+    <mergeCell ref="U20:V20"/>
+    <mergeCell ref="X20:Y20"/>
+    <mergeCell ref="AA20:AB20"/>
+    <mergeCell ref="B19:E19"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="M19:O19"/>
+    <mergeCell ref="U19:V19"/>
+    <mergeCell ref="X19:Y19"/>
+    <mergeCell ref="AA19:AB19"/>
+    <mergeCell ref="B18:E18"/>
+    <mergeCell ref="G18:I18"/>
+    <mergeCell ref="M18:O18"/>
+    <mergeCell ref="U18:V18"/>
+    <mergeCell ref="X18:Y18"/>
+    <mergeCell ref="AA18:AB18"/>
+    <mergeCell ref="B17:E17"/>
+    <mergeCell ref="G17:I17"/>
+    <mergeCell ref="M17:O17"/>
+    <mergeCell ref="U17:V17"/>
+    <mergeCell ref="X17:Y17"/>
+    <mergeCell ref="AA17:AB17"/>
+    <mergeCell ref="M15:O15"/>
+    <mergeCell ref="U15:V15"/>
+    <mergeCell ref="X15:Y15"/>
+    <mergeCell ref="AA15:AB15"/>
+    <mergeCell ref="B16:E16"/>
+    <mergeCell ref="G16:I16"/>
+    <mergeCell ref="M16:O16"/>
+    <mergeCell ref="U16:V16"/>
+    <mergeCell ref="X16:Y16"/>
+    <mergeCell ref="AA16:AB16"/>
+    <mergeCell ref="B13:E15"/>
+    <mergeCell ref="G13:I15"/>
+    <mergeCell ref="J13:K14"/>
+    <mergeCell ref="L13:O14"/>
+    <mergeCell ref="AE13:AE15"/>
+    <mergeCell ref="P14:P15"/>
+    <mergeCell ref="Q14:Q15"/>
+    <mergeCell ref="R14:V14"/>
+    <mergeCell ref="W14:AB14"/>
+    <mergeCell ref="AC14:AC15"/>
+    <mergeCell ref="AD14:AD15"/>
+    <mergeCell ref="V10:Y11"/>
+    <mergeCell ref="Z10:Z11"/>
+    <mergeCell ref="AA10:AB11"/>
+    <mergeCell ref="AC10:AE11"/>
+    <mergeCell ref="T11:U11"/>
+    <mergeCell ref="P13:AD13"/>
+    <mergeCell ref="S9:U9"/>
+    <mergeCell ref="B10:D11"/>
+    <mergeCell ref="E10:J11"/>
+    <mergeCell ref="K10:M11"/>
+    <mergeCell ref="N10:R11"/>
+    <mergeCell ref="T10:U10"/>
+    <mergeCell ref="F2:AD2"/>
+    <mergeCell ref="F3:AD3"/>
+    <mergeCell ref="F4:AD4"/>
+    <mergeCell ref="F5:AD5"/>
+    <mergeCell ref="B8:M8"/>
+    <mergeCell ref="N8:S8"/>
+    <mergeCell ref="T8:AB8"/>
+    <mergeCell ref="AC8:AE8"/>
   </mergeCells>
   <dataValidations xWindow="485" yWindow="298" count="4">
-    <dataValidation operator="equal" allowBlank="1" showErrorMessage="1" sqref="Z10:Z11" xr:uid="{2AD0450F-ADE6-416F-A079-34B6AB66A571}">
+    <dataValidation operator="equal" allowBlank="1" showErrorMessage="1" sqref="Z10:Z11" xr:uid="{F8C9630F-A1B7-421B-8FF4-12F9E1449621}">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="1" showErrorMessage="1" errorTitle="Erro! Dia de chegada inválido!" error="O dia de chegada será sempre maior ou igual ao dia de saída." sqref="P16:X27 Z16:AD16 Y17:AD27" xr:uid="{6A09CF0C-AD83-4153-AA4D-B53078F5C6CB}">
+    <dataValidation allowBlank="1" showErrorMessage="1" errorTitle="Erro! Dia de chegada inválido!" error="O dia de chegada será sempre maior ou igual ao dia de saída." sqref="P16:X27 Z16:AD16 Y17:AD27" xr:uid="{E47B48D2-28DC-4693-A0F0-8F093DDD959F}">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="time" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="FORMATO DE HORA ERRADO" error="O FORMATO DA HORA DEVE SER 00:00_x000a_" prompt="A HORA DEVE SER DIGITADA NO FORMATO 00:00_x000a_" sqref="K16:K27 M16:O27" xr:uid="{F84F1678-6F59-4ECF-B048-A1099031D530}">
+    <dataValidation type="time" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="FORMATO DE HORA ERRADO" error="O FORMATO DA HORA DEVE SER 00:00_x000a_" prompt="A HORA DEVE SER DIGITADA NO FORMATO 00:00_x000a_" sqref="K16:K27 M16:O27" xr:uid="{FAE86953-B033-4B3D-8C02-42784F45D907}">
       <formula1>0</formula1>
       <formula2>0.999988425925926</formula2>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="CÓDIGO DO DESLOCAMENTO" prompt="Informar o código do Local do Deslocamento conforme constante da Tabela de Valores das Diárias ABAIXO:_x000a_Exemplo:_x000a_1  -  D.F. / Manaus_x000a_2  -  São Paulo, etc._x000a_3  -  Demais Capitais_x000a_4  -  Munic. c/ +200.000 hab. e +70 km_x000a_5  -  Demais Deslocamentos" sqref="F16:F27" xr:uid="{91AA9632-2B73-4B9B-869E-753D5F2987B6}">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="CÓDIGO DO DESLOCAMENTO" prompt="Informar o código do Local do Deslocamento conforme constante da Tabela de Valores das Diárias ABAIXO:_x000a_Exemplo:_x000a_1  -  D.F. / Manaus_x000a_2  -  São Paulo, etc._x000a_3  -  Demais Capitais_x000a_4  -  Munic. c/ +200.000 hab. e +70 km_x000a_5  -  Demais Deslocamentos" sqref="F16:F27" xr:uid="{14938A93-AB6D-4491-AC8D-1A65664F292B}">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
@@ -7913,7 +7876,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F257CE6-AB53-4C51-B332-564371EBCE28}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{729A7BAB-EB2C-44CC-B924-1451EC8B3CDE}">
   <dimension ref="A8:AC45"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
@@ -7926,7 +7889,7 @@
     <row r="10" spans="1:29" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="15" spans="1:29" ht="15.75" x14ac:dyDescent="0.2">
       <c r="A15" s="271" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B15" s="271"/>
       <c r="C15" s="271"/>
@@ -7944,10 +7907,8 @@
       <c r="O15" s="271"/>
     </row>
     <row r="16" spans="1:29" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A16" s="272" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
+      <c r="A16" s="272" t="s">
+        <v>166</v>
       </c>
       <c r="B16" s="272"/>
       <c r="C16" s="272"/>

</xml_diff>

<commit_message>
Versao 20261013_001: corrige Diarias e atualiza modelos
</commit_message>
<xml_diff>
--- a/modelos/modelo_mapa.xlsx
+++ b/modelos/modelo_mapa.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gustavo\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09EF87C2-B1C9-4CB6-8D4F-A3E3C29FB006}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32A2EBC9-E615-4FA3-9B79-0F41000ECF1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{8800D05A-11AB-44C8-952A-A0A169E38BB0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{8800D05A-11AB-44C8-952A-A0A169E38BB0}"/>
   </bookViews>
   <sheets>
     <sheet name="Limite 50%" sheetId="1" r:id="rId1"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="176">
   <si>
     <t xml:space="preserve">SECRETARIA DE ESTADO DOS NEGÓCIOS DA SEGURANÇA PÚBLICA </t>
   </si>
@@ -583,15 +583,9 @@
     <t>II</t>
   </si>
   <si>
-    <t>215626/2026</t>
-  </si>
-  <si>
     <t>Assumir o Plantão na Central de Polícia Judiciária de {{{cidade_plantao}}}-SP, conforme determinação contida na Escala referente a {{{data_ida}}}</t>
   </si>
   <si>
-    <t>data protocoloo</t>
-  </si>
-  <si>
     <t>delegacia abrev</t>
   </si>
   <si>
@@ -601,22 +595,22 @@
     <t>CARGO E CLASSE</t>
   </si>
   <si>
-    <t>CIDADE PLANTAO</t>
-  </si>
-  <si>
     <t>MEIO</t>
   </si>
   <si>
-    <t>ida</t>
-  </si>
-  <si>
     <t>volta</t>
   </si>
   <si>
-    <t>001 / 123-4 / 123456-7</t>
-  </si>
-  <si>
     <t>123.456.789-01</t>
+  </si>
+  <si>
+    <t>001 / {{{agencia}}} / {{{conta}}}</t>
+  </si>
+  <si>
+    <t>{{{cidade_plantao}}}</t>
+  </si>
+  <si>
+    <t>{{{protocolo_requerimento}}}</t>
   </si>
 </sst>
 </file>
@@ -2721,7 +2715,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>215626/2026</c:v>
+                  <c:v>{{{protocolo_requerimento}}}</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -3115,7 +3109,7 @@
         <a:p>
           <a:pPr algn="ctr" rtl="0"/>
           <a:r>
-            <a:rPr lang="zh-CN" altLang="en-US" sz="1000" b="1">
+            <a:rPr lang="pt-BR" altLang="zh-CN" sz="1000" b="1">
               <a:solidFill>
                 <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="8"/>
               </a:solidFill>
@@ -3124,20 +3118,17 @@
               <a:cs typeface="Arial Narrow" charset="0"/>
               <a:sym typeface="Arial Narrow" charset="0"/>
             </a:rPr>
-            <a:t>DELEGACIA DE POLÍCIA </a:t>
+            <a:t>{{{delegacia2}}}</a:t>
           </a:r>
-          <a:r>
-            <a:rPr lang="zh-CN" altLang="en-US" sz="1000" b="1">
-              <a:solidFill>
-                <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="8"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" pitchFamily="7" charset="0"/>
-              <a:ea typeface="Arial" pitchFamily="7" charset="0"/>
-              <a:cs typeface="Arial" pitchFamily="7" charset="0"/>
-              <a:sym typeface="Arial" pitchFamily="7" charset="0"/>
-            </a:rPr>
-            <a:t>DE TAGUAÍ</a:t>
-          </a:r>
+          <a:endParaRPr lang="zh-CN" altLang="en-US" sz="1000" b="1">
+            <a:solidFill>
+              <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="8"/>
+            </a:solidFill>
+            <a:latin typeface="Arial" pitchFamily="7" charset="0"/>
+            <a:ea typeface="Arial" pitchFamily="7" charset="0"/>
+            <a:cs typeface="Arial" pitchFamily="7" charset="0"/>
+            <a:sym typeface="Arial" pitchFamily="7" charset="0"/>
+          </a:endParaRPr>
         </a:p>
         <a:p>
           <a:pPr algn="ctr" rtl="0"/>
@@ -3214,6 +3205,18 @@
             <a:t>{{{protocolo_mapa}}}</a:t>
           </a:r>
           <a:endParaRPr lang="zh-CN" altLang="en-US" sz="400">
+            <a:solidFill>
+              <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="8"/>
+            </a:solidFill>
+            <a:latin typeface="Arial Narrow" charset="0"/>
+            <a:ea typeface="Arial Narrow" charset="0"/>
+            <a:cs typeface="Arial Narrow" charset="0"/>
+            <a:sym typeface="Arial Narrow" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr" rtl="0"/>
+          <a:endParaRPr lang="pt-BR" altLang="zh-CN" sz="1000" b="1">
             <a:solidFill>
               <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="8"/>
             </a:solidFill>
@@ -3892,7 +3895,7 @@
     <row r="8" spans="1:38" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2"/>
       <c r="B8" s="199" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C8" s="199"/>
       <c r="D8" s="199"/>
@@ -3914,7 +3917,7 @@
       <c r="R8" s="200"/>
       <c r="S8" s="200"/>
       <c r="T8" s="201" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="U8" s="201"/>
       <c r="V8" s="201"/>
@@ -3924,8 +3927,8 @@
       <c r="Z8" s="201"/>
       <c r="AA8" s="201"/>
       <c r="AB8" s="201"/>
-      <c r="AC8" s="202" t="s">
-        <v>168</v>
+      <c r="AC8" s="202">
+        <v>46387</v>
       </c>
       <c r="AD8" s="202"/>
       <c r="AE8" s="202"/>
@@ -3990,7 +3993,7 @@
       <c r="C10" s="187"/>
       <c r="D10" s="187"/>
       <c r="E10" s="188" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="F10" s="188"/>
       <c r="G10" s="188"/>
@@ -4281,7 +4284,7 @@
     <row r="16" spans="1:38" s="38" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A16" s="2"/>
       <c r="B16" s="217" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C16" s="217"/>
       <c r="D16" s="217"/>
@@ -4290,18 +4293,18 @@
         <v>5</v>
       </c>
       <c r="G16" s="218" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="H16" s="218"/>
       <c r="I16" s="218"/>
-      <c r="J16" s="59" t="s">
-        <v>174</v>
+      <c r="J16" s="59">
+        <v>4</v>
       </c>
       <c r="K16" s="60">
         <v>5.8159722222222203E-2</v>
       </c>
       <c r="L16" s="61" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="M16" s="214">
         <v>0.52425925925925898</v>
@@ -5067,7 +5070,7 @@
       </c>
       <c r="I28" s="240"/>
       <c r="J28" s="241" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="K28" s="241"/>
       <c r="L28" s="241"/>
@@ -5081,7 +5084,7 @@
       <c r="R28" s="240"/>
       <c r="S28" s="240"/>
       <c r="T28" s="242" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="U28" s="242"/>
       <c r="V28" s="242"/>
@@ -5313,7 +5316,7 @@
     <row r="34" spans="1:32" ht="12.6" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A34" s="2"/>
       <c r="B34" s="224" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C34" s="225"/>
       <c r="D34" s="225"/>
@@ -5836,9 +5839,9 @@
       </c>
       <c r="G46" s="255"/>
       <c r="H46" s="255"/>
-      <c r="I46" s="256" t="str">
+      <c r="I46" s="256">
         <f>+AC8</f>
-        <v>data protocoloo</v>
+        <v>46387</v>
       </c>
       <c r="J46" s="256"/>
       <c r="K46" s="256"/>
@@ -7908,7 +7911,7 @@
     </row>
     <row r="16" spans="1:29" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="272" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="B16" s="272"/>
       <c r="C16" s="272"/>

</xml_diff>